<commit_message>
Add rent/vacancy sensitivity grid and Loan Sizing tab
- Sensitivity: third grid showing Cash-on-Cash across monthly rent x
  vacancy (recomputes NOI; management fee scales with EGI)
- Loan Sizing tab: max supportable loan and max purchase price at a
  target DSCR and debt yield, with price headroom vs current price

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFUKyb6gzsdDbmscePYHf6
</commit_message>
<xml_diff>
--- a/RV_Park_Underwriting.xlsx
+++ b/RV_Park_Underwriting.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Actuals vs Pro Forma" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Pro Forma &amp; Returns" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Sensitivity" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Loan Sizing" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,10 +23,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -147,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -245,6 +247,18 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -612,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
@@ -697,143 +711,150 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Sensitivity   — how Cash-on-Cash &amp; DSCR move with purchase price and interest rate.</t>
+          <t xml:space="preserve">  • Sensitivity   — how Cash-on-Cash &amp; DSCR move with price, interest rate, rent &amp; vacancy.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Loan Sizing   — max purchase price the NOI supports at your target DSCR / debt yield.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>HOW TO USE IT</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>1. Start on 'Underwriting'. Fill every yellow cell from the seller's P&amp;L and rent roll.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2. (Optional) Use 'Income Detail' for a seasonal park, then set 'Use Detailed Income Build? = Y'.</t>
+          <t>1. Start on 'Underwriting'. Fill every yellow cell from the seller's P&amp;L and rent roll.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>3. Put the seller's CURRENT numbers into the left column of 'Actuals vs Pro Forma' to see the gap.</t>
+          <t>2. (Optional) Use 'Income Detail' for a seasonal park, then set 'Use Detailed Income Build? = Y'.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>3. Put the seller's CURRENT numbers into the left column of 'Actuals vs Pro Forma' to see the gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>4. Read the headline numbers on 'Deal Summary'; stress-test on 'Sensitivity'.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>RULES OF THUMB (screening, not gospel)</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Cap rate: 8%+ is typical for RV parks; lower means you're paying up.</t>
+          <t>RULES OF THUMB (screening, not gospel)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • DSCR: lenders want 1.25x+. Below 1.20x is a financing risk.</t>
+          <t xml:space="preserve">  • Cap rate: 8%+ is typical for RV parks; lower means you're paying up.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Cash-on-Cash: 8-12%+ in year one is a healthy target.</t>
+          <t xml:space="preserve">  • DSCR: lenders want 1.25x+. Below 1.20x is a financing risk.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Expense ratio: 35-50% of EGI is normal; under 30% usually means expenses are understated.</t>
+          <t xml:space="preserve">  • Cash-on-Cash: 8-12%+ in year one is a healthy target.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • Expense ratio: 35-50% of EGI is normal; under 30% usually means expenses are understated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • Set your Exit Cap 0.5-1.0% HIGHER than the going-in cap to stay conservative.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr"/>
-    </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>RV-PARK-SPECIFIC WATCH-OUTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Transient/nightly income is seasonal and far less stable than annual/monthly tenants.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Utility metering — are sites individually metered, or is the owner eating utilities?</t>
+          <t xml:space="preserve">  • Transient/nightly income is seasonal and far less stable than annual/monthly tenants.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Infrastructure age — septic/sewer, electric pedestals (30/50 amp), water lines = big CapEx.</t>
+          <t xml:space="preserve">  • Utility metering — are sites individually metered, or is the owner eating utilities?</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Flood zone, seasonal closures, and % of park-owned rentals vs. tenant-owned rigs.</t>
+          <t xml:space="preserve">  • Infrastructure age — septic/sewer, electric pedestals (30/50 amp), water lines = big CapEx.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • Flood zone, seasonal closures, and % of park-owned rentals vs. tenant-owned rigs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • Property taxes usually RESET on sale — don't trust the seller's current tax line.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr"/>
-    </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>This is a screening tool, not investment advice. Verify every number and consult professionals.</t>
         </is>
@@ -3379,7 +3400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3407,7 +3428,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>CASH-ON-CASH RETURN  (Year 1)</t>
+          <t>CASH-ON-CASH RETURN  —  Price x Interest Rate</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3592,7 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>DEBT SERVICE COVERAGE (DSCR)</t>
+          <t>DEBT SERVICE COVERAGE (DSCR)  —  Price x Interest Rate</t>
         </is>
       </c>
     </row>
@@ -3735,16 +3756,490 @@
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>NOTE: NOI is held constant; these tables isolate price &amp; financing risk.</t>
+          <t>NOTE: the two tables above hold NOI constant to isolate price &amp; financing risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>CASH-ON-CASH RETURN  —  Monthly Rent x Vacancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="35" t="inlineStr">
+        <is>
+          <t>Rent \ Vacancy</t>
+        </is>
+      </c>
+      <c r="B24" s="39" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C24" s="39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D24" s="39" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E24" s="39" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F24" s="39" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23">
+        <f>Underwriting!B11+-100</f>
+        <v/>
+      </c>
+      <c r="B25" s="37">
+        <f>(((Underwriting!B8*$A25*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="C25" s="37">
+        <f>(((Underwriting!B8*$A25*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="D25" s="37">
+        <f>(((Underwriting!B8*$A25*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="E25" s="37">
+        <f>(((Underwriting!B8*$A25*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="F25" s="37">
+        <f>(((Underwriting!B8*$A25*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="23">
+        <f>Underwriting!B11+-50</f>
+        <v/>
+      </c>
+      <c r="B26" s="37">
+        <f>(((Underwriting!B8*$A26*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="C26" s="37">
+        <f>(((Underwriting!B8*$A26*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="D26" s="37">
+        <f>(((Underwriting!B8*$A26*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="E26" s="37">
+        <f>(((Underwriting!B8*$A26*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="F26" s="37">
+        <f>(((Underwriting!B8*$A26*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23">
+        <f>Underwriting!B11+0</f>
+        <v/>
+      </c>
+      <c r="B27" s="37">
+        <f>(((Underwriting!B8*$A27*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="C27" s="37">
+        <f>(((Underwriting!B8*$A27*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="D27" s="37">
+        <f>(((Underwriting!B8*$A27*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="E27" s="37">
+        <f>(((Underwriting!B8*$A27*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="F27" s="37">
+        <f>(((Underwriting!B8*$A27*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="23">
+        <f>Underwriting!B11+50</f>
+        <v/>
+      </c>
+      <c r="B28" s="37">
+        <f>(((Underwriting!B8*$A28*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="C28" s="37">
+        <f>(((Underwriting!B8*$A28*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="D28" s="37">
+        <f>(((Underwriting!B8*$A28*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="E28" s="37">
+        <f>(((Underwriting!B8*$A28*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="F28" s="37">
+        <f>(((Underwriting!B8*$A28*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="23">
+        <f>Underwriting!B11+100</f>
+        <v/>
+      </c>
+      <c r="B29" s="37">
+        <f>(((Underwriting!B8*$A29*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="C29" s="37">
+        <f>(((Underwriting!B8*$A29*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="D29" s="37">
+        <f>(((Underwriting!B8*$A29*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="E29" s="37">
+        <f>(((Underwriting!B8*$A29*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="F29" s="37">
+        <f>(((Underwriting!B8*$A29*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>NOTE: this table recomputes NOI (management fee scales with EGI). Uses sites x rent income, not the Income Detail build.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A23:F23"/>
     <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>LOAN SIZING — MAX PRICE AT TARGET DSCR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Works backward from how much debt the NOI supports. NOI is held at the Underwriting Year-1 figure; rate, amortization and LTV come from the Underwriting tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>TARGETS  (your / the lender's limits)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Target DSCR</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>minimum coverage lender requires</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Target Debt Yield</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>NOI / loan floor (often 9-10%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Max LTV %</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>lender's loan-to-value cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>LOAN INPUTS  (from Underwriting)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Year-1 NOI</t>
+        </is>
+      </c>
+      <c r="B10" s="20">
+        <f>Underwriting!B40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Interest Rate</t>
+        </is>
+      </c>
+      <c r="B11" s="41">
+        <f>Underwriting!B45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Amortization (yrs)</t>
+        </is>
+      </c>
+      <c r="B12" s="31">
+        <f>Underwriting!B46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Annual Debt Constant (per $1 loan)</t>
+        </is>
+      </c>
+      <c r="B13" s="42">
+        <f>PMT(B11/12,B12*12,-1)*12</f>
+        <v/>
+      </c>
+      <c r="C13" s="15">
+        <f> annual debt service per $1 borrowed</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>MAXIMUM SUPPORTABLE LOAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Max Annual Debt Service (DSCR)</t>
+        </is>
+      </c>
+      <c r="B16" s="20">
+        <f>B10/B5</f>
+        <v/>
+      </c>
+      <c r="C16" s="15">
+        <f> NOI / target DSCR</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Max Loan — DSCR constrained</t>
+        </is>
+      </c>
+      <c r="B17" s="20">
+        <f>B16/B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Max Loan — Debt-Yield constrained</t>
+        </is>
+      </c>
+      <c r="B18" s="20">
+        <f>B10/B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Binding Max Loan</t>
+        </is>
+      </c>
+      <c r="B19" s="23">
+        <f>MIN(B17,B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>the lesser of the two</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>MAXIMUM PURCHASE PRICE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Max Price — DSCR/Debt-Yield (at Max LTV)</t>
+        </is>
+      </c>
+      <c r="B22" s="25">
+        <f>B19/B7</f>
+        <v/>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>price the debt supports at your LTV</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Current Purchase Price</t>
+        </is>
+      </c>
+      <c r="B23" s="20">
+        <f>Underwriting!B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Price Headroom ($)</t>
+        </is>
+      </c>
+      <c r="B24" s="9">
+        <f>B22-B23</f>
+        <v/>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>positive = room to pay more; negative = overpaying</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Price Headroom (%)</t>
+        </is>
+      </c>
+      <c r="B25" s="14">
+        <f>B24/B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>DSCR at Current Price</t>
+        </is>
+      </c>
+      <c r="B26" s="29">
+        <f>Underwriting!B65</f>
+        <v/>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>for reference (target above)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>Required Equity at Max Price</t>
+        </is>
+      </c>
+      <c r="B27" s="20">
+        <f>B22*(1-B7)</f>
+        <v/>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>down payment if you buy at the max</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>READ: if Headroom is negative, the price is higher than the income can safely finance at your target DSCR — you'd need more equity, a lower rate, or a price cut.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Deal Scorecard tab (GOOD/OK/BAD rating)
Rates the deal on 9 metrics (cap rate, cash-on-cash, DSCR, debt yield,
cap-rate spread, expense ratio, break-even occupancy, IRR, equity multiple)
with editable Good/OK cutoffs, live color-coded ratings, a weighted score,
and an overall verdict. Defaults use industry-standard RV-park benchmarks.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFUKyb6gzsdDbmscePYHf6
</commit_message>
<xml_diff>
--- a/RV_Park_Underwriting.xlsx
+++ b/RV_Park_Underwriting.xlsx
@@ -9,12 +9,13 @@
   <sheets>
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Deal Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Underwriting" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Income Detail" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Actuals vs Pro Forma" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Pro Forma &amp; Returns" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sensitivity" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Loan Sizing" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Deal Scorecard" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Underwriting" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Income Detail" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Actuals vs Pro Forma" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Pro Forma &amp; Returns" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Sensitivity" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Loan Sizing" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +30,7 @@
     <numFmt numFmtId="166" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,6 +81,10 @@
       <b val="1"/>
       <color rgb="001F4E78"/>
       <sz val="20"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
     <font>
       <sz val="11"/>
@@ -149,13 +154,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -186,7 +191,32 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -195,9 +225,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -230,9 +257,6 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -252,9 +276,6 @@
     <xf numFmtId="165" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="10" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -265,6 +286,41 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -626,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
@@ -683,178 +739,185 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Underwriting  — the engine. Fill the YELLOW cells; everything else is a formula.</t>
+          <t xml:space="preserve">  • Deal Scorecard — rates the deal GOOD/OK/BAD on each metric with an overall verdict (editable cutoffs).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Income Detail — optional. Build income from your site mix (long-term + seasonal nightly).</t>
+          <t xml:space="preserve">  • Underwriting  — the engine. Fill the YELLOW cells; everything else is a formula.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Actuals vs Pro Forma — seller's CURRENT numbers vs your stabilized plan, side by side.</t>
+          <t xml:space="preserve">  • Income Detail — optional. Build income from your site mix (long-term + seasonal nightly).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Pro Forma &amp; Returns — 10-year projection, sale reversion, IRR &amp; equity multiple.</t>
+          <t xml:space="preserve">  • Actuals vs Pro Forma — seller's CURRENT numbers vs your stabilized plan, side by side.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Sensitivity   — how Cash-on-Cash &amp; DSCR move with price, interest rate, rent &amp; vacancy.</t>
+          <t xml:space="preserve">  • Pro Forma &amp; Returns — 10-year projection, sale reversion, IRR &amp; equity multiple.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • Sensitivity   — how Cash-on-Cash &amp; DSCR move with price, interest rate, rent &amp; vacancy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • Loan Sizing   — max purchase price the NOI supports at your target DSCR / debt yield.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>HOW TO USE IT</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>1. Start on 'Underwriting'. Fill every yellow cell from the seller's P&amp;L and rent roll.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2. (Optional) Use 'Income Detail' for a seasonal park, then set 'Use Detailed Income Build? = Y'.</t>
+          <t>1. Start on 'Underwriting'. Fill every yellow cell from the seller's P&amp;L and rent roll.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>3. Put the seller's CURRENT numbers into the left column of 'Actuals vs Pro Forma' to see the gap.</t>
+          <t>2. (Optional) Use 'Income Detail' for a seasonal park, then set 'Use Detailed Income Build? = Y'.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>3. Put the seller's CURRENT numbers into the left column of 'Actuals vs Pro Forma' to see the gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>4. Read the headline numbers on 'Deal Summary'; stress-test on 'Sensitivity'.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>RULES OF THUMB (screening, not gospel)</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Cap rate: 8%+ is typical for RV parks; lower means you're paying up.</t>
+          <t>RULES OF THUMB (screening, not gospel)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • DSCR: lenders want 1.25x+. Below 1.20x is a financing risk.</t>
+          <t xml:space="preserve">  • Cap rate: 8%+ is typical for RV parks; lower means you're paying up.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Cash-on-Cash: 8-12%+ in year one is a healthy target.</t>
+          <t xml:space="preserve">  • DSCR: lenders want 1.25x+. Below 1.20x is a financing risk.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Expense ratio: 35-50% of EGI is normal; under 30% usually means expenses are understated.</t>
+          <t xml:space="preserve">  • Cash-on-Cash: 8-12%+ in year one is a healthy target.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • Expense ratio: 35-50% of EGI is normal; under 30% usually means expenses are understated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • Set your Exit Cap 0.5-1.0% HIGHER than the going-in cap to stay conservative.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr"/>
-    </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>RV-PARK-SPECIFIC WATCH-OUTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Transient/nightly income is seasonal and far less stable than annual/monthly tenants.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Utility metering — are sites individually metered, or is the owner eating utilities?</t>
+          <t xml:space="preserve">  • Transient/nightly income is seasonal and far less stable than annual/monthly tenants.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Infrastructure age — septic/sewer, electric pedestals (30/50 amp), water lines = big CapEx.</t>
+          <t xml:space="preserve">  • Utility metering — are sites individually metered, or is the owner eating utilities?</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Flood zone, seasonal closures, and % of park-owned rentals vs. tenant-owned rigs.</t>
+          <t xml:space="preserve">  • Infrastructure age — septic/sewer, electric pedestals (30/50 amp), water lines = big CapEx.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • Flood zone, seasonal closures, and % of park-owned rentals vs. tenant-owned rigs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • Property taxes usually RESET on sale — don't trust the seller's current tax line.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
-    </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>This is a screening tool, not investment advice. Verify every number and consult professionals.</t>
         </is>
@@ -1148,6 +1211,428 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>DEAL SCORECARD — GOOD / OK / BAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Defaults are industry-standard RV-park benchmarks. The GREEN cutoff cells are EDITABLE — replace them with your own (or a course/video's) numbers and the ratings update live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Deal Value</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Better</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>Good cutoff</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>OK cutoff</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="G4" s="16" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Going-in Cap Rate</t>
+        </is>
+      </c>
+      <c r="B5" s="14">
+        <f>Underwriting!B62</f>
+        <v/>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F5" s="20">
+        <f>IF(B5&gt;=D5,"GOOD",IF(B5&gt;=E5,"OK","BAD"))</f>
+        <v/>
+      </c>
+      <c r="G5" s="18">
+        <f>IF(F5="GOOD",2,IF(F5="OK",1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Cash-on-Cash (Yr 1)</t>
+        </is>
+      </c>
+      <c r="B6" s="14">
+        <f>Underwriting!B64</f>
+        <v/>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F6" s="20">
+        <f>IF(B6&gt;=D6,"GOOD",IF(B6&gt;=E6,"OK","BAD"))</f>
+        <v/>
+      </c>
+      <c r="G6" s="18">
+        <f>IF(F6="GOOD",2,IF(F6="OK",1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>DSCR</t>
+        </is>
+      </c>
+      <c r="B7" s="21">
+        <f>Underwriting!B65</f>
+        <v/>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E7" s="22" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F7" s="20">
+        <f>IF(B7&gt;=D7,"GOOD",IF(B7&gt;=E7,"OK","BAD"))</f>
+        <v/>
+      </c>
+      <c r="G7" s="18">
+        <f>IF(F7="GOOD",2,IF(F7="OK",1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Debt Yield</t>
+        </is>
+      </c>
+      <c r="B8" s="14">
+        <f>Underwriting!B40/Underwriting!B54</f>
+        <v/>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F8" s="20">
+        <f>IF(B8&gt;=D8,"GOOD",IF(B8&gt;=E8,"OK","BAD"))</f>
+        <v/>
+      </c>
+      <c r="G8" s="18">
+        <f>IF(F8="GOOD",2,IF(F8="OK",1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Cap Rate − Interest (spread)</t>
+        </is>
+      </c>
+      <c r="B9" s="14">
+        <f>Underwriting!B62-Underwriting!B45</f>
+        <v/>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="F9" s="20">
+        <f>IF(B9&gt;=D9,"GOOD",IF(B9&gt;=E9,"OK","BAD"))</f>
+        <v/>
+      </c>
+      <c r="G9" s="18">
+        <f>IF(F9="GOOD",2,IF(F9="OK",1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Operating Expense Ratio</t>
+        </is>
+      </c>
+      <c r="B10" s="14">
+        <f>Underwriting!B36</f>
+        <v/>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F10" s="20">
+        <f>IF(B10&lt;=D10,"GOOD",IF(B10&lt;=E10,"OK","BAD"))</f>
+        <v/>
+      </c>
+      <c r="G10" s="18">
+        <f>IF(F10="GOOD",2,IF(F10="OK",1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Break-even Occupancy</t>
+        </is>
+      </c>
+      <c r="B11" s="14">
+        <f>Underwriting!B67</f>
+        <v/>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F11" s="20">
+        <f>IF(B11&lt;=D11,"GOOD",IF(B11&lt;=E11,"OK","BAD"))</f>
+        <v/>
+      </c>
+      <c r="G11" s="18">
+        <f>IF(F11="GOOD",2,IF(F11="OK",1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Levered IRR</t>
+        </is>
+      </c>
+      <c r="B12" s="14">
+        <f>'Pro Forma &amp; Returns'!B18</f>
+        <v/>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F12" s="20">
+        <f>IF(B12&gt;=D12,"GOOD",IF(B12&gt;=E12,"OK","BAD"))</f>
+        <v/>
+      </c>
+      <c r="G12" s="18">
+        <f>IF(F12="GOOD",2,IF(F12="OK",1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Equity Multiple</t>
+        </is>
+      </c>
+      <c r="B13" s="21">
+        <f>'Pro Forma &amp; Returns'!B19</f>
+        <v/>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="22" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F13" s="20">
+        <f>IF(B13&gt;=D13,"GOOD",IF(B13&gt;=E13,"OK","BAD"))</f>
+        <v/>
+      </c>
+      <c r="G13" s="18">
+        <f>IF(F13="GOOD",2,IF(F13="OK",1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>OVERALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="B16" s="23">
+        <f>SUM(G5:G13)</f>
+        <v/>
+      </c>
+      <c r="C16" s="15">
+        <f>"of "&amp;(13-5+1)*2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Score %</t>
+        </is>
+      </c>
+      <c r="B17" s="14">
+        <f>B16/((13-5+1)*2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>VERDICT</t>
+        </is>
+      </c>
+      <c r="B18" s="25">
+        <f>IF(B17&gt;=0.8,"STRONG DEAL",IF(B17&gt;=0.6,"OK — NEEDS WORK","PASS / BAD DEAL"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Scoring: GOOD=2, OK=1, BAD=0 pts. Verdict: &gt;=80% STRONG, 60-79% OK/NEEDS WORK, &lt;60% PASS. These are screening guides, not gospel — edit the cutoffs to match your strategy or market.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A15:G15"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F5:F13">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"GOOD"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"BAD"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B18">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
+      <formula>"STRONG DEAL"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
+      <formula>"OK — NEEDS WORK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2">
+      <formula>"PASS / BAD DEAL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1164,12 +1649,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Property Name</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="26" t="inlineStr">
         <is>
           <t>Enter property name</t>
         </is>
@@ -1181,24 +1666,24 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Location (City, ST)</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="26" t="inlineStr">
         <is>
           <t>City, ST</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Analysis Date</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
@@ -1212,12 +1697,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Number of RV Sites (pads)</t>
         </is>
       </c>
-      <c r="B8" s="18" t="n">
+      <c r="B8" s="27" t="n">
         <v>50</v>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -1227,22 +1712,22 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Purchase Price</t>
         </is>
       </c>
-      <c r="B9" s="19" t="n">
+      <c r="B9" s="28" t="n">
         <v>1500000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">  Price per Site</t>
         </is>
       </c>
-      <c r="B10" s="20">
+      <c r="B10" s="29">
         <f>B9/B8</f>
         <v/>
       </c>
@@ -1253,12 +1738,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Avg. Monthly Rent per Site</t>
         </is>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="28" t="n">
         <v>450</v>
       </c>
       <c r="C11" s="15" t="inlineStr">
@@ -1268,12 +1753,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Vacancy &amp; Credit Loss %</t>
         </is>
       </c>
-      <c r="B12" s="21" t="n">
+      <c r="B12" s="19" t="n">
         <v>0.15</v>
       </c>
       <c r="C12" s="15" t="inlineStr">
@@ -1283,12 +1768,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Other Income (monthly)</t>
         </is>
       </c>
-      <c r="B13" s="19" t="n">
+      <c r="B13" s="28" t="n">
         <v>1500</v>
       </c>
       <c r="C13" s="15" t="inlineStr">
@@ -1298,12 +1783,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Management Fee (% of EGI)</t>
         </is>
       </c>
-      <c r="B14" s="21" t="n">
+      <c r="B14" s="19" t="n">
         <v>0.08</v>
       </c>
       <c r="C14" s="15" t="inlineStr">
@@ -1313,12 +1798,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Replacement Reserves / site / yr</t>
         </is>
       </c>
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="28" t="n">
         <v>100</v>
       </c>
       <c r="C15" s="15" t="inlineStr">
@@ -1328,12 +1813,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Annual Rent Growth %</t>
         </is>
       </c>
-      <c r="B16" s="21" t="n">
+      <c r="B16" s="19" t="n">
         <v>0.03</v>
       </c>
       <c r="C16" s="15" t="inlineStr">
@@ -1343,12 +1828,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Annual Expense Growth %</t>
         </is>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17" s="19" t="n">
         <v>0.025</v>
       </c>
       <c r="C17" s="15" t="inlineStr">
@@ -1358,12 +1843,12 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Use Detailed Income Build? (Y/N)</t>
         </is>
       </c>
-      <c r="B18" s="22" t="inlineStr">
+      <c r="B18" s="30" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1382,12 +1867,12 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>Gross Potential Rent (GPR)</t>
         </is>
       </c>
-      <c r="B21" s="20">
+      <c r="B21" s="29">
         <f>IF(B18="Y",'Income Detail'!E30,B8*B11*12)</f>
         <v/>
       </c>
@@ -1398,23 +1883,23 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Less: Vacancy &amp; Credit Loss</t>
         </is>
       </c>
-      <c r="B22" s="20">
+      <c r="B22" s="29">
         <f>-B21*B12</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Plus: Other Income</t>
         </is>
       </c>
-      <c r="B23" s="20">
+      <c r="B23" s="29">
         <f>B13*12</f>
         <v/>
       </c>
@@ -1425,7 +1910,7 @@
           <t>Effective Gross Income (EGI)</t>
         </is>
       </c>
-      <c r="B24" s="23">
+      <c r="B24" s="31">
         <f>B21+B22+B23</f>
         <v/>
       </c>
@@ -1438,32 +1923,32 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>Property Taxes</t>
         </is>
       </c>
-      <c r="B27" s="19" t="n">
+      <c r="B27" s="28" t="n">
         <v>18000</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="B28" s="19" t="n">
+      <c r="B28" s="28" t="n">
         <v>9000</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Utilities (water/sewer/trash/elec)</t>
         </is>
       </c>
-      <c r="B29" s="19" t="n">
+      <c r="B29" s="28" t="n">
         <v>36000</v>
       </c>
       <c r="C29" s="15" t="inlineStr">
@@ -1473,42 +1958,42 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>Repairs &amp; Maintenance</t>
         </is>
       </c>
-      <c r="B30" s="19" t="n">
+      <c r="B30" s="28" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>Payroll / Onsite Manager</t>
         </is>
       </c>
-      <c r="B31" s="19" t="n">
+      <c r="B31" s="28" t="n">
         <v>24000</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Marketing, Admin, Office</t>
         </is>
       </c>
-      <c r="B32" s="19" t="n">
+      <c r="B32" s="28" t="n">
         <v>8000</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>Management Fee</t>
         </is>
       </c>
-      <c r="B33" s="20">
+      <c r="B33" s="29">
         <f>B14*B24</f>
         <v/>
       </c>
@@ -1518,12 +2003,12 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Replacement Reserves</t>
         </is>
       </c>
-      <c r="B34" s="20">
+      <c r="B34" s="29">
         <f>B15*B8</f>
         <v/>
       </c>
@@ -1534,18 +2019,18 @@
           <t>Total Operating Expenses</t>
         </is>
       </c>
-      <c r="B35" s="23">
+      <c r="B35" s="31">
         <f>SUM(B27:B34)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="inlineStr">
+      <c r="A36" s="17" t="inlineStr">
         <is>
           <t>Operating Expense Ratio</t>
         </is>
       </c>
-      <c r="B36" s="24">
+      <c r="B36" s="32">
         <f>B35/B24</f>
         <v/>
       </c>
@@ -1556,12 +2041,12 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>Expenses per Site</t>
         </is>
       </c>
-      <c r="B37" s="20">
+      <c r="B37" s="29">
         <f>B35/B8</f>
         <v/>
       </c>
@@ -1579,18 +2064,18 @@
           <t>Net Operating Income (NOI)</t>
         </is>
       </c>
-      <c r="B40" s="25">
+      <c r="B40" s="33">
         <f>B24-B35</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>NOI per Site</t>
         </is>
       </c>
-      <c r="B41" s="20">
+      <c r="B41" s="29">
         <f>B40/B8</f>
         <v/>
       </c>
@@ -1603,22 +2088,22 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="16" t="inlineStr">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>Loan-to-Value (LTV) %</t>
         </is>
       </c>
-      <c r="B44" s="21" t="n">
+      <c r="B44" s="19" t="n">
         <v>0.7</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>Interest Rate %</t>
         </is>
       </c>
-      <c r="B45" s="26" t="n">
+      <c r="B45" s="34" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="C45" s="15" t="inlineStr">
@@ -1628,22 +2113,22 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="16" t="inlineStr">
+      <c r="A46" s="17" t="inlineStr">
         <is>
           <t>Amortization (years)</t>
         </is>
       </c>
-      <c r="B46" s="18" t="n">
+      <c r="B46" s="27" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="16" t="inlineStr">
+      <c r="A47" s="17" t="inlineStr">
         <is>
           <t>Closing Costs %</t>
         </is>
       </c>
-      <c r="B47" s="21" t="n">
+      <c r="B47" s="19" t="n">
         <v>0.03</v>
       </c>
       <c r="C47" s="15" t="inlineStr">
@@ -1653,12 +2138,12 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="16" t="inlineStr">
+      <c r="A48" s="17" t="inlineStr">
         <is>
           <t>Initial CapEx / Rehab</t>
         </is>
       </c>
-      <c r="B48" s="19" t="n">
+      <c r="B48" s="28" t="n">
         <v>50000</v>
       </c>
       <c r="C48" s="15" t="inlineStr">
@@ -1668,12 +2153,12 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="16" t="inlineStr">
+      <c r="A49" s="17" t="inlineStr">
         <is>
           <t>Hold Period (years)</t>
         </is>
       </c>
-      <c r="B49" s="18" t="n">
+      <c r="B49" s="27" t="n">
         <v>5</v>
       </c>
       <c r="C49" s="15" t="inlineStr">
@@ -1683,12 +2168,12 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="16" t="inlineStr">
+      <c r="A50" s="17" t="inlineStr">
         <is>
           <t>Exit Cap Rate %</t>
         </is>
       </c>
-      <c r="B50" s="26" t="n">
+      <c r="B50" s="34" t="n">
         <v>0.08500000000000001</v>
       </c>
       <c r="C50" s="15" t="inlineStr">
@@ -1698,12 +2183,12 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="16" t="inlineStr">
+      <c r="A51" s="17" t="inlineStr">
         <is>
           <t>Selling Costs %</t>
         </is>
       </c>
-      <c r="B51" s="21" t="n">
+      <c r="B51" s="19" t="n">
         <v>0.05</v>
       </c>
       <c r="C51" s="15" t="inlineStr">
@@ -1720,34 +2205,34 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="16" t="inlineStr">
+      <c r="A54" s="17" t="inlineStr">
         <is>
           <t>Loan Amount</t>
         </is>
       </c>
-      <c r="B54" s="20">
+      <c r="B54" s="29">
         <f>B9*B44</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="16" t="inlineStr">
+      <c r="A55" s="17" t="inlineStr">
         <is>
           <t>Down Payment (Equity)</t>
         </is>
       </c>
-      <c r="B55" s="20">
+      <c r="B55" s="29">
         <f>B9-B54</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="16" t="inlineStr">
+      <c r="A56" s="17" t="inlineStr">
         <is>
           <t>Closing Costs</t>
         </is>
       </c>
-      <c r="B56" s="20">
+      <c r="B56" s="29">
         <f>B9*B47</f>
         <v/>
       </c>
@@ -1758,18 +2243,18 @@
           <t>Total Cash Required</t>
         </is>
       </c>
-      <c r="B57" s="23">
+      <c r="B57" s="31">
         <f>B55+B56+B48</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="16" t="inlineStr">
+      <c r="A58" s="17" t="inlineStr">
         <is>
           <t>Monthly Debt Payment</t>
         </is>
       </c>
-      <c r="B58" s="20">
+      <c r="B58" s="29">
         <f>PMT(B45/12,B46*12,-B54)</f>
         <v/>
       </c>
@@ -1798,7 +2283,7 @@
           <t>Going-in Cap Rate</t>
         </is>
       </c>
-      <c r="B62" s="27">
+      <c r="B62" s="35">
         <f>B40/B9</f>
         <v/>
       </c>
@@ -1814,7 +2299,7 @@
           <t>Cash Flow Before Tax (CFBT)</t>
         </is>
       </c>
-      <c r="B63" s="25">
+      <c r="B63" s="33">
         <f>B40-B59</f>
         <v/>
       </c>
@@ -1825,7 +2310,7 @@
           <t>Cash-on-Cash Return</t>
         </is>
       </c>
-      <c r="B64" s="27">
+      <c r="B64" s="35">
         <f>B63/B57</f>
         <v/>
       </c>
@@ -1841,7 +2326,7 @@
           <t>Debt Service Coverage (DSCR)</t>
         </is>
       </c>
-      <c r="B65" s="28">
+      <c r="B65" s="36">
         <f>B40/B59</f>
         <v/>
       </c>
@@ -1852,23 +2337,23 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="16" t="inlineStr">
+      <c r="A66" s="17" t="inlineStr">
         <is>
           <t>Gross Rent Multiplier (GRM)</t>
         </is>
       </c>
-      <c r="B66" s="29">
+      <c r="B66" s="37">
         <f>B9/B21</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="16" t="inlineStr">
+      <c r="A67" s="17" t="inlineStr">
         <is>
           <t>Break-even Occupancy</t>
         </is>
       </c>
-      <c r="B67" s="24">
+      <c r="B67" s="32">
         <f>(B35+B59)/(B21+B23)</f>
         <v/>
       </c>
@@ -1879,12 +2364,12 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="16" t="inlineStr">
+      <c r="A68" s="17" t="inlineStr">
         <is>
           <t>Debt Yield</t>
         </is>
       </c>
-      <c r="B68" s="24">
+      <c r="B68" s="32">
         <f>B40/B54</f>
         <v/>
       </c>
@@ -1909,7 +2394,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1979,16 +2464,16 @@
           <t>Monthly tenants</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="27" t="n">
         <v>30</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="28" t="n">
         <v>450</v>
       </c>
-      <c r="D6" s="21" t="n">
+      <c r="D6" s="19" t="n">
         <v>0.95</v>
       </c>
-      <c r="E6" s="20">
+      <c r="E6" s="29">
         <f>B6*C6*12*D6</f>
         <v/>
       </c>
@@ -1999,16 +2484,16 @@
           <t>Annual / seasonal leases</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="28" t="n">
         <v>400</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="E7" s="20">
+      <c r="E7" s="29">
         <f>B7*C7*12*D7</f>
         <v/>
       </c>
@@ -2023,7 +2508,7 @@
         <f>SUM(B6:B7)</f>
         <v/>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="31">
         <f>SUM(E6:E7)</f>
         <v/>
       </c>
@@ -2041,7 +2526,7 @@
           <t># Transient sites</t>
         </is>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="27" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2051,7 +2536,7 @@
           <t>Avg nightly rate</t>
         </is>
       </c>
-      <c r="B12" s="19" t="n">
+      <c r="B12" s="28" t="n">
         <v>55</v>
       </c>
     </row>
@@ -2078,205 +2563,205 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="B15" s="30" t="n">
+      <c r="B15" s="38" t="n">
         <v>31</v>
       </c>
-      <c r="C15" s="21" t="n">
+      <c r="C15" s="19" t="n">
         <v>0.3</v>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="29">
         <f>$B$11*$B$12*B15*C15</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="B16" s="30" t="n">
+      <c r="B16" s="38" t="n">
         <v>28</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="19" t="n">
         <v>0.3</v>
       </c>
-      <c r="D16" s="20">
+      <c r="D16" s="29">
         <f>$B$11*$B$12*B16*C16</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="B17" s="30" t="n">
+      <c r="B17" s="38" t="n">
         <v>31</v>
       </c>
-      <c r="C17" s="21" t="n">
+      <c r="C17" s="19" t="n">
         <v>0.45</v>
       </c>
-      <c r="D17" s="20">
+      <c r="D17" s="29">
         <f>$B$11*$B$12*B17*C17</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="B18" s="30" t="n">
+      <c r="B18" s="38" t="n">
         <v>30</v>
       </c>
-      <c r="C18" s="21" t="n">
+      <c r="C18" s="19" t="n">
         <v>0.55</v>
       </c>
-      <c r="D18" s="20">
+      <c r="D18" s="29">
         <f>$B$11*$B$12*B18*C18</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="B19" s="30" t="n">
+      <c r="B19" s="38" t="n">
         <v>31</v>
       </c>
-      <c r="C19" s="21" t="n">
+      <c r="C19" s="19" t="n">
         <v>0.7</v>
       </c>
-      <c r="D19" s="20">
+      <c r="D19" s="29">
         <f>$B$11*$B$12*B19*C19</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="B20" s="30" t="n">
+      <c r="B20" s="38" t="n">
         <v>30</v>
       </c>
-      <c r="C20" s="21" t="n">
+      <c r="C20" s="19" t="n">
         <v>0.85</v>
       </c>
-      <c r="D20" s="20">
+      <c r="D20" s="29">
         <f>$B$11*$B$12*B20*C20</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="B21" s="30" t="n">
+      <c r="B21" s="38" t="n">
         <v>31</v>
       </c>
-      <c r="C21" s="21" t="n">
+      <c r="C21" s="19" t="n">
         <v>0.95</v>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="29">
         <f>$B$11*$B$12*B21*C21</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="B22" s="30" t="n">
+      <c r="B22" s="38" t="n">
         <v>31</v>
       </c>
-      <c r="C22" s="21" t="n">
+      <c r="C22" s="19" t="n">
         <v>0.95</v>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="29">
         <f>$B$11*$B$12*B22*C22</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="B23" s="30" t="n">
+      <c r="B23" s="38" t="n">
         <v>30</v>
       </c>
-      <c r="C23" s="21" t="n">
+      <c r="C23" s="19" t="n">
         <v>0.75</v>
       </c>
-      <c r="D23" s="20">
+      <c r="D23" s="29">
         <f>$B$11*$B$12*B23*C23</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="B24" s="30" t="n">
+      <c r="B24" s="38" t="n">
         <v>31</v>
       </c>
-      <c r="C24" s="21" t="n">
+      <c r="C24" s="19" t="n">
         <v>0.55</v>
       </c>
-      <c r="D24" s="20">
+      <c r="D24" s="29">
         <f>$B$11*$B$12*B24*C24</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="B25" s="30" t="n">
+      <c r="B25" s="38" t="n">
         <v>30</v>
       </c>
-      <c r="C25" s="21" t="n">
+      <c r="C25" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="D25" s="20">
+      <c r="D25" s="29">
         <f>$B$11*$B$12*B25*C25</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="B26" s="30" t="n">
+      <c r="B26" s="38" t="n">
         <v>31</v>
       </c>
-      <c r="C26" s="21" t="n">
+      <c r="C26" s="19" t="n">
         <v>0.3</v>
       </c>
-      <c r="D26" s="20">
+      <c r="D26" s="29">
         <f>$B$11*$B$12*B26*C26</f>
         <v/>
       </c>
@@ -2287,18 +2772,18 @@
           <t>Subtotal — transient</t>
         </is>
       </c>
-      <c r="D27" s="23">
+      <c r="D27" s="31">
         <f>SUM(D15:D26)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>Avg transient occupancy</t>
         </is>
       </c>
-      <c r="C28" s="24">
+      <c r="C28" s="32">
         <f>SUMPRODUCT(B15:B26,C15:C26)/SUM(B15:B26)</f>
         <v/>
       </c>
@@ -2316,7 +2801,7 @@
           <t>Total Potential Annual Site Revenue</t>
         </is>
       </c>
-      <c r="E30" s="25">
+      <c r="E30" s="33">
         <f>E8+D27</f>
         <v/>
       </c>
@@ -2327,7 +2812,7 @@
           <t>Total sites in build</t>
         </is>
       </c>
-      <c r="E31" s="31">
+      <c r="E31" s="39">
         <f>B8+B11</f>
         <v/>
       </c>
@@ -2338,7 +2823,7 @@
           <t>Implied blended monthly rent / site</t>
         </is>
       </c>
-      <c r="E32" s="20">
+      <c r="E32" s="29">
         <f>E30/E31/12</f>
         <v/>
       </c>
@@ -2361,7 +2846,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2391,77 +2876,77 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="32" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Line Item</t>
         </is>
       </c>
-      <c r="B4" s="32" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>In-Place / Actuals</t>
         </is>
       </c>
-      <c r="C4" s="32" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>Stabilized Pro Forma</t>
         </is>
       </c>
-      <c r="D4" s="32" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>Variance</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Gross Potential Rent</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
+      <c r="B5" s="28" t="n">
         <v>240000</v>
       </c>
-      <c r="C5" s="20">
+      <c r="C5" s="29">
         <f>Underwriting!B21</f>
         <v/>
       </c>
-      <c r="D5" s="20">
+      <c r="D5" s="29">
         <f>C5-B5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Vacancy &amp; Credit Loss</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
+      <c r="B6" s="28" t="n">
         <v>-48000</v>
       </c>
-      <c r="C6" s="20">
+      <c r="C6" s="29">
         <f>Underwriting!B22</f>
         <v/>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="29">
         <f>C6-B6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Other Income</t>
         </is>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="28" t="n">
         <v>12000</v>
       </c>
-      <c r="C7" s="20">
+      <c r="C7" s="29">
         <f>Underwriting!B23</f>
         <v/>
       </c>
-      <c r="D7" s="20">
+      <c r="D7" s="29">
         <f>C7-B7</f>
         <v/>
       </c>
@@ -2472,159 +2957,159 @@
           <t>Effective Gross Income</t>
         </is>
       </c>
-      <c r="B8" s="23">
+      <c r="B8" s="31">
         <f>B5+B6+B7</f>
         <v/>
       </c>
-      <c r="C8" s="23">
+      <c r="C8" s="31">
         <f>Underwriting!B24</f>
         <v/>
       </c>
-      <c r="D8" s="20">
+      <c r="D8" s="29">
         <f>C8-B8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Property Taxes</t>
         </is>
       </c>
-      <c r="B9" s="19" t="n">
+      <c r="B9" s="28" t="n">
         <v>12000</v>
       </c>
-      <c r="C9" s="20">
+      <c r="C9" s="29">
         <f>Underwriting!B27</f>
         <v/>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="29">
         <f>C9-B9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="B10" s="19" t="n">
+      <c r="B10" s="28" t="n">
         <v>8000</v>
       </c>
-      <c r="C10" s="20">
+      <c r="C10" s="29">
         <f>Underwriting!B28</f>
         <v/>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="29">
         <f>C10-B10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Utilities</t>
         </is>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="28" t="n">
         <v>38000</v>
       </c>
-      <c r="C11" s="20">
+      <c r="C11" s="29">
         <f>Underwriting!B29</f>
         <v/>
       </c>
-      <c r="D11" s="20">
+      <c r="D11" s="29">
         <f>C11-B11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Repairs &amp; Maintenance</t>
         </is>
       </c>
-      <c r="B12" s="19" t="n">
+      <c r="B12" s="28" t="n">
         <v>20000</v>
       </c>
-      <c r="C12" s="20">
+      <c r="C12" s="29">
         <f>Underwriting!B30</f>
         <v/>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="29">
         <f>C12-B12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Payroll / Onsite Mgr</t>
         </is>
       </c>
-      <c r="B13" s="19" t="n">
+      <c r="B13" s="28" t="n">
         <v>20000</v>
       </c>
-      <c r="C13" s="20">
+      <c r="C13" s="29">
         <f>Underwriting!B31</f>
         <v/>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="29">
         <f>C13-B13</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Marketing, Admin, Office</t>
         </is>
       </c>
-      <c r="B14" s="19" t="n">
+      <c r="B14" s="28" t="n">
         <v>6000</v>
       </c>
-      <c r="C14" s="20">
+      <c r="C14" s="29">
         <f>Underwriting!B32</f>
         <v/>
       </c>
-      <c r="D14" s="20">
+      <c r="D14" s="29">
         <f>C14-B14</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Management Fee</t>
         </is>
       </c>
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="20">
+      <c r="C15" s="29">
         <f>Underwriting!B33</f>
         <v/>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="29">
         <f>C15-B15</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Replacement Reserves</t>
         </is>
       </c>
-      <c r="B16" s="19" t="n">
+      <c r="B16" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="20">
+      <c r="C16" s="29">
         <f>Underwriting!B34</f>
         <v/>
       </c>
-      <c r="D16" s="20">
+      <c r="D16" s="29">
         <f>C16-B16</f>
         <v/>
       </c>
@@ -2635,15 +3120,15 @@
           <t>Total Operating Expenses</t>
         </is>
       </c>
-      <c r="B17" s="23">
+      <c r="B17" s="31">
         <f>SUM(B9:B16)</f>
         <v/>
       </c>
-      <c r="C17" s="23">
+      <c r="C17" s="31">
         <f>Underwriting!B35</f>
         <v/>
       </c>
-      <c r="D17" s="20">
+      <c r="D17" s="29">
         <f>C17-B17</f>
         <v/>
       </c>
@@ -2654,15 +3139,15 @@
           <t>Net Operating Income</t>
         </is>
       </c>
-      <c r="B18" s="25">
+      <c r="B18" s="33">
         <f>B8-B17</f>
         <v/>
       </c>
-      <c r="C18" s="25">
+      <c r="C18" s="33">
         <f>Underwriting!B40</f>
         <v/>
       </c>
-      <c r="D18" s="20">
+      <c r="D18" s="29">
         <f>C18-B18</f>
         <v/>
       </c>
@@ -2673,11 +3158,11 @@
           <t>Cap Rate at Purchase Price</t>
         </is>
       </c>
-      <c r="B20" s="27">
+      <c r="B20" s="35">
         <f>B18/Underwriting!B9</f>
         <v/>
       </c>
-      <c r="C20" s="27">
+      <c r="C20" s="35">
         <f>Underwriting!B62</f>
         <v/>
       </c>
@@ -2697,7 +3182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2728,182 +3213,182 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="33" t="inlineStr">
+      <c r="A3" s="40" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B3" s="32" t="n">
+      <c r="B3" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="C3" s="32" t="n">
+      <c r="C3" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="32" t="n">
+      <c r="D3" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="32" t="n">
+      <c r="E3" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="F3" s="32" t="n">
+      <c r="F3" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="G3" s="32" t="n">
+      <c r="G3" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="H3" s="32" t="n">
+      <c r="H3" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="I3" s="32" t="n">
+      <c r="I3" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="J3" s="32" t="n">
+      <c r="J3" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="K3" s="32" t="n">
+      <c r="K3" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="L3" s="32" t="n">
+      <c r="L3" s="16" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Gross Potential Rent</t>
         </is>
       </c>
-      <c r="C5" s="20">
+      <c r="C5" s="29">
         <f>Underwriting!B21*(1+Underwriting!B16)^0</f>
         <v/>
       </c>
-      <c r="D5" s="20">
+      <c r="D5" s="29">
         <f>Underwriting!B21*(1+Underwriting!B16)^1</f>
         <v/>
       </c>
-      <c r="E5" s="20">
+      <c r="E5" s="29">
         <f>Underwriting!B21*(1+Underwriting!B16)^2</f>
         <v/>
       </c>
-      <c r="F5" s="20">
+      <c r="F5" s="29">
         <f>Underwriting!B21*(1+Underwriting!B16)^3</f>
         <v/>
       </c>
-      <c r="G5" s="20">
+      <c r="G5" s="29">
         <f>Underwriting!B21*(1+Underwriting!B16)^4</f>
         <v/>
       </c>
-      <c r="H5" s="20">
+      <c r="H5" s="29">
         <f>Underwriting!B21*(1+Underwriting!B16)^5</f>
         <v/>
       </c>
-      <c r="I5" s="20">
+      <c r="I5" s="29">
         <f>Underwriting!B21*(1+Underwriting!B16)^6</f>
         <v/>
       </c>
-      <c r="J5" s="20">
+      <c r="J5" s="29">
         <f>Underwriting!B21*(1+Underwriting!B16)^7</f>
         <v/>
       </c>
-      <c r="K5" s="20">
+      <c r="K5" s="29">
         <f>Underwriting!B21*(1+Underwriting!B16)^8</f>
         <v/>
       </c>
-      <c r="L5" s="20">
+      <c r="L5" s="29">
         <f>Underwriting!B21*(1+Underwriting!B16)^9</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Less: Vacancy &amp; Credit Loss</t>
         </is>
       </c>
-      <c r="C6" s="20">
+      <c r="C6" s="29">
         <f>-C5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="29">
         <f>-D5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="E6" s="20">
+      <c r="E6" s="29">
         <f>-E5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="29">
         <f>-F5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="29">
         <f>-G5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="H6" s="20">
+      <c r="H6" s="29">
         <f>-H5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="I6" s="20">
+      <c r="I6" s="29">
         <f>-I5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="J6" s="20">
+      <c r="J6" s="29">
         <f>-J5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="K6" s="20">
+      <c r="K6" s="29">
         <f>-K5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="L6" s="20">
+      <c r="L6" s="29">
         <f>-L5*Underwriting!B12</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Other Income</t>
         </is>
       </c>
-      <c r="C7" s="20">
+      <c r="C7" s="29">
         <f>Underwriting!B23*(1+Underwriting!B16)^0</f>
         <v/>
       </c>
-      <c r="D7" s="20">
+      <c r="D7" s="29">
         <f>Underwriting!B23*(1+Underwriting!B16)^1</f>
         <v/>
       </c>
-      <c r="E7" s="20">
+      <c r="E7" s="29">
         <f>Underwriting!B23*(1+Underwriting!B16)^2</f>
         <v/>
       </c>
-      <c r="F7" s="20">
+      <c r="F7" s="29">
         <f>Underwriting!B23*(1+Underwriting!B16)^3</f>
         <v/>
       </c>
-      <c r="G7" s="20">
+      <c r="G7" s="29">
         <f>Underwriting!B23*(1+Underwriting!B16)^4</f>
         <v/>
       </c>
-      <c r="H7" s="20">
+      <c r="H7" s="29">
         <f>Underwriting!B23*(1+Underwriting!B16)^5</f>
         <v/>
       </c>
-      <c r="I7" s="20">
+      <c r="I7" s="29">
         <f>Underwriting!B23*(1+Underwriting!B16)^6</f>
         <v/>
       </c>
-      <c r="J7" s="20">
+      <c r="J7" s="29">
         <f>Underwriting!B23*(1+Underwriting!B16)^7</f>
         <v/>
       </c>
-      <c r="K7" s="20">
+      <c r="K7" s="29">
         <f>Underwriting!B23*(1+Underwriting!B16)^8</f>
         <v/>
       </c>
-      <c r="L7" s="20">
+      <c r="L7" s="29">
         <f>Underwriting!B23*(1+Underwriting!B16)^9</f>
         <v/>
       </c>
@@ -2914,90 +3399,90 @@
           <t>Effective Gross Income</t>
         </is>
       </c>
-      <c r="C8" s="23">
+      <c r="C8" s="31">
         <f>C5+C6+C7</f>
         <v/>
       </c>
-      <c r="D8" s="23">
+      <c r="D8" s="31">
         <f>D5+D6+D7</f>
         <v/>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="31">
         <f>E5+E6+E7</f>
         <v/>
       </c>
-      <c r="F8" s="23">
+      <c r="F8" s="31">
         <f>F5+F6+F7</f>
         <v/>
       </c>
-      <c r="G8" s="23">
+      <c r="G8" s="31">
         <f>G5+G6+G7</f>
         <v/>
       </c>
-      <c r="H8" s="23">
+      <c r="H8" s="31">
         <f>H5+H6+H7</f>
         <v/>
       </c>
-      <c r="I8" s="23">
+      <c r="I8" s="31">
         <f>I5+I6+I7</f>
         <v/>
       </c>
-      <c r="J8" s="23">
+      <c r="J8" s="31">
         <f>J5+J6+J7</f>
         <v/>
       </c>
-      <c r="K8" s="23">
+      <c r="K8" s="31">
         <f>K5+K6+K7</f>
         <v/>
       </c>
-      <c r="L8" s="23">
+      <c r="L8" s="31">
         <f>L5+L6+L7</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Operating Expenses</t>
         </is>
       </c>
-      <c r="C9" s="20">
+      <c r="C9" s="29">
         <f>Underwriting!B35*(1+Underwriting!B17)^0</f>
         <v/>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="29">
         <f>Underwriting!B35*(1+Underwriting!B17)^1</f>
         <v/>
       </c>
-      <c r="E9" s="20">
+      <c r="E9" s="29">
         <f>Underwriting!B35*(1+Underwriting!B17)^2</f>
         <v/>
       </c>
-      <c r="F9" s="20">
+      <c r="F9" s="29">
         <f>Underwriting!B35*(1+Underwriting!B17)^3</f>
         <v/>
       </c>
-      <c r="G9" s="20">
+      <c r="G9" s="29">
         <f>Underwriting!B35*(1+Underwriting!B17)^4</f>
         <v/>
       </c>
-      <c r="H9" s="20">
+      <c r="H9" s="29">
         <f>Underwriting!B35*(1+Underwriting!B17)^5</f>
         <v/>
       </c>
-      <c r="I9" s="20">
+      <c r="I9" s="29">
         <f>Underwriting!B35*(1+Underwriting!B17)^6</f>
         <v/>
       </c>
-      <c r="J9" s="20">
+      <c r="J9" s="29">
         <f>Underwriting!B35*(1+Underwriting!B17)^7</f>
         <v/>
       </c>
-      <c r="K9" s="20">
+      <c r="K9" s="29">
         <f>Underwriting!B35*(1+Underwriting!B17)^8</f>
         <v/>
       </c>
-      <c r="L9" s="20">
+      <c r="L9" s="29">
         <f>Underwriting!B35*(1+Underwriting!B17)^9</f>
         <v/>
       </c>
@@ -3008,141 +3493,141 @@
           <t>Net Operating Income</t>
         </is>
       </c>
-      <c r="C10" s="25">
+      <c r="C10" s="33">
         <f>C8-C9</f>
         <v/>
       </c>
-      <c r="D10" s="25">
+      <c r="D10" s="33">
         <f>D8-D9</f>
         <v/>
       </c>
-      <c r="E10" s="25">
+      <c r="E10" s="33">
         <f>E8-E9</f>
         <v/>
       </c>
-      <c r="F10" s="25">
+      <c r="F10" s="33">
         <f>F8-F9</f>
         <v/>
       </c>
-      <c r="G10" s="25">
+      <c r="G10" s="33">
         <f>G8-G9</f>
         <v/>
       </c>
-      <c r="H10" s="25">
+      <c r="H10" s="33">
         <f>H8-H9</f>
         <v/>
       </c>
-      <c r="I10" s="25">
+      <c r="I10" s="33">
         <f>I8-I9</f>
         <v/>
       </c>
-      <c r="J10" s="25">
+      <c r="J10" s="33">
         <f>J8-J9</f>
         <v/>
       </c>
-      <c r="K10" s="25">
+      <c r="K10" s="33">
         <f>K8-K9</f>
         <v/>
       </c>
-      <c r="L10" s="25">
+      <c r="L10" s="33">
         <f>L8-L9</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Annual Debt Service</t>
         </is>
       </c>
-      <c r="C11" s="20">
+      <c r="C11" s="29">
         <f>IF(1&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="D11" s="20">
+      <c r="D11" s="29">
         <f>IF(2&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="29">
         <f>IF(3&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="F11" s="20">
+      <c r="F11" s="29">
         <f>IF(4&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="G11" s="20">
+      <c r="G11" s="29">
         <f>IF(5&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="H11" s="20">
+      <c r="H11" s="29">
         <f>IF(6&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="I11" s="20">
+      <c r="I11" s="29">
         <f>IF(7&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="J11" s="20">
+      <c r="J11" s="29">
         <f>IF(8&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="K11" s="20">
+      <c r="K11" s="29">
         <f>IF(9&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="L11" s="20">
+      <c r="L11" s="29">
         <f>IF(10&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Loan Balance (end of yr)</t>
         </is>
       </c>
-      <c r="B12" s="20">
+      <c r="B12" s="29">
         <f>Underwriting!B54</f>
         <v/>
       </c>
-      <c r="C12" s="20">
+      <c r="C12" s="29">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(1,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(1,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="29">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(2,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(2,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="29">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(3,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(3,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="29">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(4,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(4,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="G12" s="20">
+      <c r="G12" s="29">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(5,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(5,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="H12" s="20">
+      <c r="H12" s="29">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(6,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(6,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="I12" s="20">
+      <c r="I12" s="29">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(7,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(7,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="J12" s="20">
+      <c r="J12" s="29">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(8,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(8,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="K12" s="20">
+      <c r="K12" s="29">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(9,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(9,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="L12" s="20">
+      <c r="L12" s="29">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(10,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(10,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
@@ -3195,48 +3680,48 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Net Sale Proceeds (reversion)</t>
         </is>
       </c>
-      <c r="C14" s="34">
+      <c r="C14" s="41">
         <f>IF(1=Underwriting!B49,((C10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-C12,0)</f>
         <v/>
       </c>
-      <c r="D14" s="34">
+      <c r="D14" s="41">
         <f>IF(2=Underwriting!B49,((D10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-D12,0)</f>
         <v/>
       </c>
-      <c r="E14" s="34">
+      <c r="E14" s="41">
         <f>IF(3=Underwriting!B49,((E10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-E12,0)</f>
         <v/>
       </c>
-      <c r="F14" s="34">
+      <c r="F14" s="41">
         <f>IF(4=Underwriting!B49,((F10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-F12,0)</f>
         <v/>
       </c>
-      <c r="G14" s="34">
+      <c r="G14" s="41">
         <f>IF(5=Underwriting!B49,((G10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-G12,0)</f>
         <v/>
       </c>
-      <c r="H14" s="34">
+      <c r="H14" s="41">
         <f>IF(6=Underwriting!B49,((H10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-H12,0)</f>
         <v/>
       </c>
-      <c r="I14" s="34">
+      <c r="I14" s="41">
         <f>IF(7=Underwriting!B49,((I10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-I12,0)</f>
         <v/>
       </c>
-      <c r="J14" s="34">
+      <c r="J14" s="41">
         <f>IF(8=Underwriting!B49,((J10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-J12,0)</f>
         <v/>
       </c>
-      <c r="K14" s="34">
+      <c r="K14" s="41">
         <f>IF(9=Underwriting!B49,((K10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-K12,0)</f>
         <v/>
       </c>
-      <c r="L14" s="34">
+      <c r="L14" s="41">
         <f>IF(10=Underwriting!B49,((L10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-L12,0)</f>
         <v/>
       </c>
@@ -3247,47 +3732,47 @@
           <t>Total Cash Flow (for IRR)</t>
         </is>
       </c>
-      <c r="B15" s="25">
+      <c r="B15" s="33">
         <f>-Underwriting!B57</f>
         <v/>
       </c>
-      <c r="C15" s="25">
+      <c r="C15" s="33">
         <f>C13+C14</f>
         <v/>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="33">
         <f>D13+D14</f>
         <v/>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="33">
         <f>E13+E14</f>
         <v/>
       </c>
-      <c r="F15" s="25">
+      <c r="F15" s="33">
         <f>F13+F14</f>
         <v/>
       </c>
-      <c r="G15" s="25">
+      <c r="G15" s="33">
         <f>G13+G14</f>
         <v/>
       </c>
-      <c r="H15" s="25">
+      <c r="H15" s="33">
         <f>H13+H14</f>
         <v/>
       </c>
-      <c r="I15" s="25">
+      <c r="I15" s="33">
         <f>I13+I14</f>
         <v/>
       </c>
-      <c r="J15" s="25">
+      <c r="J15" s="33">
         <f>J13+J14</f>
         <v/>
       </c>
-      <c r="K15" s="25">
+      <c r="K15" s="33">
         <f>K13+K14</f>
         <v/>
       </c>
-      <c r="L15" s="25">
+      <c r="L15" s="33">
         <f>L13+L14</f>
         <v/>
       </c>
@@ -3305,7 +3790,7 @@
           <t>Levered IRR</t>
         </is>
       </c>
-      <c r="B18" s="27">
+      <c r="B18" s="35">
         <f>IRR(B15:L15)</f>
         <v/>
       </c>
@@ -3321,7 +3806,7 @@
           <t>Equity Multiple</t>
         </is>
       </c>
-      <c r="B19" s="28">
+      <c r="B19" s="36">
         <f>(SUM(C13:L13)+SUM(C14:L14))/-B15</f>
         <v/>
       </c>
@@ -3337,7 +3822,7 @@
           <t>Avg. Cash-on-Cash</t>
         </is>
       </c>
-      <c r="B20" s="27">
+      <c r="B20" s="35">
         <f>AVERAGEIF(C11:L11,"&gt;0",C13:L13)/Underwriting!B57</f>
         <v/>
       </c>
@@ -3353,7 +3838,7 @@
           <t>Year-1 Cash-on-Cash</t>
         </is>
       </c>
-      <c r="B21" s="27">
+      <c r="B21" s="35">
         <f>Underwriting!B64</f>
         <v/>
       </c>
@@ -3364,7 +3849,7 @@
           <t>Going-in Cap Rate</t>
         </is>
       </c>
-      <c r="B22" s="27">
+      <c r="B22" s="35">
         <f>Underwriting!B62</f>
         <v/>
       </c>
@@ -3375,7 +3860,7 @@
           <t>Total Profit</t>
         </is>
       </c>
-      <c r="B23" s="25">
+      <c r="B23" s="33">
         <f>SUM(C13:L13)+SUM(C14:L14)+B15</f>
         <v/>
       </c>
@@ -3394,7 +3879,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3433,158 +3918,158 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="35" t="inlineStr">
+      <c r="A5" s="42" t="inlineStr">
         <is>
           <t>Price \ Rate</t>
         </is>
       </c>
-      <c r="B5" s="36">
+      <c r="B5" s="43">
         <f>Underwriting!B45+-0.01</f>
         <v/>
       </c>
-      <c r="C5" s="36">
+      <c r="C5" s="43">
         <f>Underwriting!B45+-0.005</f>
         <v/>
       </c>
-      <c r="D5" s="36">
+      <c r="D5" s="43">
         <f>Underwriting!B45+0</f>
         <v/>
       </c>
-      <c r="E5" s="36">
+      <c r="E5" s="43">
         <f>Underwriting!B45+0.005</f>
         <v/>
       </c>
-      <c r="F5" s="36">
+      <c r="F5" s="43">
         <f>Underwriting!B45+0.01</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23">
+      <c r="A6" s="31">
         <f>Underwriting!B9*0.9</f>
         <v/>
       </c>
-      <c r="B6" s="37">
+      <c r="B6" s="44">
         <f>(Underwriting!B40-((($A6*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="C6" s="37">
+      <c r="C6" s="44">
         <f>(Underwriting!B40-((($A6*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="D6" s="37">
+      <c r="D6" s="44">
         <f>(Underwriting!B40-((($A6*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="E6" s="37">
+      <c r="E6" s="44">
         <f>(Underwriting!B40-((($A6*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="F6" s="37">
+      <c r="F6" s="44">
         <f>(Underwriting!B40-((($A6*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23">
+      <c r="A7" s="31">
         <f>Underwriting!B9*0.95</f>
         <v/>
       </c>
-      <c r="B7" s="37">
+      <c r="B7" s="44">
         <f>(Underwriting!B40-((($A7*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="C7" s="37">
+      <c r="C7" s="44">
         <f>(Underwriting!B40-((($A7*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="D7" s="37">
+      <c r="D7" s="44">
         <f>(Underwriting!B40-((($A7*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="E7" s="37">
+      <c r="E7" s="44">
         <f>(Underwriting!B40-((($A7*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="F7" s="37">
+      <c r="F7" s="44">
         <f>(Underwriting!B40-((($A7*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23">
+      <c r="A8" s="31">
         <f>Underwriting!B9*1.0</f>
         <v/>
       </c>
-      <c r="B8" s="37">
+      <c r="B8" s="44">
         <f>(Underwriting!B40-((($A8*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="C8" s="37">
+      <c r="C8" s="44">
         <f>(Underwriting!B40-((($A8*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="D8" s="37">
+      <c r="D8" s="44">
         <f>(Underwriting!B40-((($A8*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="E8" s="37">
+      <c r="E8" s="44">
         <f>(Underwriting!B40-((($A8*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="F8" s="37">
+      <c r="F8" s="44">
         <f>(Underwriting!B40-((($A8*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23">
+      <c r="A9" s="31">
         <f>Underwriting!B9*1.05</f>
         <v/>
       </c>
-      <c r="B9" s="37">
+      <c r="B9" s="44">
         <f>(Underwriting!B40-((($A9*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="C9" s="37">
+      <c r="C9" s="44">
         <f>(Underwriting!B40-((($A9*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="D9" s="37">
+      <c r="D9" s="44">
         <f>(Underwriting!B40-((($A9*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="E9" s="37">
+      <c r="E9" s="44">
         <f>(Underwriting!B40-((($A9*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="F9" s="37">
+      <c r="F9" s="44">
         <f>(Underwriting!B40-((($A9*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23">
+      <c r="A10" s="31">
         <f>Underwriting!B9*1.1</f>
         <v/>
       </c>
-      <c r="B10" s="37">
+      <c r="B10" s="44">
         <f>(Underwriting!B40-((($A10*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="C10" s="37">
+      <c r="C10" s="44">
         <f>(Underwriting!B40-((($A10*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="D10" s="37">
+      <c r="D10" s="44">
         <f>(Underwriting!B40-((($A10*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="44">
         <f>(Underwriting!B40-((($A10*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="F10" s="37">
+      <c r="F10" s="44">
         <f>(Underwriting!B40-((($A10*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
@@ -3597,158 +4082,158 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="35" t="inlineStr">
+      <c r="A14" s="42" t="inlineStr">
         <is>
           <t>Price \ Rate</t>
         </is>
       </c>
-      <c r="B14" s="36">
+      <c r="B14" s="43">
         <f>Underwriting!B45+-0.01</f>
         <v/>
       </c>
-      <c r="C14" s="36">
+      <c r="C14" s="43">
         <f>Underwriting!B45+-0.005</f>
         <v/>
       </c>
-      <c r="D14" s="36">
+      <c r="D14" s="43">
         <f>Underwriting!B45+0</f>
         <v/>
       </c>
-      <c r="E14" s="36">
+      <c r="E14" s="43">
         <f>Underwriting!B45+0.005</f>
         <v/>
       </c>
-      <c r="F14" s="36">
+      <c r="F14" s="43">
         <f>Underwriting!B45+0.01</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23">
+      <c r="A15" s="31">
         <f>Underwriting!B9*0.9</f>
         <v/>
       </c>
-      <c r="B15" s="38">
+      <c r="B15" s="45">
         <f>Underwriting!B40/((($A15*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="C15" s="38">
+      <c r="C15" s="45">
         <f>Underwriting!B40/((($A15*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="D15" s="38">
+      <c r="D15" s="45">
         <f>Underwriting!B40/((($A15*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="E15" s="38">
+      <c r="E15" s="45">
         <f>Underwriting!B40/((($A15*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="F15" s="38">
+      <c r="F15" s="45">
         <f>Underwriting!B40/((($A15*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23">
+      <c r="A16" s="31">
         <f>Underwriting!B9*0.95</f>
         <v/>
       </c>
-      <c r="B16" s="38">
+      <c r="B16" s="45">
         <f>Underwriting!B40/((($A16*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="C16" s="38">
+      <c r="C16" s="45">
         <f>Underwriting!B40/((($A16*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="D16" s="38">
+      <c r="D16" s="45">
         <f>Underwriting!B40/((($A16*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="E16" s="38">
+      <c r="E16" s="45">
         <f>Underwriting!B40/((($A16*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="F16" s="38">
+      <c r="F16" s="45">
         <f>Underwriting!B40/((($A16*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23">
+      <c r="A17" s="31">
         <f>Underwriting!B9*1.0</f>
         <v/>
       </c>
-      <c r="B17" s="38">
+      <c r="B17" s="45">
         <f>Underwriting!B40/((($A17*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="C17" s="38">
+      <c r="C17" s="45">
         <f>Underwriting!B40/((($A17*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="D17" s="38">
+      <c r="D17" s="45">
         <f>Underwriting!B40/((($A17*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="E17" s="38">
+      <c r="E17" s="45">
         <f>Underwriting!B40/((($A17*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="F17" s="38">
+      <c r="F17" s="45">
         <f>Underwriting!B40/((($A17*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="23">
+      <c r="A18" s="31">
         <f>Underwriting!B9*1.05</f>
         <v/>
       </c>
-      <c r="B18" s="38">
+      <c r="B18" s="45">
         <f>Underwriting!B40/((($A18*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="C18" s="38">
+      <c r="C18" s="45">
         <f>Underwriting!B40/((($A18*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="D18" s="38">
+      <c r="D18" s="45">
         <f>Underwriting!B40/((($A18*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="E18" s="38">
+      <c r="E18" s="45">
         <f>Underwriting!B40/((($A18*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="F18" s="38">
+      <c r="F18" s="45">
         <f>Underwriting!B40/((($A18*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23">
+      <c r="A19" s="31">
         <f>Underwriting!B9*1.1</f>
         <v/>
       </c>
-      <c r="B19" s="38">
+      <c r="B19" s="45">
         <f>Underwriting!B40/((($A19*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="C19" s="38">
+      <c r="C19" s="45">
         <f>Underwriting!B40/((($A19*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="D19" s="38">
+      <c r="D19" s="45">
         <f>Underwriting!B40/((($A19*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="E19" s="38">
+      <c r="E19" s="45">
         <f>Underwriting!B40/((($A19*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="F19" s="38">
+      <c r="F19" s="45">
         <f>Underwriting!B40/((($A19*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
@@ -3768,153 +4253,153 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="35" t="inlineStr">
+      <c r="A24" s="42" t="inlineStr">
         <is>
           <t>Rent \ Vacancy</t>
         </is>
       </c>
-      <c r="B24" s="39" t="n">
+      <c r="B24" s="46" t="n">
         <v>0.05</v>
       </c>
-      <c r="C24" s="39" t="n">
+      <c r="C24" s="46" t="n">
         <v>0.1</v>
       </c>
-      <c r="D24" s="39" t="n">
+      <c r="D24" s="46" t="n">
         <v>0.15</v>
       </c>
-      <c r="E24" s="39" t="n">
+      <c r="E24" s="46" t="n">
         <v>0.2</v>
       </c>
-      <c r="F24" s="39" t="n">
+      <c r="F24" s="46" t="n">
         <v>0.25</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="23">
+      <c r="A25" s="31">
         <f>Underwriting!B11+-100</f>
         <v/>
       </c>
-      <c r="B25" s="37">
+      <c r="B25" s="44">
         <f>(((Underwriting!B8*$A25*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="C25" s="37">
+      <c r="C25" s="44">
         <f>(((Underwriting!B8*$A25*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="D25" s="37">
+      <c r="D25" s="44">
         <f>(((Underwriting!B8*$A25*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="E25" s="37">
+      <c r="E25" s="44">
         <f>(((Underwriting!B8*$A25*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="F25" s="37">
+      <c r="F25" s="44">
         <f>(((Underwriting!B8*$A25*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="23">
+      <c r="A26" s="31">
         <f>Underwriting!B11+-50</f>
         <v/>
       </c>
-      <c r="B26" s="37">
+      <c r="B26" s="44">
         <f>(((Underwriting!B8*$A26*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="C26" s="37">
+      <c r="C26" s="44">
         <f>(((Underwriting!B8*$A26*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="D26" s="37">
+      <c r="D26" s="44">
         <f>(((Underwriting!B8*$A26*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="E26" s="37">
+      <c r="E26" s="44">
         <f>(((Underwriting!B8*$A26*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="F26" s="37">
+      <c r="F26" s="44">
         <f>(((Underwriting!B8*$A26*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="23">
+      <c r="A27" s="31">
         <f>Underwriting!B11+0</f>
         <v/>
       </c>
-      <c r="B27" s="37">
+      <c r="B27" s="44">
         <f>(((Underwriting!B8*$A27*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="C27" s="37">
+      <c r="C27" s="44">
         <f>(((Underwriting!B8*$A27*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="D27" s="37">
+      <c r="D27" s="44">
         <f>(((Underwriting!B8*$A27*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="E27" s="37">
+      <c r="E27" s="44">
         <f>(((Underwriting!B8*$A27*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="F27" s="37">
+      <c r="F27" s="44">
         <f>(((Underwriting!B8*$A27*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="23">
+      <c r="A28" s="31">
         <f>Underwriting!B11+50</f>
         <v/>
       </c>
-      <c r="B28" s="37">
+      <c r="B28" s="44">
         <f>(((Underwriting!B8*$A28*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="C28" s="37">
+      <c r="C28" s="44">
         <f>(((Underwriting!B8*$A28*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="D28" s="37">
+      <c r="D28" s="44">
         <f>(((Underwriting!B8*$A28*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="E28" s="37">
+      <c r="E28" s="44">
         <f>(((Underwriting!B8*$A28*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="F28" s="37">
+      <c r="F28" s="44">
         <f>(((Underwriting!B8*$A28*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="23">
+      <c r="A29" s="31">
         <f>Underwriting!B11+100</f>
         <v/>
       </c>
-      <c r="B29" s="37">
+      <c r="B29" s="44">
         <f>(((Underwriting!B8*$A29*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="C29" s="37">
+      <c r="C29" s="44">
         <f>(((Underwriting!B8*$A29*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="D29" s="37">
+      <c r="D29" s="44">
         <f>(((Underwriting!B8*$A29*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="E29" s="37">
+      <c r="E29" s="44">
         <f>(((Underwriting!B8*$A29*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="F29" s="37">
+      <c r="F29" s="44">
         <f>(((Underwriting!B8*$A29*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
@@ -3937,7 +4422,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3973,12 +4458,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Target DSCR</t>
         </is>
       </c>
-      <c r="B5" s="40" t="n">
+      <c r="B5" s="22" t="n">
         <v>1.25</v>
       </c>
       <c r="C5" s="15" t="inlineStr">
@@ -3988,12 +4473,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Target Debt Yield</t>
         </is>
       </c>
-      <c r="B6" s="21" t="n">
+      <c r="B6" s="19" t="n">
         <v>0.1</v>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -4003,12 +4488,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Max LTV %</t>
         </is>
       </c>
-      <c r="B7" s="21" t="n">
+      <c r="B7" s="19" t="n">
         <v>0.75</v>
       </c>
       <c r="C7" s="15" t="inlineStr">
@@ -4025,45 +4510,45 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Year-1 NOI</t>
         </is>
       </c>
-      <c r="B10" s="20">
+      <c r="B10" s="29">
         <f>Underwriting!B40</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Interest Rate</t>
         </is>
       </c>
-      <c r="B11" s="41">
+      <c r="B11" s="47">
         <f>Underwriting!B45</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Amortization (yrs)</t>
         </is>
       </c>
-      <c r="B12" s="31">
+      <c r="B12" s="39">
         <f>Underwriting!B46</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Annual Debt Constant (per $1 loan)</t>
         </is>
       </c>
-      <c r="B13" s="42">
+      <c r="B13" s="48">
         <f>PMT(B11/12,B12*12,-1)*12</f>
         <v/>
       </c>
@@ -4080,12 +4565,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Max Annual Debt Service (DSCR)</t>
         </is>
       </c>
-      <c r="B16" s="20">
+      <c r="B16" s="29">
         <f>B10/B5</f>
         <v/>
       </c>
@@ -4095,23 +4580,23 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Max Loan — DSCR constrained</t>
         </is>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="29">
         <f>B16/B13</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Max Loan — Debt-Yield constrained</t>
         </is>
       </c>
-      <c r="B18" s="20">
+      <c r="B18" s="29">
         <f>B10/B6</f>
         <v/>
       </c>
@@ -4122,7 +4607,7 @@
           <t>Binding Max Loan</t>
         </is>
       </c>
-      <c r="B19" s="23">
+      <c r="B19" s="31">
         <f>MIN(B17,B18)</f>
         <v/>
       </c>
@@ -4145,7 +4630,7 @@
           <t>Max Price — DSCR/Debt-Yield (at Max LTV)</t>
         </is>
       </c>
-      <c r="B22" s="25">
+      <c r="B22" s="33">
         <f>B19/B7</f>
         <v/>
       </c>
@@ -4156,12 +4641,12 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Current Purchase Price</t>
         </is>
       </c>
-      <c r="B23" s="20">
+      <c r="B23" s="29">
         <f>Underwriting!B9</f>
         <v/>
       </c>
@@ -4194,12 +4679,12 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>DSCR at Current Price</t>
         </is>
       </c>
-      <c r="B26" s="29">
+      <c r="B26" s="37">
         <f>Underwriting!B65</f>
         <v/>
       </c>
@@ -4210,12 +4695,12 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>Required Equity at Max Price</t>
         </is>
       </c>
-      <c r="B27" s="20">
+      <c r="B27" s="29">
         <f>B22*(1-B7)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Rebuild underwriting sheet on AJ Kukra's framework + Whisper SOP
Spreadsheet:
- Deal Scorecard rewritten to AJ's exact thresholds: DSCR>=1.35 and
  Cash-on-Cash>=10% as go/no-go, plus his 5 quick hacks (1% rule, 10x/GRM,
  quick DSCR, expense-ratio BAND with <30%=fiction, negative-leverage spread)
  and his go / conditional / no-go verdict.
- New Normalization tab: rebuilds seller NOI with AJ's 4 adjustments
  (mgmt 10%, R&M 5%, capex +3%, taxes +20%) and shows NOI haircut +
  overpayment risk.
- Read Me rewritten around AJ's methodology; notes MHP applicability.

Skill: make Whisper transcription the standing SOP for shared video links.

Source: AJ Kukra, RV Park Profit Blueprint workshop (user-provided transcript).
</commit_message>
<xml_diff>
--- a/RV_Park_Underwriting.xlsx
+++ b/RV_Park_Underwriting.xlsx
@@ -11,11 +11,12 @@
     <sheet name="Deal Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Deal Scorecard" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Underwriting" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Income Detail" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Actuals vs Pro Forma" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Pro Forma &amp; Returns" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Sensitivity" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Loan Sizing" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Normalization" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Income Detail" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Actuals vs Pro Forma" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Pro Forma &amp; Returns" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Sensitivity" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Loan Sizing" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +31,7 @@
     <numFmt numFmtId="166" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,6 +85,11 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="13"/>
     </font>
     <font>
@@ -95,7 +101,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -127,6 +133,11 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -154,13 +165,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -195,15 +206,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -211,10 +213,16 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -239,9 +247,6 @@
     <xf numFmtId="164" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="165" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -249,6 +254,16 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -266,9 +281,6 @@
     </xf>
     <xf numFmtId="10" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -682,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
@@ -708,118 +720,118 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>A deal-screening model for buying RV parks. Plug in a property's numbers and it returns the cap rate,</t>
+          <t>An RV-park deal-screening model built on AJ Kukra's 'RV Park Profit Blueprint' framework. Drop in a</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>cash flow, cash-on-cash, DSCR, debt yield, and a 5-10 year IRR so you can decide fast if a deal works.</t>
+          <t>deal's numbers and it tells you in minutes whether it makes money — using AJ's 5 key metrics, his 5</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>quick hacks, NOI normalization, and his go / conditional / no-go rule. Works for RV parks and adapts</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>THE TABS (left to right)</t>
+          <t>directly to mobile home parks (same lot-rent math). Source: AJ Kukra, RV Park Profit Blueprint workshop.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Deal Summary  — one-page headline view; print/screenshot this for lenders &amp; partners.</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Deal Scorecard — rates the deal GOOD/OK/BAD on each metric with an overall verdict (editable cutoffs).</t>
+          <t>AJ'S 5 KEY METRICS (the heartbeat of the deal)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Underwriting  — the engine. Fill the YELLOW cells; everything else is a formula.</t>
+          <t xml:space="preserve">  1. NOI — effective gross income (EGI) minus operating expenses. Every other metric flows from it.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Income Detail — optional. Build income from your site mix (long-term + seasonal nightly).</t>
+          <t xml:space="preserve">  2. Cap Rate = NOI / price. Higher = paying less. But a very high cap (14%+) usually means hidden risk.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Actuals vs Pro Forma — seller's CURRENT numbers vs your stabilized plan, side by side.</t>
+          <t xml:space="preserve">  3. DSCR = NOI / annual debt. AJ's floor is 1.35x — that's YOUR target, not just the lender's.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Pro Forma &amp; Returns — 10-year projection, sale reversion, IRR &amp; equity multiple.</t>
+          <t xml:space="preserve">  4. Net Profit = what's left after opex AND debt service.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Sensitivity   — how Cash-on-Cash &amp; DSCR move with price, interest rate, rent &amp; vacancy.</t>
+          <t xml:space="preserve">  5. Cash-on-Cash = net profit / cash invested. AJ's target is 10%+.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Loan Sizing   — max purchase price the NOI supports at your target DSCR / debt yield.</t>
-        </is>
-      </c>
+      <c r="A15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>AJ'S 5 QUICK HACKS (screen any listing in ~2 minutes) — see the Deal Scorecard tab</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>HOW TO USE IT</t>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. 1% Rule — monthly gross &gt;= 1% of price = likely good (cross the last two zeros off the price).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>1. Start on 'Underwriting'. Fill every yellow cell from the seller's P&amp;L and rent roll.</t>
+          <t xml:space="preserve">  2. 10x Rule (GRM) — price / annual gross; want UNDER 10. Over ~15 is expensive.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2. (Optional) Use 'Income Detail' for a seasonal park, then set 'Use Detailed Income Build? = Y'.</t>
+          <t xml:space="preserve">  3. Quick DSCR — NOI / (price x interest rate): &gt;1.5 good, 1.25-1.5 closer look, &lt;1.25 lending risk.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>3. Put the seller's CURRENT numbers into the left column of 'Actuals vs Pro Forma' to see the gap.</t>
+          <t xml:space="preserve">  4. Expense Ratio — OpEx / gross: UNDER 30% = numbers are fiction; 35-65% normal; over 70% a problem.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>4. Read the headline numbers on 'Deal Summary'; stress-test on 'Sensitivity'.</t>
+          <t xml:space="preserve">  5. Negative Leverage — if cap rate &lt; your interest rate you lose money day one. Want cap ABOVE rate.</t>
         </is>
       </c>
     </row>
@@ -829,87 +841,83 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>RULES OF THUMB (screening, not gospel)</t>
+          <t>NORMALIZE THE NOI (AJ: never trust the seller's NOI) — see the Normalization tab</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Cap rate: 8%+ is typical for RV parks; lower means you're paying up.</t>
+          <t xml:space="preserve">  The OM is the seller's best case; the Pro Forma is fantasy; the T12 is your start but needs adjusting.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • DSCR: lenders want 1.25x+. Below 1.20x is a financing risk.</t>
+          <t xml:space="preserve">  AJ's 4 standard adjustments: management -&gt; 10% of EGI, repairs -&gt; 5% (or prior year), capex -&gt; +3%,</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Cash-on-Cash: 8-12%+ in year one is a healthy target.</t>
+          <t xml:space="preserve">  property taxes -&gt; +20% (they reset on sale). A small NOI cut at an 8-10% cap = a huge price difference.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Expense ratio: 35-50% of EGI is normal; under 30% usually means expenses are understated.</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Set your Exit Cap 0.5-1.0% HIGHER than the going-in cap to stay conservative.</t>
+          <t>THE BAD-DAY TEST (break the deal on purpose) — use the Sensitivity tab</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Cut occupancy 10-15%, add 1-2% to the interest rate, raise expenses 10-15%. Does DSCR still clear?</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>RV-PARK-SPECIFIC WATCH-OUTS</t>
-        </is>
-      </c>
+      <c r="A30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Transient/nightly income is seasonal and far less stable than annual/monthly tenants.</t>
+          <t>THE DECISION (after normalizing)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Utility metering — are sites individually metered, or is the owner eating utilities?</t>
+          <t xml:space="preserve">  Both DSCR (&gt;=1.35) AND Cash-on-Cash (&gt;=10%) clear -&gt; GO. One fails -&gt; CONDITIONAL (restructure).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Infrastructure age — septic/sewer, electric pedestals (30/50 amp), water lines = big CapEx.</t>
+          <t xml:space="preserve">  Both fail -&gt; likely NO-GO. To save a conditional deal, use AJ's 3 levers: lower the price to your</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Flood zone, seasonal closures, and % of park-owned rentals vs. tenant-owned rigs.</t>
+          <t xml:space="preserve">  MAO, ask the seller to carry a slice (blended rate drops), or add down payment. Don't pay the seller</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Property taxes usually RESET on sale — don't trust the seller's current tax line.</t>
+          <t xml:space="preserve">  for value YOU will create (rent bumps to market, occupancy, utility bill-back, added revenue).</t>
         </is>
       </c>
     </row>
@@ -919,11 +927,474 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
+          <t>THE TABS (left to right)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Deal Summary  — one-page headline view; print/screenshot for lenders &amp; partners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Deal Scorecard — AJ's metrics + 5 hacks rated GOOD/OK/BAD with his go / conditional / no-go verdict.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Underwriting  — the engine. Fill the YELLOW cells; everything else is a formula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Normalization — rebuild the seller's NOI with AJ's 4 adjustments; shows the overpayment risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Income Detail — optional. Build income from your site mix (long-term + seasonal nightly).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Actuals vs Pro Forma — seller's CURRENT numbers vs your stabilized plan, side by side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Pro Forma &amp; Returns — 10-year projection, sale reversion, IRR &amp; equity multiple.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Sensitivity   — the Bad-Day Test: CoC &amp; DSCR vs price, interest rate, rent &amp; vacancy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Loan Sizing   — max purchase price the NOI supports at your target DSCR / debt yield.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>HOW TO USE IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>1. Normalization tab: enter the seller's reported expenses; read off your normalized NOI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2. Underwriting tab: fill the yellow cells using those NORMALIZED numbers, not the seller's.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>3. Deal Scorecard: read the GOOD/OK/BAD ratings and the GO / CONDITIONAL / NO-GO verdict.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>4. Sensitivity: run the bad-day stress test. Deal Summary: the one-page headline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>RV-PARK / MHP WATCH-OUTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Nondisclosure states: sellers needn't volunteer problems (failing septic, AC, zoning). Dig.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Transient/nightly income is seasonal and far less stable than annual/monthly tenants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Utility metering — are sites individually metered, or is the owner eating utilities? (ratio bill-back).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Infrastructure age — septic/sewer, electric pedestals (30/50 amp), water lines = big CapEx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Property taxes usually RESET on sale — don't trust the seller's current tax line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
           <t>This is a screening tool, not investment advice. Verify every number and consult professionals.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>LOAN SIZING — MAX PRICE AT TARGET DSCR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Works backward from how much debt the NOI supports. NOI is held at the Underwriting Year-1 figure; rate, amortization and LTV come from the Underwriting tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>TARGETS  (your / the lender's limits)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Target DSCR</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>minimum coverage lender requires</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Target Debt Yield</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>NOI / loan floor (often 9-10%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Max LTV %</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>lender's loan-to-value cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>LOAN INPUTS  (from Underwriting)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Year-1 NOI</t>
+        </is>
+      </c>
+      <c r="B10" s="28">
+        <f>Underwriting!B40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Interest Rate</t>
+        </is>
+      </c>
+      <c r="B11" s="48">
+        <f>Underwriting!B45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Amortization (yrs)</t>
+        </is>
+      </c>
+      <c r="B12" s="41">
+        <f>Underwriting!B46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Annual Debt Constant (per $1 loan)</t>
+        </is>
+      </c>
+      <c r="B13" s="49">
+        <f>PMT(B11/12,B12*12,-1)*12</f>
+        <v/>
+      </c>
+      <c r="C13" s="15">
+        <f> annual debt service per $1 borrowed</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>MAXIMUM SUPPORTABLE LOAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Max Annual Debt Service (DSCR)</t>
+        </is>
+      </c>
+      <c r="B16" s="28">
+        <f>B10/B5</f>
+        <v/>
+      </c>
+      <c r="C16" s="15">
+        <f> NOI / target DSCR</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Max Loan — DSCR constrained</t>
+        </is>
+      </c>
+      <c r="B17" s="28">
+        <f>B16/B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Max Loan — Debt-Yield constrained</t>
+        </is>
+      </c>
+      <c r="B18" s="28">
+        <f>B10/B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Binding Max Loan</t>
+        </is>
+      </c>
+      <c r="B19" s="30">
+        <f>MIN(B17,B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>the lesser of the two</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>MAXIMUM PURCHASE PRICE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Max Price — DSCR/Debt-Yield (at Max LTV)</t>
+        </is>
+      </c>
+      <c r="B22" s="32">
+        <f>B19/B7</f>
+        <v/>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>price the debt supports at your LTV</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Current Purchase Price</t>
+        </is>
+      </c>
+      <c r="B23" s="28">
+        <f>Underwriting!B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Price Headroom ($)</t>
+        </is>
+      </c>
+      <c r="B24" s="9">
+        <f>B22-B23</f>
+        <v/>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>positive = room to pay more; negative = overpaying</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Price Headroom (%)</t>
+        </is>
+      </c>
+      <c r="B25" s="14">
+        <f>B24/B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>DSCR at Current Price</t>
+        </is>
+      </c>
+      <c r="B26" s="35">
+        <f>Underwriting!B65</f>
+        <v/>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>for reference (target above)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Required Equity at Max Price</t>
+        </is>
+      </c>
+      <c r="B27" s="28">
+        <f>B22*(1-B7)</f>
+        <v/>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>down payment if you buy at the max</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>READ: if Headroom is negative, the price is higher than the income can safely finance at your target DSCR — you'd need more equity, a lower rate, or a price cut.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1211,29 +1682,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>DEAL SCORECARD — GOOD / OK / BAD</t>
+          <t>DEAL SCORECARD — AJ KUKRA 'RV PARK PROFIT BLUEPRINT'</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Defaults are industry-standard RV-park benchmarks. The GREEN cutoff cells are EDITABLE — replace them with your own (or a course/video's) numbers and the ratings update live.</t>
+          <t>AJ's framework. Underwrite to the NORMALIZED NOI (see Normalization tab) before trusting these. GREEN cutoff cells are editable. Source: AJ Kukra, RV Park Profit Blueprint workshop.</t>
         </is>
       </c>
     </row>
@@ -1250,358 +1722,311 @@
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>Better</t>
+          <t>AJ's rule</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>Good cutoff</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
-          <t>OK cutoff</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
+          <t>(band)</t>
+        </is>
+      </c>
+      <c r="G4" s="16" t="inlineStr">
+        <is>
+          <t>(band)</t>
+        </is>
+      </c>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
           <t>Rating</t>
         </is>
       </c>
-      <c r="G4" s="16" t="inlineStr">
-        <is>
-          <t>Pts</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="17" t="inlineStr">
-        <is>
-          <t>Going-in Cap Rate</t>
-        </is>
-      </c>
-      <c r="B5" s="14">
-        <f>Underwriting!B62</f>
-        <v/>
-      </c>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D5" s="19" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E5" s="19" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F5" s="20">
-        <f>IF(B5&gt;=D5,"GOOD",IF(B5&gt;=E5,"OK","BAD"))</f>
-        <v/>
-      </c>
-      <c r="G5" s="18">
-        <f>IF(F5="GOOD",2,IF(F5="OK",1,0))</f>
-        <v/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>GO / NO-GO METRICS  (after normalizing the NOI)</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>Cash-on-Cash (Yr 1)</t>
-        </is>
-      </c>
-      <c r="B6" s="14">
-        <f>Underwriting!B64</f>
-        <v/>
-      </c>
-      <c r="C6" s="18" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>DSCR</t>
+        </is>
+      </c>
+      <c r="B6" s="18">
+        <f>Underwriting!B65</f>
+        <v/>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>AJ floor 1.35x to GO</t>
         </is>
       </c>
       <c r="D6" s="19" t="n">
-        <v>0.1</v>
+        <v>1.5</v>
       </c>
       <c r="E6" s="19" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="F6" s="20">
+        <v>1.35</v>
+      </c>
+      <c r="H6" s="20">
         <f>IF(B6&gt;=D6,"GOOD",IF(B6&gt;=E6,"OK","BAD"))</f>
-        <v/>
-      </c>
-      <c r="G6" s="18">
-        <f>IF(F6="GOOD",2,IF(F6="OK",1,0))</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>DSCR</t>
-        </is>
-      </c>
-      <c r="B7" s="21">
-        <f>Underwriting!B65</f>
-        <v/>
-      </c>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D7" s="22" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="E7" s="22" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="F7" s="20">
+          <t>Cash-on-Cash Return</t>
+        </is>
+      </c>
+      <c r="B7" s="14">
+        <f>Underwriting!B64</f>
+        <v/>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>AJ target 10%+ to GO</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H7" s="20">
         <f>IF(B7&gt;=D7,"GOOD",IF(B7&gt;=E7,"OK","BAD"))</f>
         <v/>
       </c>
-      <c r="G7" s="18">
-        <f>IF(F7="GOOD",2,IF(F7="OK",1,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>Debt Yield</t>
-        </is>
-      </c>
-      <c r="B8" s="14">
-        <f>Underwriting!B40/Underwriting!B54</f>
-        <v/>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D8" s="19" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E8" s="19" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F8" s="20">
-        <f>IF(B8&gt;=D8,"GOOD",IF(B8&gt;=E8,"OK","BAD"))</f>
-        <v/>
-      </c>
-      <c r="G8" s="18">
-        <f>IF(F8="GOOD",2,IF(F8="OK",1,0))</f>
-        <v/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>THE 5 QUICK HACKS  (screen any listing in ~2 min)</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>Cap Rate − Interest (spread)</t>
-        </is>
-      </c>
-      <c r="B9" s="14">
-        <f>Underwriting!B62-Underwriting!B45</f>
-        <v/>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D9" s="19" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="F9" s="20">
+          <t>1% Rule  (monthly gross / price)</t>
+        </is>
+      </c>
+      <c r="B9" s="10">
+        <f>(Underwriting!B24/12)/Underwriting!B9</f>
+        <v/>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>&gt;=1% likely good</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="H9" s="20">
         <f>IF(B9&gt;=D9,"GOOD",IF(B9&gt;=E9,"OK","BAD"))</f>
-        <v/>
-      </c>
-      <c r="G9" s="18">
-        <f>IF(F9="GOOD",2,IF(F9="OK",1,0))</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
         <is>
-          <t>Operating Expense Ratio</t>
-        </is>
-      </c>
-      <c r="B10" s="14">
-        <f>Underwriting!B36</f>
-        <v/>
-      </c>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>10x Rule — GRM  (price / annual gross)</t>
+        </is>
+      </c>
+      <c r="B10" s="18">
+        <f>Underwriting!B9/Underwriting!B24</f>
+        <v/>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>&lt;10 ideal; &gt;12 pricey</t>
         </is>
       </c>
       <c r="D10" s="19" t="n">
-        <v>0.4</v>
+        <v>10</v>
       </c>
       <c r="E10" s="19" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="F10" s="20">
+        <v>12</v>
+      </c>
+      <c r="H10" s="20">
         <f>IF(B10&lt;=D10,"GOOD",IF(B10&lt;=E10,"OK","BAD"))</f>
-        <v/>
-      </c>
-      <c r="G10" s="18">
-        <f>IF(F10="GOOD",2,IF(F10="OK",1,0))</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>Break-even Occupancy</t>
-        </is>
-      </c>
-      <c r="B11" s="14">
-        <f>Underwriting!B67</f>
-        <v/>
-      </c>
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>Quick DSCR  (NOI / (price x rate))</t>
+        </is>
+      </c>
+      <c r="B11" s="18">
+        <f>Underwriting!B40/(Underwriting!B9*Underwriting!B45)</f>
+        <v/>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>&gt;1.5 good; &lt;1.25 risk</t>
         </is>
       </c>
       <c r="D11" s="19" t="n">
-        <v>0.7</v>
+        <v>1.5</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F11" s="20">
-        <f>IF(B11&lt;=D11,"GOOD",IF(B11&lt;=E11,"OK","BAD"))</f>
-        <v/>
-      </c>
-      <c r="G11" s="18">
-        <f>IF(F11="GOOD",2,IF(F11="OK",1,0))</f>
+        <v>1.25</v>
+      </c>
+      <c r="H11" s="20">
+        <f>IF(B11&gt;=D11,"GOOD",IF(B11&gt;=E11,"OK","BAD"))</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="17" t="inlineStr">
         <is>
-          <t>Levered IRR</t>
+          <t>Expense Ratio  (OpEx / gross)</t>
         </is>
       </c>
       <c r="B12" s="14">
-        <f>'Pro Forma &amp; Returns'!B18</f>
-        <v/>
-      </c>
-      <c r="C12" s="18" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E12" s="19" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F12" s="20">
-        <f>IF(B12&gt;=D12,"GOOD",IF(B12&gt;=E12,"OK","BAD"))</f>
-        <v/>
-      </c>
-      <c r="G12" s="18">
-        <f>IF(F12="GOOD",2,IF(F12="OK",1,0))</f>
+        <f>Underwriting!B36</f>
+        <v/>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>35-65% healthy; &lt;30%=fiction</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E12" s="21" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F12" s="21" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G12" s="21" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H12" s="20">
+        <f>IF(OR(B12&lt;D12,B12&gt;G12),"BAD",IF(AND(B12&gt;=E12,B12&lt;=F12),"GOOD","OK"))</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>Equity Multiple</t>
-        </is>
-      </c>
-      <c r="B13" s="21">
-        <f>'Pro Forma &amp; Returns'!B19</f>
-        <v/>
-      </c>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D13" s="22" t="n">
-        <v>2</v>
-      </c>
-      <c r="E13" s="22" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F13" s="20">
+          <t>Leverage spread  (cap - interest)</t>
+        </is>
+      </c>
+      <c r="B13" s="14">
+        <f>Underwriting!B62-Underwriting!B45</f>
+        <v/>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>cap&gt;rate = positive leverage</t>
+        </is>
+      </c>
+      <c r="D13" s="21" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="20">
         <f>IF(B13&gt;=D13,"GOOD",IF(B13&gt;=E13,"OK","BAD"))</f>
         <v/>
       </c>
-      <c r="G13" s="18">
-        <f>IF(F13="GOOD",2,IF(F13="OK",1,0))</f>
-        <v/>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Expense Ratio is a BAND: below D = BAD (NOI likely inflated / 'fiction') · D-E and F-G = OK · E-F = GOOD (healthy) · above G = BAD.  D,E,F,G default to 30/35/65/70%.</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>OVERALL</t>
+          <t>VERDICT  (AJ's rule: both DSCR and Cash-on-Cash must clear)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Score</t>
-        </is>
-      </c>
-      <c r="B16" s="23">
-        <f>SUM(G5:G13)</f>
-        <v/>
-      </c>
-      <c r="C16" s="15">
-        <f>"of "&amp;(13-5+1)*2</f>
+          <t>DSCR clears floor?</t>
+        </is>
+      </c>
+      <c r="B16" s="20">
+        <f>IF(B6&gt;=E6,"YES","NO")</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Score %</t>
-        </is>
-      </c>
-      <c r="B17" s="14">
-        <f>B16/((13-5+1)*2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="24" t="inlineStr">
+          <t>Cash-on-Cash clears target?</t>
+        </is>
+      </c>
+      <c r="B17" s="20">
+        <f>IF(B7&gt;=D7,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>VERDICT</t>
         </is>
       </c>
-      <c r="B18" s="25">
-        <f>IF(B17&gt;=0.8,"STRONG DEAL",IF(B17&gt;=0.6,"OK — NEEDS WORK","PASS / BAD DEAL"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
-        <is>
-          <t>Scoring: GOOD=2, OK=1, BAD=0 pts. Verdict: &gt;=80% STRONG, 60-79% OK/NEEDS WORK, &lt;60% PASS. These are screening guides, not gospel — edit the cutoffs to match your strategy or market.</t>
+      <c r="B19" s="24">
+        <f>IF(AND(B6&gt;=E6,B7&gt;=D7),"GO - both clear",IF(OR(B6&gt;=E6,B7&gt;=D7),"CONDITIONAL - restructure","LIKELY NO-GO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Red flags (BAD ratings)</t>
+        </is>
+      </c>
+      <c r="B21" s="20">
+        <f>COUNTIF(H5:H13,"BAD")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>CONDITIONAL means restructure to save it (AJ's 3 levers): (1) lower price to your MAO, (2) ask the seller to carry a slice — blended rate drops, DSCR clears, CoC jumps, (3) more down payment. If none work and the seller won't budge, your underwriting just saved you from an expensive mistake.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A15:G15"/>
+  <mergeCells count="5">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A8:H8"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F13">
+  <conditionalFormatting sqref="H5:H13">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"GOOD"</formula>
     </cfRule>
@@ -1612,15 +2037,15 @@
       <formula>"BAD"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B18">
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
-      <formula>"STRONG DEAL"</formula>
+  <conditionalFormatting sqref="B19">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>LEFT($B$19,2)="GO"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
-      <formula>"OK — NEEDS WORK"</formula>
+    <cfRule type="expression" priority="5" dxfId="1">
+      <formula>ISNUMBER(SEARCH("CONDITIONAL",$B$19))</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2">
-      <formula>"PASS / BAD DEAL"</formula>
+    <cfRule type="expression" priority="6" dxfId="2">
+      <formula>ISNUMBER(SEARCH("NO-GO",$B$19))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1654,7 +2079,7 @@
           <t>Property Name</t>
         </is>
       </c>
-      <c r="B3" s="26" t="inlineStr">
+      <c r="B3" s="25" t="inlineStr">
         <is>
           <t>Enter property name</t>
         </is>
@@ -1671,7 +2096,7 @@
           <t>Location (City, ST)</t>
         </is>
       </c>
-      <c r="B4" s="26" t="inlineStr">
+      <c r="B4" s="25" t="inlineStr">
         <is>
           <t>City, ST</t>
         </is>
@@ -1683,7 +2108,7 @@
           <t>Analysis Date</t>
         </is>
       </c>
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
@@ -1702,7 +2127,7 @@
           <t>Number of RV Sites (pads)</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
+      <c r="B8" s="26" t="n">
         <v>50</v>
       </c>
       <c r="C8" s="15" t="inlineStr">
@@ -1717,7 +2142,7 @@
           <t>Purchase Price</t>
         </is>
       </c>
-      <c r="B9" s="28" t="n">
+      <c r="B9" s="27" t="n">
         <v>1500000</v>
       </c>
     </row>
@@ -1727,7 +2152,7 @@
           <t xml:space="preserve">  Price per Site</t>
         </is>
       </c>
-      <c r="B10" s="29">
+      <c r="B10" s="28">
         <f>B9/B8</f>
         <v/>
       </c>
@@ -1743,7 +2168,7 @@
           <t>Avg. Monthly Rent per Site</t>
         </is>
       </c>
-      <c r="B11" s="28" t="n">
+      <c r="B11" s="27" t="n">
         <v>450</v>
       </c>
       <c r="C11" s="15" t="inlineStr">
@@ -1758,7 +2183,7 @@
           <t>Vacancy &amp; Credit Loss %</t>
         </is>
       </c>
-      <c r="B12" s="19" t="n">
+      <c r="B12" s="21" t="n">
         <v>0.15</v>
       </c>
       <c r="C12" s="15" t="inlineStr">
@@ -1773,7 +2198,7 @@
           <t>Other Income (monthly)</t>
         </is>
       </c>
-      <c r="B13" s="28" t="n">
+      <c r="B13" s="27" t="n">
         <v>1500</v>
       </c>
       <c r="C13" s="15" t="inlineStr">
@@ -1788,7 +2213,7 @@
           <t>Management Fee (% of EGI)</t>
         </is>
       </c>
-      <c r="B14" s="19" t="n">
+      <c r="B14" s="21" t="n">
         <v>0.08</v>
       </c>
       <c r="C14" s="15" t="inlineStr">
@@ -1803,7 +2228,7 @@
           <t>Replacement Reserves / site / yr</t>
         </is>
       </c>
-      <c r="B15" s="28" t="n">
+      <c r="B15" s="27" t="n">
         <v>100</v>
       </c>
       <c r="C15" s="15" t="inlineStr">
@@ -1818,7 +2243,7 @@
           <t>Annual Rent Growth %</t>
         </is>
       </c>
-      <c r="B16" s="19" t="n">
+      <c r="B16" s="21" t="n">
         <v>0.03</v>
       </c>
       <c r="C16" s="15" t="inlineStr">
@@ -1833,7 +2258,7 @@
           <t>Annual Expense Growth %</t>
         </is>
       </c>
-      <c r="B17" s="19" t="n">
+      <c r="B17" s="21" t="n">
         <v>0.025</v>
       </c>
       <c r="C17" s="15" t="inlineStr">
@@ -1848,7 +2273,7 @@
           <t>Use Detailed Income Build? (Y/N)</t>
         </is>
       </c>
-      <c r="B18" s="30" t="inlineStr">
+      <c r="B18" s="29" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1872,7 +2297,7 @@
           <t>Gross Potential Rent (GPR)</t>
         </is>
       </c>
-      <c r="B21" s="29">
+      <c r="B21" s="28">
         <f>IF(B18="Y",'Income Detail'!E30,B8*B11*12)</f>
         <v/>
       </c>
@@ -1888,7 +2313,7 @@
           <t>Less: Vacancy &amp; Credit Loss</t>
         </is>
       </c>
-      <c r="B22" s="29">
+      <c r="B22" s="28">
         <f>-B21*B12</f>
         <v/>
       </c>
@@ -1899,7 +2324,7 @@
           <t>Plus: Other Income</t>
         </is>
       </c>
-      <c r="B23" s="29">
+      <c r="B23" s="28">
         <f>B13*12</f>
         <v/>
       </c>
@@ -1910,7 +2335,7 @@
           <t>Effective Gross Income (EGI)</t>
         </is>
       </c>
-      <c r="B24" s="31">
+      <c r="B24" s="30">
         <f>B21+B22+B23</f>
         <v/>
       </c>
@@ -1928,7 +2353,7 @@
           <t>Property Taxes</t>
         </is>
       </c>
-      <c r="B27" s="28" t="n">
+      <c r="B27" s="27" t="n">
         <v>18000</v>
       </c>
     </row>
@@ -1938,7 +2363,7 @@
           <t>Insurance</t>
         </is>
       </c>
-      <c r="B28" s="28" t="n">
+      <c r="B28" s="27" t="n">
         <v>9000</v>
       </c>
     </row>
@@ -1948,7 +2373,7 @@
           <t>Utilities (water/sewer/trash/elec)</t>
         </is>
       </c>
-      <c r="B29" s="28" t="n">
+      <c r="B29" s="27" t="n">
         <v>36000</v>
       </c>
       <c r="C29" s="15" t="inlineStr">
@@ -1963,7 +2388,7 @@
           <t>Repairs &amp; Maintenance</t>
         </is>
       </c>
-      <c r="B30" s="28" t="n">
+      <c r="B30" s="27" t="n">
         <v>15000</v>
       </c>
     </row>
@@ -1973,7 +2398,7 @@
           <t>Payroll / Onsite Manager</t>
         </is>
       </c>
-      <c r="B31" s="28" t="n">
+      <c r="B31" s="27" t="n">
         <v>24000</v>
       </c>
     </row>
@@ -1983,7 +2408,7 @@
           <t>Marketing, Admin, Office</t>
         </is>
       </c>
-      <c r="B32" s="28" t="n">
+      <c r="B32" s="27" t="n">
         <v>8000</v>
       </c>
     </row>
@@ -1993,7 +2418,7 @@
           <t>Management Fee</t>
         </is>
       </c>
-      <c r="B33" s="29">
+      <c r="B33" s="28">
         <f>B14*B24</f>
         <v/>
       </c>
@@ -2008,7 +2433,7 @@
           <t>Replacement Reserves</t>
         </is>
       </c>
-      <c r="B34" s="29">
+      <c r="B34" s="28">
         <f>B15*B8</f>
         <v/>
       </c>
@@ -2019,7 +2444,7 @@
           <t>Total Operating Expenses</t>
         </is>
       </c>
-      <c r="B35" s="31">
+      <c r="B35" s="30">
         <f>SUM(B27:B34)</f>
         <v/>
       </c>
@@ -2030,7 +2455,7 @@
           <t>Operating Expense Ratio</t>
         </is>
       </c>
-      <c r="B36" s="32">
+      <c r="B36" s="31">
         <f>B35/B24</f>
         <v/>
       </c>
@@ -2046,7 +2471,7 @@
           <t>Expenses per Site</t>
         </is>
       </c>
-      <c r="B37" s="29">
+      <c r="B37" s="28">
         <f>B35/B8</f>
         <v/>
       </c>
@@ -2064,7 +2489,7 @@
           <t>Net Operating Income (NOI)</t>
         </is>
       </c>
-      <c r="B40" s="33">
+      <c r="B40" s="32">
         <f>B24-B35</f>
         <v/>
       </c>
@@ -2075,7 +2500,7 @@
           <t>NOI per Site</t>
         </is>
       </c>
-      <c r="B41" s="29">
+      <c r="B41" s="28">
         <f>B40/B8</f>
         <v/>
       </c>
@@ -2093,7 +2518,7 @@
           <t>Loan-to-Value (LTV) %</t>
         </is>
       </c>
-      <c r="B44" s="19" t="n">
+      <c r="B44" s="21" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -2103,7 +2528,7 @@
           <t>Interest Rate %</t>
         </is>
       </c>
-      <c r="B45" s="34" t="n">
+      <c r="B45" s="22" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="C45" s="15" t="inlineStr">
@@ -2118,7 +2543,7 @@
           <t>Amortization (years)</t>
         </is>
       </c>
-      <c r="B46" s="27" t="n">
+      <c r="B46" s="26" t="n">
         <v>25</v>
       </c>
     </row>
@@ -2128,7 +2553,7 @@
           <t>Closing Costs %</t>
         </is>
       </c>
-      <c r="B47" s="19" t="n">
+      <c r="B47" s="21" t="n">
         <v>0.03</v>
       </c>
       <c r="C47" s="15" t="inlineStr">
@@ -2143,7 +2568,7 @@
           <t>Initial CapEx / Rehab</t>
         </is>
       </c>
-      <c r="B48" s="28" t="n">
+      <c r="B48" s="27" t="n">
         <v>50000</v>
       </c>
       <c r="C48" s="15" t="inlineStr">
@@ -2158,7 +2583,7 @@
           <t>Hold Period (years)</t>
         </is>
       </c>
-      <c r="B49" s="27" t="n">
+      <c r="B49" s="26" t="n">
         <v>5</v>
       </c>
       <c r="C49" s="15" t="inlineStr">
@@ -2173,7 +2598,7 @@
           <t>Exit Cap Rate %</t>
         </is>
       </c>
-      <c r="B50" s="34" t="n">
+      <c r="B50" s="22" t="n">
         <v>0.08500000000000001</v>
       </c>
       <c r="C50" s="15" t="inlineStr">
@@ -2188,7 +2613,7 @@
           <t>Selling Costs %</t>
         </is>
       </c>
-      <c r="B51" s="19" t="n">
+      <c r="B51" s="21" t="n">
         <v>0.05</v>
       </c>
       <c r="C51" s="15" t="inlineStr">
@@ -2210,7 +2635,7 @@
           <t>Loan Amount</t>
         </is>
       </c>
-      <c r="B54" s="29">
+      <c r="B54" s="28">
         <f>B9*B44</f>
         <v/>
       </c>
@@ -2221,7 +2646,7 @@
           <t>Down Payment (Equity)</t>
         </is>
       </c>
-      <c r="B55" s="29">
+      <c r="B55" s="28">
         <f>B9-B54</f>
         <v/>
       </c>
@@ -2232,7 +2657,7 @@
           <t>Closing Costs</t>
         </is>
       </c>
-      <c r="B56" s="29">
+      <c r="B56" s="28">
         <f>B9*B47</f>
         <v/>
       </c>
@@ -2243,7 +2668,7 @@
           <t>Total Cash Required</t>
         </is>
       </c>
-      <c r="B57" s="31">
+      <c r="B57" s="30">
         <f>B55+B56+B48</f>
         <v/>
       </c>
@@ -2254,7 +2679,7 @@
           <t>Monthly Debt Payment</t>
         </is>
       </c>
-      <c r="B58" s="29">
+      <c r="B58" s="28">
         <f>PMT(B45/12,B46*12,-B54)</f>
         <v/>
       </c>
@@ -2283,7 +2708,7 @@
           <t>Going-in Cap Rate</t>
         </is>
       </c>
-      <c r="B62" s="35">
+      <c r="B62" s="33">
         <f>B40/B9</f>
         <v/>
       </c>
@@ -2299,7 +2724,7 @@
           <t>Cash Flow Before Tax (CFBT)</t>
         </is>
       </c>
-      <c r="B63" s="33">
+      <c r="B63" s="32">
         <f>B40-B59</f>
         <v/>
       </c>
@@ -2310,7 +2735,7 @@
           <t>Cash-on-Cash Return</t>
         </is>
       </c>
-      <c r="B64" s="35">
+      <c r="B64" s="33">
         <f>B63/B57</f>
         <v/>
       </c>
@@ -2326,7 +2751,7 @@
           <t>Debt Service Coverage (DSCR)</t>
         </is>
       </c>
-      <c r="B65" s="36">
+      <c r="B65" s="34">
         <f>B40/B59</f>
         <v/>
       </c>
@@ -2342,7 +2767,7 @@
           <t>Gross Rent Multiplier (GRM)</t>
         </is>
       </c>
-      <c r="B66" s="37">
+      <c r="B66" s="35">
         <f>B9/B21</f>
         <v/>
       </c>
@@ -2353,7 +2778,7 @@
           <t>Break-even Occupancy</t>
         </is>
       </c>
-      <c r="B67" s="32">
+      <c r="B67" s="31">
         <f>(B35+B59)/(B21+B23)</f>
         <v/>
       </c>
@@ -2369,7 +2794,7 @@
           <t>Debt Yield</t>
         </is>
       </c>
-      <c r="B68" s="32">
+      <c r="B68" s="31">
         <f>B40/B54</f>
         <v/>
       </c>
@@ -2400,6 +2825,428 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>NORMALIZE THE NOI — BUILD YOUR OWN NUMBERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>AJ: the T12 is your starting point but never trusted as-is. Enter the SELLER'S reported figures (yellow); the Normalized column rebuilds the NOI with AJ's 4 adjustments. Source: AJ Kukra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>AJ'S NORMALIZATION RULES (editable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Management Fee (% of EGI)</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>self-managed owners show little or none</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance (% of EGI)</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>or use the prior-year actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>CapEx / Reserves (% of EGI)</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>a real cost that's rarely in the P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Property Tax bump (%)</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>taxes reset on sale in disclosure states</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>INCOME</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Effective Gross Income (EGI)</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="n">
+        <v>247500</v>
+      </c>
+      <c r="C11" s="9">
+        <f>B11</f>
+        <v/>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>seller's real top line (AJ: gross income = EGI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>OPERATING EXPENSES</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Seller Reported</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Normalized</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>AJ adjustment</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Property Taxes</t>
+        </is>
+      </c>
+      <c r="B15" s="27" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C15" s="36">
+        <f>B15*(1+B8)</f>
+        <v/>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>+20%: resets on sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="B16" s="27" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C16" s="36">
+        <f>B16</f>
+        <v/>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>pass-through</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Utilities (W/S/trash/elec)</t>
+        </is>
+      </c>
+      <c r="B17" s="27" t="n">
+        <v>38000</v>
+      </c>
+      <c r="C17" s="36">
+        <f>B17</f>
+        <v/>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>pass-through</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Repairs &amp; Maintenance</t>
+        </is>
+      </c>
+      <c r="B18" s="27" t="n">
+        <v>4200</v>
+      </c>
+      <c r="C18" s="36">
+        <f>MAX(B18,B6*B11)</f>
+        <v/>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>use &gt;=5%% of EGI (deferred maint)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Management Fee</t>
+        </is>
+      </c>
+      <c r="B19" s="27" t="n">
+        <v>3500</v>
+      </c>
+      <c r="C19" s="36">
+        <f>MAX(B19,B5*B11)</f>
+        <v/>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>use &gt;=10%% of EGI (self-mgmt understates)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>CapEx / Reserves</t>
+        </is>
+      </c>
+      <c r="B20" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="36">
+        <f>MAX(B20,B7*B11)</f>
+        <v/>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>add &gt;=3%% of EGI (never in P&amp;L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Payroll / Onsite</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="36">
+        <f>B21</f>
+        <v/>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>pass-through</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Marketing / Admin / Other</t>
+        </is>
+      </c>
+      <c r="B22" s="27" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C22" s="36">
+        <f>B22</f>
+        <v/>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>pass-through</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Total Operating Expenses</t>
+        </is>
+      </c>
+      <c r="B23" s="30">
+        <f>SUM(B15:B22)</f>
+        <v/>
+      </c>
+      <c r="C23" s="30">
+        <f>SUM(C15:C22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>Expense Ratio</t>
+        </is>
+      </c>
+      <c r="B24" s="37">
+        <f>B23/B11</f>
+        <v/>
+      </c>
+      <c r="C24" s="37">
+        <f>C23/C11</f>
+        <v/>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>AJ: under 30% means something's missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>RESULT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Net Operating Income (NOI)</t>
+        </is>
+      </c>
+      <c r="B27" s="32">
+        <f>B11-B23</f>
+        <v/>
+      </c>
+      <c r="C27" s="32">
+        <f>C11-C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>NOI Haircut ($ cut from seller's NOI)</t>
+        </is>
+      </c>
+      <c r="C28" s="9">
+        <f>B27-C27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>NOI Haircut (%)</t>
+        </is>
+      </c>
+      <c r="C29" s="37">
+        <f>(B27-C27)/B27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Valuation Cap Rate (for overpayment calc)</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="38" t="inlineStr">
+        <is>
+          <t>OVERPAYMENT RISK  (haircut / cap rate)</t>
+        </is>
+      </c>
+      <c r="C31" s="39">
+        <f>(B27-C27)/B30</f>
+        <v/>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>AJ: a small NOI cut = a huge price difference</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>NEXT: carry the NORMALIZED expense figures (column C) into the Underwriting tab so every metric and the Deal Scorecard reflect YOUR numbers, not the seller's.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A13:D13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2464,16 +3311,16 @@
           <t>Monthly tenants</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
+      <c r="B6" s="26" t="n">
         <v>30</v>
       </c>
-      <c r="C6" s="28" t="n">
+      <c r="C6" s="27" t="n">
         <v>450</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="21" t="n">
         <v>0.95</v>
       </c>
-      <c r="E6" s="29">
+      <c r="E6" s="28">
         <f>B6*C6*12*D6</f>
         <v/>
       </c>
@@ -2484,16 +3331,16 @@
           <t>Annual / seasonal leases</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
+      <c r="B7" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="C7" s="28" t="n">
+      <c r="C7" s="27" t="n">
         <v>400</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="21" t="n">
         <v>0.9</v>
       </c>
-      <c r="E7" s="29">
+      <c r="E7" s="28">
         <f>B7*C7*12*D7</f>
         <v/>
       </c>
@@ -2508,7 +3355,7 @@
         <f>SUM(B6:B7)</f>
         <v/>
       </c>
-      <c r="E8" s="31">
+      <c r="E8" s="30">
         <f>SUM(E6:E7)</f>
         <v/>
       </c>
@@ -2526,7 +3373,7 @@
           <t># Transient sites</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
+      <c r="B11" s="26" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2536,7 +3383,7 @@
           <t>Avg nightly rate</t>
         </is>
       </c>
-      <c r="B12" s="28" t="n">
+      <c r="B12" s="27" t="n">
         <v>55</v>
       </c>
     </row>
@@ -2568,13 +3415,13 @@
           <t>Jan</t>
         </is>
       </c>
-      <c r="B15" s="38" t="n">
+      <c r="B15" s="40" t="n">
         <v>31</v>
       </c>
-      <c r="C15" s="19" t="n">
+      <c r="C15" s="21" t="n">
         <v>0.3</v>
       </c>
-      <c r="D15" s="29">
+      <c r="D15" s="28">
         <f>$B$11*$B$12*B15*C15</f>
         <v/>
       </c>
@@ -2585,13 +3432,13 @@
           <t>Feb</t>
         </is>
       </c>
-      <c r="B16" s="38" t="n">
+      <c r="B16" s="40" t="n">
         <v>28</v>
       </c>
-      <c r="C16" s="19" t="n">
+      <c r="C16" s="21" t="n">
         <v>0.3</v>
       </c>
-      <c r="D16" s="29">
+      <c r="D16" s="28">
         <f>$B$11*$B$12*B16*C16</f>
         <v/>
       </c>
@@ -2602,13 +3449,13 @@
           <t>Mar</t>
         </is>
       </c>
-      <c r="B17" s="38" t="n">
+      <c r="B17" s="40" t="n">
         <v>31</v>
       </c>
-      <c r="C17" s="19" t="n">
+      <c r="C17" s="21" t="n">
         <v>0.45</v>
       </c>
-      <c r="D17" s="29">
+      <c r="D17" s="28">
         <f>$B$11*$B$12*B17*C17</f>
         <v/>
       </c>
@@ -2619,13 +3466,13 @@
           <t>Apr</t>
         </is>
       </c>
-      <c r="B18" s="38" t="n">
+      <c r="B18" s="40" t="n">
         <v>30</v>
       </c>
-      <c r="C18" s="19" t="n">
+      <c r="C18" s="21" t="n">
         <v>0.55</v>
       </c>
-      <c r="D18" s="29">
+      <c r="D18" s="28">
         <f>$B$11*$B$12*B18*C18</f>
         <v/>
       </c>
@@ -2636,13 +3483,13 @@
           <t>May</t>
         </is>
       </c>
-      <c r="B19" s="38" t="n">
+      <c r="B19" s="40" t="n">
         <v>31</v>
       </c>
-      <c r="C19" s="19" t="n">
+      <c r="C19" s="21" t="n">
         <v>0.7</v>
       </c>
-      <c r="D19" s="29">
+      <c r="D19" s="28">
         <f>$B$11*$B$12*B19*C19</f>
         <v/>
       </c>
@@ -2653,13 +3500,13 @@
           <t>Jun</t>
         </is>
       </c>
-      <c r="B20" s="38" t="n">
+      <c r="B20" s="40" t="n">
         <v>30</v>
       </c>
-      <c r="C20" s="19" t="n">
+      <c r="C20" s="21" t="n">
         <v>0.85</v>
       </c>
-      <c r="D20" s="29">
+      <c r="D20" s="28">
         <f>$B$11*$B$12*B20*C20</f>
         <v/>
       </c>
@@ -2670,13 +3517,13 @@
           <t>Jul</t>
         </is>
       </c>
-      <c r="B21" s="38" t="n">
+      <c r="B21" s="40" t="n">
         <v>31</v>
       </c>
-      <c r="C21" s="19" t="n">
+      <c r="C21" s="21" t="n">
         <v>0.95</v>
       </c>
-      <c r="D21" s="29">
+      <c r="D21" s="28">
         <f>$B$11*$B$12*B21*C21</f>
         <v/>
       </c>
@@ -2687,13 +3534,13 @@
           <t>Aug</t>
         </is>
       </c>
-      <c r="B22" s="38" t="n">
+      <c r="B22" s="40" t="n">
         <v>31</v>
       </c>
-      <c r="C22" s="19" t="n">
+      <c r="C22" s="21" t="n">
         <v>0.95</v>
       </c>
-      <c r="D22" s="29">
+      <c r="D22" s="28">
         <f>$B$11*$B$12*B22*C22</f>
         <v/>
       </c>
@@ -2704,13 +3551,13 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="B23" s="38" t="n">
+      <c r="B23" s="40" t="n">
         <v>30</v>
       </c>
-      <c r="C23" s="19" t="n">
+      <c r="C23" s="21" t="n">
         <v>0.75</v>
       </c>
-      <c r="D23" s="29">
+      <c r="D23" s="28">
         <f>$B$11*$B$12*B23*C23</f>
         <v/>
       </c>
@@ -2721,13 +3568,13 @@
           <t>Oct</t>
         </is>
       </c>
-      <c r="B24" s="38" t="n">
+      <c r="B24" s="40" t="n">
         <v>31</v>
       </c>
-      <c r="C24" s="19" t="n">
+      <c r="C24" s="21" t="n">
         <v>0.55</v>
       </c>
-      <c r="D24" s="29">
+      <c r="D24" s="28">
         <f>$B$11*$B$12*B24*C24</f>
         <v/>
       </c>
@@ -2738,13 +3585,13 @@
           <t>Nov</t>
         </is>
       </c>
-      <c r="B25" s="38" t="n">
+      <c r="B25" s="40" t="n">
         <v>30</v>
       </c>
-      <c r="C25" s="19" t="n">
+      <c r="C25" s="21" t="n">
         <v>0.35</v>
       </c>
-      <c r="D25" s="29">
+      <c r="D25" s="28">
         <f>$B$11*$B$12*B25*C25</f>
         <v/>
       </c>
@@ -2755,13 +3602,13 @@
           <t>Dec</t>
         </is>
       </c>
-      <c r="B26" s="38" t="n">
+      <c r="B26" s="40" t="n">
         <v>31</v>
       </c>
-      <c r="C26" s="19" t="n">
+      <c r="C26" s="21" t="n">
         <v>0.3</v>
       </c>
-      <c r="D26" s="29">
+      <c r="D26" s="28">
         <f>$B$11*$B$12*B26*C26</f>
         <v/>
       </c>
@@ -2772,7 +3619,7 @@
           <t>Subtotal — transient</t>
         </is>
       </c>
-      <c r="D27" s="31">
+      <c r="D27" s="30">
         <f>SUM(D15:D26)</f>
         <v/>
       </c>
@@ -2783,7 +3630,7 @@
           <t>Avg transient occupancy</t>
         </is>
       </c>
-      <c r="C28" s="32">
+      <c r="C28" s="31">
         <f>SUMPRODUCT(B15:B26,C15:C26)/SUM(B15:B26)</f>
         <v/>
       </c>
@@ -2801,7 +3648,7 @@
           <t>Total Potential Annual Site Revenue</t>
         </is>
       </c>
-      <c r="E30" s="33">
+      <c r="E30" s="32">
         <f>E8+D27</f>
         <v/>
       </c>
@@ -2812,7 +3659,7 @@
           <t>Total sites in build</t>
         </is>
       </c>
-      <c r="E31" s="39">
+      <c r="E31" s="41">
         <f>B8+B11</f>
         <v/>
       </c>
@@ -2823,7 +3670,7 @@
           <t>Implied blended monthly rent / site</t>
         </is>
       </c>
-      <c r="E32" s="29">
+      <c r="E32" s="28">
         <f>E30/E31/12</f>
         <v/>
       </c>
@@ -2846,7 +3693,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2903,14 +3750,14 @@
           <t>Gross Potential Rent</t>
         </is>
       </c>
-      <c r="B5" s="28" t="n">
+      <c r="B5" s="27" t="n">
         <v>240000</v>
       </c>
-      <c r="C5" s="29">
+      <c r="C5" s="28">
         <f>Underwriting!B21</f>
         <v/>
       </c>
-      <c r="D5" s="29">
+      <c r="D5" s="28">
         <f>C5-B5</f>
         <v/>
       </c>
@@ -2921,14 +3768,14 @@
           <t>Vacancy &amp; Credit Loss</t>
         </is>
       </c>
-      <c r="B6" s="28" t="n">
+      <c r="B6" s="27" t="n">
         <v>-48000</v>
       </c>
-      <c r="C6" s="29">
+      <c r="C6" s="28">
         <f>Underwriting!B22</f>
         <v/>
       </c>
-      <c r="D6" s="29">
+      <c r="D6" s="28">
         <f>C6-B6</f>
         <v/>
       </c>
@@ -2939,14 +3786,14 @@
           <t>Other Income</t>
         </is>
       </c>
-      <c r="B7" s="28" t="n">
+      <c r="B7" s="27" t="n">
         <v>12000</v>
       </c>
-      <c r="C7" s="29">
+      <c r="C7" s="28">
         <f>Underwriting!B23</f>
         <v/>
       </c>
-      <c r="D7" s="29">
+      <c r="D7" s="28">
         <f>C7-B7</f>
         <v/>
       </c>
@@ -2957,15 +3804,15 @@
           <t>Effective Gross Income</t>
         </is>
       </c>
-      <c r="B8" s="31">
+      <c r="B8" s="30">
         <f>B5+B6+B7</f>
         <v/>
       </c>
-      <c r="C8" s="31">
+      <c r="C8" s="30">
         <f>Underwriting!B24</f>
         <v/>
       </c>
-      <c r="D8" s="29">
+      <c r="D8" s="28">
         <f>C8-B8</f>
         <v/>
       </c>
@@ -2976,14 +3823,14 @@
           <t>Property Taxes</t>
         </is>
       </c>
-      <c r="B9" s="28" t="n">
+      <c r="B9" s="27" t="n">
         <v>12000</v>
       </c>
-      <c r="C9" s="29">
+      <c r="C9" s="28">
         <f>Underwriting!B27</f>
         <v/>
       </c>
-      <c r="D9" s="29">
+      <c r="D9" s="28">
         <f>C9-B9</f>
         <v/>
       </c>
@@ -2994,14 +3841,14 @@
           <t>Insurance</t>
         </is>
       </c>
-      <c r="B10" s="28" t="n">
+      <c r="B10" s="27" t="n">
         <v>8000</v>
       </c>
-      <c r="C10" s="29">
+      <c r="C10" s="28">
         <f>Underwriting!B28</f>
         <v/>
       </c>
-      <c r="D10" s="29">
+      <c r="D10" s="28">
         <f>C10-B10</f>
         <v/>
       </c>
@@ -3012,14 +3859,14 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="B11" s="28" t="n">
+      <c r="B11" s="27" t="n">
         <v>38000</v>
       </c>
-      <c r="C11" s="29">
+      <c r="C11" s="28">
         <f>Underwriting!B29</f>
         <v/>
       </c>
-      <c r="D11" s="29">
+      <c r="D11" s="28">
         <f>C11-B11</f>
         <v/>
       </c>
@@ -3030,14 +3877,14 @@
           <t>Repairs &amp; Maintenance</t>
         </is>
       </c>
-      <c r="B12" s="28" t="n">
+      <c r="B12" s="27" t="n">
         <v>20000</v>
       </c>
-      <c r="C12" s="29">
+      <c r="C12" s="28">
         <f>Underwriting!B30</f>
         <v/>
       </c>
-      <c r="D12" s="29">
+      <c r="D12" s="28">
         <f>C12-B12</f>
         <v/>
       </c>
@@ -3048,14 +3895,14 @@
           <t>Payroll / Onsite Mgr</t>
         </is>
       </c>
-      <c r="B13" s="28" t="n">
+      <c r="B13" s="27" t="n">
         <v>20000</v>
       </c>
-      <c r="C13" s="29">
+      <c r="C13" s="28">
         <f>Underwriting!B31</f>
         <v/>
       </c>
-      <c r="D13" s="29">
+      <c r="D13" s="28">
         <f>C13-B13</f>
         <v/>
       </c>
@@ -3066,14 +3913,14 @@
           <t>Marketing, Admin, Office</t>
         </is>
       </c>
-      <c r="B14" s="28" t="n">
+      <c r="B14" s="27" t="n">
         <v>6000</v>
       </c>
-      <c r="C14" s="29">
+      <c r="C14" s="28">
         <f>Underwriting!B32</f>
         <v/>
       </c>
-      <c r="D14" s="29">
+      <c r="D14" s="28">
         <f>C14-B14</f>
         <v/>
       </c>
@@ -3084,14 +3931,14 @@
           <t>Management Fee</t>
         </is>
       </c>
-      <c r="B15" s="28" t="n">
+      <c r="B15" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="28">
         <f>Underwriting!B33</f>
         <v/>
       </c>
-      <c r="D15" s="29">
+      <c r="D15" s="28">
         <f>C15-B15</f>
         <v/>
       </c>
@@ -3102,14 +3949,14 @@
           <t>Replacement Reserves</t>
         </is>
       </c>
-      <c r="B16" s="28" t="n">
+      <c r="B16" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="29">
+      <c r="C16" s="28">
         <f>Underwriting!B34</f>
         <v/>
       </c>
-      <c r="D16" s="29">
+      <c r="D16" s="28">
         <f>C16-B16</f>
         <v/>
       </c>
@@ -3120,15 +3967,15 @@
           <t>Total Operating Expenses</t>
         </is>
       </c>
-      <c r="B17" s="31">
+      <c r="B17" s="30">
         <f>SUM(B9:B16)</f>
         <v/>
       </c>
-      <c r="C17" s="31">
+      <c r="C17" s="30">
         <f>Underwriting!B35</f>
         <v/>
       </c>
-      <c r="D17" s="29">
+      <c r="D17" s="28">
         <f>C17-B17</f>
         <v/>
       </c>
@@ -3139,15 +3986,15 @@
           <t>Net Operating Income</t>
         </is>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="32">
         <f>B8-B17</f>
         <v/>
       </c>
-      <c r="C18" s="33">
+      <c r="C18" s="32">
         <f>Underwriting!B40</f>
         <v/>
       </c>
-      <c r="D18" s="29">
+      <c r="D18" s="28">
         <f>C18-B18</f>
         <v/>
       </c>
@@ -3158,11 +4005,11 @@
           <t>Cap Rate at Purchase Price</t>
         </is>
       </c>
-      <c r="B20" s="35">
+      <c r="B20" s="33">
         <f>B18/Underwriting!B9</f>
         <v/>
       </c>
-      <c r="C20" s="35">
+      <c r="C20" s="33">
         <f>Underwriting!B62</f>
         <v/>
       </c>
@@ -3182,7 +4029,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3213,7 +4060,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="40" t="inlineStr">
+      <c r="A3" s="42" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
@@ -3258,43 +4105,43 @@
           <t>Gross Potential Rent</t>
         </is>
       </c>
-      <c r="C5" s="29">
+      <c r="C5" s="28">
         <f>Underwriting!B21*(1+Underwriting!B16)^0</f>
         <v/>
       </c>
-      <c r="D5" s="29">
+      <c r="D5" s="28">
         <f>Underwriting!B21*(1+Underwriting!B16)^1</f>
         <v/>
       </c>
-      <c r="E5" s="29">
+      <c r="E5" s="28">
         <f>Underwriting!B21*(1+Underwriting!B16)^2</f>
         <v/>
       </c>
-      <c r="F5" s="29">
+      <c r="F5" s="28">
         <f>Underwriting!B21*(1+Underwriting!B16)^3</f>
         <v/>
       </c>
-      <c r="G5" s="29">
+      <c r="G5" s="28">
         <f>Underwriting!B21*(1+Underwriting!B16)^4</f>
         <v/>
       </c>
-      <c r="H5" s="29">
+      <c r="H5" s="28">
         <f>Underwriting!B21*(1+Underwriting!B16)^5</f>
         <v/>
       </c>
-      <c r="I5" s="29">
+      <c r="I5" s="28">
         <f>Underwriting!B21*(1+Underwriting!B16)^6</f>
         <v/>
       </c>
-      <c r="J5" s="29">
+      <c r="J5" s="28">
         <f>Underwriting!B21*(1+Underwriting!B16)^7</f>
         <v/>
       </c>
-      <c r="K5" s="29">
+      <c r="K5" s="28">
         <f>Underwriting!B21*(1+Underwriting!B16)^8</f>
         <v/>
       </c>
-      <c r="L5" s="29">
+      <c r="L5" s="28">
         <f>Underwriting!B21*(1+Underwriting!B16)^9</f>
         <v/>
       </c>
@@ -3305,43 +4152,43 @@
           <t>Less: Vacancy &amp; Credit Loss</t>
         </is>
       </c>
-      <c r="C6" s="29">
+      <c r="C6" s="28">
         <f>-C5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="D6" s="29">
+      <c r="D6" s="28">
         <f>-D5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="E6" s="29">
+      <c r="E6" s="28">
         <f>-E5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="F6" s="29">
+      <c r="F6" s="28">
         <f>-F5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="G6" s="29">
+      <c r="G6" s="28">
         <f>-G5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="H6" s="29">
+      <c r="H6" s="28">
         <f>-H5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="I6" s="29">
+      <c r="I6" s="28">
         <f>-I5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="J6" s="29">
+      <c r="J6" s="28">
         <f>-J5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="K6" s="29">
+      <c r="K6" s="28">
         <f>-K5*Underwriting!B12</f>
         <v/>
       </c>
-      <c r="L6" s="29">
+      <c r="L6" s="28">
         <f>-L5*Underwriting!B12</f>
         <v/>
       </c>
@@ -3352,43 +4199,43 @@
           <t>Other Income</t>
         </is>
       </c>
-      <c r="C7" s="29">
+      <c r="C7" s="28">
         <f>Underwriting!B23*(1+Underwriting!B16)^0</f>
         <v/>
       </c>
-      <c r="D7" s="29">
+      <c r="D7" s="28">
         <f>Underwriting!B23*(1+Underwriting!B16)^1</f>
         <v/>
       </c>
-      <c r="E7" s="29">
+      <c r="E7" s="28">
         <f>Underwriting!B23*(1+Underwriting!B16)^2</f>
         <v/>
       </c>
-      <c r="F7" s="29">
+      <c r="F7" s="28">
         <f>Underwriting!B23*(1+Underwriting!B16)^3</f>
         <v/>
       </c>
-      <c r="G7" s="29">
+      <c r="G7" s="28">
         <f>Underwriting!B23*(1+Underwriting!B16)^4</f>
         <v/>
       </c>
-      <c r="H7" s="29">
+      <c r="H7" s="28">
         <f>Underwriting!B23*(1+Underwriting!B16)^5</f>
         <v/>
       </c>
-      <c r="I7" s="29">
+      <c r="I7" s="28">
         <f>Underwriting!B23*(1+Underwriting!B16)^6</f>
         <v/>
       </c>
-      <c r="J7" s="29">
+      <c r="J7" s="28">
         <f>Underwriting!B23*(1+Underwriting!B16)^7</f>
         <v/>
       </c>
-      <c r="K7" s="29">
+      <c r="K7" s="28">
         <f>Underwriting!B23*(1+Underwriting!B16)^8</f>
         <v/>
       </c>
-      <c r="L7" s="29">
+      <c r="L7" s="28">
         <f>Underwriting!B23*(1+Underwriting!B16)^9</f>
         <v/>
       </c>
@@ -3399,43 +4246,43 @@
           <t>Effective Gross Income</t>
         </is>
       </c>
-      <c r="C8" s="31">
+      <c r="C8" s="30">
         <f>C5+C6+C7</f>
         <v/>
       </c>
-      <c r="D8" s="31">
+      <c r="D8" s="30">
         <f>D5+D6+D7</f>
         <v/>
       </c>
-      <c r="E8" s="31">
+      <c r="E8" s="30">
         <f>E5+E6+E7</f>
         <v/>
       </c>
-      <c r="F8" s="31">
+      <c r="F8" s="30">
         <f>F5+F6+F7</f>
         <v/>
       </c>
-      <c r="G8" s="31">
+      <c r="G8" s="30">
         <f>G5+G6+G7</f>
         <v/>
       </c>
-      <c r="H8" s="31">
+      <c r="H8" s="30">
         <f>H5+H6+H7</f>
         <v/>
       </c>
-      <c r="I8" s="31">
+      <c r="I8" s="30">
         <f>I5+I6+I7</f>
         <v/>
       </c>
-      <c r="J8" s="31">
+      <c r="J8" s="30">
         <f>J5+J6+J7</f>
         <v/>
       </c>
-      <c r="K8" s="31">
+      <c r="K8" s="30">
         <f>K5+K6+K7</f>
         <v/>
       </c>
-      <c r="L8" s="31">
+      <c r="L8" s="30">
         <f>L5+L6+L7</f>
         <v/>
       </c>
@@ -3446,43 +4293,43 @@
           <t>Operating Expenses</t>
         </is>
       </c>
-      <c r="C9" s="29">
+      <c r="C9" s="28">
         <f>Underwriting!B35*(1+Underwriting!B17)^0</f>
         <v/>
       </c>
-      <c r="D9" s="29">
+      <c r="D9" s="28">
         <f>Underwriting!B35*(1+Underwriting!B17)^1</f>
         <v/>
       </c>
-      <c r="E9" s="29">
+      <c r="E9" s="28">
         <f>Underwriting!B35*(1+Underwriting!B17)^2</f>
         <v/>
       </c>
-      <c r="F9" s="29">
+      <c r="F9" s="28">
         <f>Underwriting!B35*(1+Underwriting!B17)^3</f>
         <v/>
       </c>
-      <c r="G9" s="29">
+      <c r="G9" s="28">
         <f>Underwriting!B35*(1+Underwriting!B17)^4</f>
         <v/>
       </c>
-      <c r="H9" s="29">
+      <c r="H9" s="28">
         <f>Underwriting!B35*(1+Underwriting!B17)^5</f>
         <v/>
       </c>
-      <c r="I9" s="29">
+      <c r="I9" s="28">
         <f>Underwriting!B35*(1+Underwriting!B17)^6</f>
         <v/>
       </c>
-      <c r="J9" s="29">
+      <c r="J9" s="28">
         <f>Underwriting!B35*(1+Underwriting!B17)^7</f>
         <v/>
       </c>
-      <c r="K9" s="29">
+      <c r="K9" s="28">
         <f>Underwriting!B35*(1+Underwriting!B17)^8</f>
         <v/>
       </c>
-      <c r="L9" s="29">
+      <c r="L9" s="28">
         <f>Underwriting!B35*(1+Underwriting!B17)^9</f>
         <v/>
       </c>
@@ -3493,43 +4340,43 @@
           <t>Net Operating Income</t>
         </is>
       </c>
-      <c r="C10" s="33">
+      <c r="C10" s="32">
         <f>C8-C9</f>
         <v/>
       </c>
-      <c r="D10" s="33">
+      <c r="D10" s="32">
         <f>D8-D9</f>
         <v/>
       </c>
-      <c r="E10" s="33">
+      <c r="E10" s="32">
         <f>E8-E9</f>
         <v/>
       </c>
-      <c r="F10" s="33">
+      <c r="F10" s="32">
         <f>F8-F9</f>
         <v/>
       </c>
-      <c r="G10" s="33">
+      <c r="G10" s="32">
         <f>G8-G9</f>
         <v/>
       </c>
-      <c r="H10" s="33">
+      <c r="H10" s="32">
         <f>H8-H9</f>
         <v/>
       </c>
-      <c r="I10" s="33">
+      <c r="I10" s="32">
         <f>I8-I9</f>
         <v/>
       </c>
-      <c r="J10" s="33">
+      <c r="J10" s="32">
         <f>J8-J9</f>
         <v/>
       </c>
-      <c r="K10" s="33">
+      <c r="K10" s="32">
         <f>K8-K9</f>
         <v/>
       </c>
-      <c r="L10" s="33">
+      <c r="L10" s="32">
         <f>L8-L9</f>
         <v/>
       </c>
@@ -3540,43 +4387,43 @@
           <t>Annual Debt Service</t>
         </is>
       </c>
-      <c r="C11" s="29">
+      <c r="C11" s="28">
         <f>IF(1&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="D11" s="29">
+      <c r="D11" s="28">
         <f>IF(2&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="E11" s="29">
+      <c r="E11" s="28">
         <f>IF(3&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="F11" s="29">
+      <c r="F11" s="28">
         <f>IF(4&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="G11" s="29">
+      <c r="G11" s="28">
         <f>IF(5&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="H11" s="29">
+      <c r="H11" s="28">
         <f>IF(6&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="I11" s="29">
+      <c r="I11" s="28">
         <f>IF(7&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="J11" s="29">
+      <c r="J11" s="28">
         <f>IF(8&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="K11" s="29">
+      <c r="K11" s="28">
         <f>IF(9&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
-      <c r="L11" s="29">
+      <c r="L11" s="28">
         <f>IF(10&lt;=Underwriting!B49,Underwriting!B59,0)</f>
         <v/>
       </c>
@@ -3587,47 +4434,47 @@
           <t>Loan Balance (end of yr)</t>
         </is>
       </c>
-      <c r="B12" s="29">
+      <c r="B12" s="28">
         <f>Underwriting!B54</f>
         <v/>
       </c>
-      <c r="C12" s="29">
+      <c r="C12" s="28">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(1,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(1,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="D12" s="29">
+      <c r="D12" s="28">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(2,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(2,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="E12" s="29">
+      <c r="E12" s="28">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(3,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(3,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="F12" s="29">
+      <c r="F12" s="28">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(4,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(4,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="G12" s="29">
+      <c r="G12" s="28">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(5,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(5,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="H12" s="29">
+      <c r="H12" s="28">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(6,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(6,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="I12" s="29">
+      <c r="I12" s="28">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(7,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(7,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="J12" s="29">
+      <c r="J12" s="28">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(8,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(8,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="K12" s="29">
+      <c r="K12" s="28">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(9,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(9,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
-      <c r="L12" s="29">
+      <c r="L12" s="28">
         <f>Underwriting!B54*(1+(Underwriting!B45/12))^(MIN(10,Underwriting!B46)*12)-Underwriting!B58*(((1+(Underwriting!B45/12))^(MIN(10,Underwriting!B46)*12)-1)/(Underwriting!B45/12))</f>
         <v/>
       </c>
@@ -3685,43 +4532,43 @@
           <t>Net Sale Proceeds (reversion)</t>
         </is>
       </c>
-      <c r="C14" s="41">
+      <c r="C14" s="43">
         <f>IF(1=Underwriting!B49,((C10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-C12,0)</f>
         <v/>
       </c>
-      <c r="D14" s="41">
+      <c r="D14" s="43">
         <f>IF(2=Underwriting!B49,((D10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-D12,0)</f>
         <v/>
       </c>
-      <c r="E14" s="41">
+      <c r="E14" s="43">
         <f>IF(3=Underwriting!B49,((E10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-E12,0)</f>
         <v/>
       </c>
-      <c r="F14" s="41">
+      <c r="F14" s="43">
         <f>IF(4=Underwriting!B49,((F10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-F12,0)</f>
         <v/>
       </c>
-      <c r="G14" s="41">
+      <c r="G14" s="43">
         <f>IF(5=Underwriting!B49,((G10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-G12,0)</f>
         <v/>
       </c>
-      <c r="H14" s="41">
+      <c r="H14" s="43">
         <f>IF(6=Underwriting!B49,((H10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-H12,0)</f>
         <v/>
       </c>
-      <c r="I14" s="41">
+      <c r="I14" s="43">
         <f>IF(7=Underwriting!B49,((I10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-I12,0)</f>
         <v/>
       </c>
-      <c r="J14" s="41">
+      <c r="J14" s="43">
         <f>IF(8=Underwriting!B49,((J10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-J12,0)</f>
         <v/>
       </c>
-      <c r="K14" s="41">
+      <c r="K14" s="43">
         <f>IF(9=Underwriting!B49,((K10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-K12,0)</f>
         <v/>
       </c>
-      <c r="L14" s="41">
+      <c r="L14" s="43">
         <f>IF(10=Underwriting!B49,((L10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-L12,0)</f>
         <v/>
       </c>
@@ -3732,47 +4579,47 @@
           <t>Total Cash Flow (for IRR)</t>
         </is>
       </c>
-      <c r="B15" s="33">
+      <c r="B15" s="32">
         <f>-Underwriting!B57</f>
         <v/>
       </c>
-      <c r="C15" s="33">
+      <c r="C15" s="32">
         <f>C13+C14</f>
         <v/>
       </c>
-      <c r="D15" s="33">
+      <c r="D15" s="32">
         <f>D13+D14</f>
         <v/>
       </c>
-      <c r="E15" s="33">
+      <c r="E15" s="32">
         <f>E13+E14</f>
         <v/>
       </c>
-      <c r="F15" s="33">
+      <c r="F15" s="32">
         <f>F13+F14</f>
         <v/>
       </c>
-      <c r="G15" s="33">
+      <c r="G15" s="32">
         <f>G13+G14</f>
         <v/>
       </c>
-      <c r="H15" s="33">
+      <c r="H15" s="32">
         <f>H13+H14</f>
         <v/>
       </c>
-      <c r="I15" s="33">
+      <c r="I15" s="32">
         <f>I13+I14</f>
         <v/>
       </c>
-      <c r="J15" s="33">
+      <c r="J15" s="32">
         <f>J13+J14</f>
         <v/>
       </c>
-      <c r="K15" s="33">
+      <c r="K15" s="32">
         <f>K13+K14</f>
         <v/>
       </c>
-      <c r="L15" s="33">
+      <c r="L15" s="32">
         <f>L13+L14</f>
         <v/>
       </c>
@@ -3790,7 +4637,7 @@
           <t>Levered IRR</t>
         </is>
       </c>
-      <c r="B18" s="35">
+      <c r="B18" s="33">
         <f>IRR(B15:L15)</f>
         <v/>
       </c>
@@ -3806,7 +4653,7 @@
           <t>Equity Multiple</t>
         </is>
       </c>
-      <c r="B19" s="36">
+      <c r="B19" s="34">
         <f>(SUM(C13:L13)+SUM(C14:L14))/-B15</f>
         <v/>
       </c>
@@ -3822,7 +4669,7 @@
           <t>Avg. Cash-on-Cash</t>
         </is>
       </c>
-      <c r="B20" s="35">
+      <c r="B20" s="33">
         <f>AVERAGEIF(C11:L11,"&gt;0",C13:L13)/Underwriting!B57</f>
         <v/>
       </c>
@@ -3838,7 +4685,7 @@
           <t>Year-1 Cash-on-Cash</t>
         </is>
       </c>
-      <c r="B21" s="35">
+      <c r="B21" s="33">
         <f>Underwriting!B64</f>
         <v/>
       </c>
@@ -3849,7 +4696,7 @@
           <t>Going-in Cap Rate</t>
         </is>
       </c>
-      <c r="B22" s="35">
+      <c r="B22" s="33">
         <f>Underwriting!B62</f>
         <v/>
       </c>
@@ -3860,7 +4707,7 @@
           <t>Total Profit</t>
         </is>
       </c>
-      <c r="B23" s="33">
+      <c r="B23" s="32">
         <f>SUM(C13:L13)+SUM(C14:L14)+B15</f>
         <v/>
       </c>
@@ -3879,7 +4726,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3918,158 +4765,158 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="42" t="inlineStr">
+      <c r="A5" s="44" t="inlineStr">
         <is>
           <t>Price \ Rate</t>
         </is>
       </c>
-      <c r="B5" s="43">
+      <c r="B5" s="45">
         <f>Underwriting!B45+-0.01</f>
         <v/>
       </c>
-      <c r="C5" s="43">
+      <c r="C5" s="45">
         <f>Underwriting!B45+-0.005</f>
         <v/>
       </c>
-      <c r="D5" s="43">
+      <c r="D5" s="45">
         <f>Underwriting!B45+0</f>
         <v/>
       </c>
-      <c r="E5" s="43">
+      <c r="E5" s="45">
         <f>Underwriting!B45+0.005</f>
         <v/>
       </c>
-      <c r="F5" s="43">
+      <c r="F5" s="45">
         <f>Underwriting!B45+0.01</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="31">
+      <c r="A6" s="30">
         <f>Underwriting!B9*0.9</f>
         <v/>
       </c>
-      <c r="B6" s="44">
+      <c r="B6" s="37">
         <f>(Underwriting!B40-((($A6*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="C6" s="44">
+      <c r="C6" s="37">
         <f>(Underwriting!B40-((($A6*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="D6" s="44">
+      <c r="D6" s="37">
         <f>(Underwriting!B40-((($A6*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="E6" s="44">
+      <c r="E6" s="37">
         <f>(Underwriting!B40-((($A6*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="F6" s="44">
+      <c r="F6" s="37">
         <f>(Underwriting!B40-((($A6*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="31">
+      <c r="A7" s="30">
         <f>Underwriting!B9*0.95</f>
         <v/>
       </c>
-      <c r="B7" s="44">
+      <c r="B7" s="37">
         <f>(Underwriting!B40-((($A7*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="C7" s="44">
+      <c r="C7" s="37">
         <f>(Underwriting!B40-((($A7*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="D7" s="44">
+      <c r="D7" s="37">
         <f>(Underwriting!B40-((($A7*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="E7" s="44">
+      <c r="E7" s="37">
         <f>(Underwriting!B40-((($A7*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="F7" s="44">
+      <c r="F7" s="37">
         <f>(Underwriting!B40-((($A7*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="31">
+      <c r="A8" s="30">
         <f>Underwriting!B9*1.0</f>
         <v/>
       </c>
-      <c r="B8" s="44">
+      <c r="B8" s="37">
         <f>(Underwriting!B40-((($A8*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="C8" s="44">
+      <c r="C8" s="37">
         <f>(Underwriting!B40-((($A8*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="D8" s="44">
+      <c r="D8" s="37">
         <f>(Underwriting!B40-((($A8*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="E8" s="44">
+      <c r="E8" s="37">
         <f>(Underwriting!B40-((($A8*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="F8" s="44">
+      <c r="F8" s="37">
         <f>(Underwriting!B40-((($A8*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31">
+      <c r="A9" s="30">
         <f>Underwriting!B9*1.05</f>
         <v/>
       </c>
-      <c r="B9" s="44">
+      <c r="B9" s="37">
         <f>(Underwriting!B40-((($A9*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="C9" s="44">
+      <c r="C9" s="37">
         <f>(Underwriting!B40-((($A9*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="D9" s="44">
+      <c r="D9" s="37">
         <f>(Underwriting!B40-((($A9*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="E9" s="44">
+      <c r="E9" s="37">
         <f>(Underwriting!B40-((($A9*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="F9" s="44">
+      <c r="F9" s="37">
         <f>(Underwriting!B40-((($A9*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="31">
+      <c r="A10" s="30">
         <f>Underwriting!B9*1.1</f>
         <v/>
       </c>
-      <c r="B10" s="44">
+      <c r="B10" s="37">
         <f>(Underwriting!B40-((($A10*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="C10" s="44">
+      <c r="C10" s="37">
         <f>(Underwriting!B40-((($A10*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="D10" s="44">
+      <c r="D10" s="37">
         <f>(Underwriting!B40-((($A10*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="E10" s="44">
+      <c r="E10" s="37">
         <f>(Underwriting!B40-((($A10*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
-      <c r="F10" s="44">
+      <c r="F10" s="37">
         <f>(Underwriting!B40-((($A10*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
         <v/>
       </c>
@@ -4082,158 +4929,158 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="42" t="inlineStr">
+      <c r="A14" s="44" t="inlineStr">
         <is>
           <t>Price \ Rate</t>
         </is>
       </c>
-      <c r="B14" s="43">
+      <c r="B14" s="45">
         <f>Underwriting!B45+-0.01</f>
         <v/>
       </c>
-      <c r="C14" s="43">
+      <c r="C14" s="45">
         <f>Underwriting!B45+-0.005</f>
         <v/>
       </c>
-      <c r="D14" s="43">
+      <c r="D14" s="45">
         <f>Underwriting!B45+0</f>
         <v/>
       </c>
-      <c r="E14" s="43">
+      <c r="E14" s="45">
         <f>Underwriting!B45+0.005</f>
         <v/>
       </c>
-      <c r="F14" s="43">
+      <c r="F14" s="45">
         <f>Underwriting!B45+0.01</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="31">
+      <c r="A15" s="30">
         <f>Underwriting!B9*0.9</f>
         <v/>
       </c>
-      <c r="B15" s="45">
+      <c r="B15" s="46">
         <f>Underwriting!B40/((($A15*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="C15" s="45">
+      <c r="C15" s="46">
         <f>Underwriting!B40/((($A15*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="D15" s="45">
+      <c r="D15" s="46">
         <f>Underwriting!B40/((($A15*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="E15" s="45">
+      <c r="E15" s="46">
         <f>Underwriting!B40/((($A15*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="F15" s="45">
+      <c r="F15" s="46">
         <f>Underwriting!B40/((($A15*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="31">
+      <c r="A16" s="30">
         <f>Underwriting!B9*0.95</f>
         <v/>
       </c>
-      <c r="B16" s="45">
+      <c r="B16" s="46">
         <f>Underwriting!B40/((($A16*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="C16" s="45">
+      <c r="C16" s="46">
         <f>Underwriting!B40/((($A16*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="D16" s="45">
+      <c r="D16" s="46">
         <f>Underwriting!B40/((($A16*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="E16" s="45">
+      <c r="E16" s="46">
         <f>Underwriting!B40/((($A16*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="F16" s="45">
+      <c r="F16" s="46">
         <f>Underwriting!B40/((($A16*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="31">
+      <c r="A17" s="30">
         <f>Underwriting!B9*1.0</f>
         <v/>
       </c>
-      <c r="B17" s="45">
+      <c r="B17" s="46">
         <f>Underwriting!B40/((($A17*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="C17" s="45">
+      <c r="C17" s="46">
         <f>Underwriting!B40/((($A17*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="D17" s="45">
+      <c r="D17" s="46">
         <f>Underwriting!B40/((($A17*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="E17" s="45">
+      <c r="E17" s="46">
         <f>Underwriting!B40/((($A17*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="F17" s="45">
+      <c r="F17" s="46">
         <f>Underwriting!B40/((($A17*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="31">
+      <c r="A18" s="30">
         <f>Underwriting!B9*1.05</f>
         <v/>
       </c>
-      <c r="B18" s="45">
+      <c r="B18" s="46">
         <f>Underwriting!B40/((($A18*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="C18" s="45">
+      <c r="C18" s="46">
         <f>Underwriting!B40/((($A18*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="D18" s="45">
+      <c r="D18" s="46">
         <f>Underwriting!B40/((($A18*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="E18" s="45">
+      <c r="E18" s="46">
         <f>Underwriting!B40/((($A18*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="F18" s="45">
+      <c r="F18" s="46">
         <f>Underwriting!B40/((($A18*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="31">
+      <c r="A19" s="30">
         <f>Underwriting!B9*1.1</f>
         <v/>
       </c>
-      <c r="B19" s="45">
+      <c r="B19" s="46">
         <f>Underwriting!B40/((($A19*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="C19" s="45">
+      <c r="C19" s="46">
         <f>Underwriting!B40/((($A19*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="D19" s="45">
+      <c r="D19" s="46">
         <f>Underwriting!B40/((($A19*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="E19" s="45">
+      <c r="E19" s="46">
         <f>Underwriting!B40/((($A19*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
-      <c r="F19" s="45">
+      <c r="F19" s="46">
         <f>Underwriting!B40/((($A19*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
         <v/>
       </c>
@@ -4253,153 +5100,153 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="42" t="inlineStr">
+      <c r="A24" s="44" t="inlineStr">
         <is>
           <t>Rent \ Vacancy</t>
         </is>
       </c>
-      <c r="B24" s="46" t="n">
+      <c r="B24" s="47" t="n">
         <v>0.05</v>
       </c>
-      <c r="C24" s="46" t="n">
+      <c r="C24" s="47" t="n">
         <v>0.1</v>
       </c>
-      <c r="D24" s="46" t="n">
+      <c r="D24" s="47" t="n">
         <v>0.15</v>
       </c>
-      <c r="E24" s="46" t="n">
+      <c r="E24" s="47" t="n">
         <v>0.2</v>
       </c>
-      <c r="F24" s="46" t="n">
+      <c r="F24" s="47" t="n">
         <v>0.25</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="31">
+      <c r="A25" s="30">
         <f>Underwriting!B11+-100</f>
         <v/>
       </c>
-      <c r="B25" s="44">
+      <c r="B25" s="37">
         <f>(((Underwriting!B8*$A25*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="C25" s="44">
+      <c r="C25" s="37">
         <f>(((Underwriting!B8*$A25*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="D25" s="44">
+      <c r="D25" s="37">
         <f>(((Underwriting!B8*$A25*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="E25" s="44">
+      <c r="E25" s="37">
         <f>(((Underwriting!B8*$A25*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="F25" s="44">
+      <c r="F25" s="37">
         <f>(((Underwriting!B8*$A25*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="31">
+      <c r="A26" s="30">
         <f>Underwriting!B11+-50</f>
         <v/>
       </c>
-      <c r="B26" s="44">
+      <c r="B26" s="37">
         <f>(((Underwriting!B8*$A26*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="C26" s="44">
+      <c r="C26" s="37">
         <f>(((Underwriting!B8*$A26*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="D26" s="44">
+      <c r="D26" s="37">
         <f>(((Underwriting!B8*$A26*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="E26" s="44">
+      <c r="E26" s="37">
         <f>(((Underwriting!B8*$A26*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="F26" s="44">
+      <c r="F26" s="37">
         <f>(((Underwriting!B8*$A26*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="31">
+      <c r="A27" s="30">
         <f>Underwriting!B11+0</f>
         <v/>
       </c>
-      <c r="B27" s="44">
+      <c r="B27" s="37">
         <f>(((Underwriting!B8*$A27*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="C27" s="44">
+      <c r="C27" s="37">
         <f>(((Underwriting!B8*$A27*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="D27" s="44">
+      <c r="D27" s="37">
         <f>(((Underwriting!B8*$A27*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="E27" s="44">
+      <c r="E27" s="37">
         <f>(((Underwriting!B8*$A27*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="F27" s="44">
+      <c r="F27" s="37">
         <f>(((Underwriting!B8*$A27*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="31">
+      <c r="A28" s="30">
         <f>Underwriting!B11+50</f>
         <v/>
       </c>
-      <c r="B28" s="44">
+      <c r="B28" s="37">
         <f>(((Underwriting!B8*$A28*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="C28" s="44">
+      <c r="C28" s="37">
         <f>(((Underwriting!B8*$A28*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="D28" s="44">
+      <c r="D28" s="37">
         <f>(((Underwriting!B8*$A28*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="E28" s="44">
+      <c r="E28" s="37">
         <f>(((Underwriting!B8*$A28*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="F28" s="44">
+      <c r="F28" s="37">
         <f>(((Underwriting!B8*$A28*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="31">
+      <c r="A29" s="30">
         <f>Underwriting!B11+100</f>
         <v/>
       </c>
-      <c r="B29" s="44">
+      <c r="B29" s="37">
         <f>(((Underwriting!B8*$A29*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="C29" s="44">
+      <c r="C29" s="37">
         <f>(((Underwriting!B8*$A29*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="D29" s="44">
+      <c r="D29" s="37">
         <f>(((Underwriting!B8*$A29*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="E29" s="44">
+      <c r="E29" s="37">
         <f>(((Underwriting!B8*$A29*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
-      <c r="F29" s="44">
+      <c r="F29" s="37">
         <f>(((Underwriting!B8*$A29*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
         <v/>
       </c>
@@ -4420,311 +5267,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>LOAN SIZING — MAX PRICE AT TARGET DSCR</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="15" t="inlineStr">
-        <is>
-          <t>Works backward from how much debt the NOI supports. NOI is held at the Underwriting Year-1 figure; rate, amortization and LTV come from the Underwriting tab.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>TARGETS  (your / the lender's limits)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="17" t="inlineStr">
-        <is>
-          <t>Target DSCR</t>
-        </is>
-      </c>
-      <c r="B5" s="22" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>minimum coverage lender requires</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Target Debt Yield</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>NOI / loan floor (often 9-10%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>Max LTV %</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>lender's loan-to-value cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>LOAN INPUTS  (from Underwriting)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>Year-1 NOI</t>
-        </is>
-      </c>
-      <c r="B10" s="29">
-        <f>Underwriting!B40</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="17" t="inlineStr">
-        <is>
-          <t>Interest Rate</t>
-        </is>
-      </c>
-      <c r="B11" s="47">
-        <f>Underwriting!B45</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="17" t="inlineStr">
-        <is>
-          <t>Amortization (yrs)</t>
-        </is>
-      </c>
-      <c r="B12" s="39">
-        <f>Underwriting!B46</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>Annual Debt Constant (per $1 loan)</t>
-        </is>
-      </c>
-      <c r="B13" s="48">
-        <f>PMT(B11/12,B12*12,-1)*12</f>
-        <v/>
-      </c>
-      <c r="C13" s="15">
-        <f> annual debt service per $1 borrowed</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>MAXIMUM SUPPORTABLE LOAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>Max Annual Debt Service (DSCR)</t>
-        </is>
-      </c>
-      <c r="B16" s="29">
-        <f>B10/B5</f>
-        <v/>
-      </c>
-      <c r="C16" s="15">
-        <f> NOI / target DSCR</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Max Loan — DSCR constrained</t>
-        </is>
-      </c>
-      <c r="B17" s="29">
-        <f>B16/B13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Max Loan — Debt-Yield constrained</t>
-        </is>
-      </c>
-      <c r="B18" s="29">
-        <f>B10/B6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>Binding Max Loan</t>
-        </is>
-      </c>
-      <c r="B19" s="31">
-        <f>MIN(B17,B18)</f>
-        <v/>
-      </c>
-      <c r="C19" s="15" t="inlineStr">
-        <is>
-          <t>the lesser of the two</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>MAXIMUM PURCHASE PRICE</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Max Price — DSCR/Debt-Yield (at Max LTV)</t>
-        </is>
-      </c>
-      <c r="B22" s="33">
-        <f>B19/B7</f>
-        <v/>
-      </c>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>price the debt supports at your LTV</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="17" t="inlineStr">
-        <is>
-          <t>Current Purchase Price</t>
-        </is>
-      </c>
-      <c r="B23" s="29">
-        <f>Underwriting!B9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>Price Headroom ($)</t>
-        </is>
-      </c>
-      <c r="B24" s="9">
-        <f>B22-B23</f>
-        <v/>
-      </c>
-      <c r="C24" s="15" t="inlineStr">
-        <is>
-          <t>positive = room to pay more; negative = overpaying</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>Price Headroom (%)</t>
-        </is>
-      </c>
-      <c r="B25" s="14">
-        <f>B24/B23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="17" t="inlineStr">
-        <is>
-          <t>DSCR at Current Price</t>
-        </is>
-      </c>
-      <c r="B26" s="37">
-        <f>Underwriting!B65</f>
-        <v/>
-      </c>
-      <c r="C26" s="15" t="inlineStr">
-        <is>
-          <t>for reference (target above)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="17" t="inlineStr">
-        <is>
-          <t>Required Equity at Max Price</t>
-        </is>
-      </c>
-      <c r="B27" s="29">
-        <f>B22*(1-B7)</f>
-        <v/>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>down payment if you buy at the max</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="15" t="inlineStr">
-        <is>
-          <t>READ: if Headroom is negative, the price is higher than the income can safely finance at your target DSCR — you'd need more equity, a lower rate, or a price cut.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A4:C4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Offer Structures tab (AJ's 4-column engine + MAO + seller carry)
New tab mirroring AJ Kukra's Module-5 spreadsheet:
- 4 side-by-side offers: Seller Asking / Conventional / Partial seller carry
  / Full seller carry, each with its own editable levers.
- Two-lien debt stack (bank + seller carry), interest-only toggles, blended
  rate, DSCR on total debt service.
- Auto-solved Maximum Allowable Offer (highest price where DSCR>=1.35 AND
  CoC>=10% both clear) plus manual price entry with live GO/CONDITIONAL/NO-GO.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFUKyb6gzsdDbmscePYHf6
</commit_message>
<xml_diff>
--- a/RV_Park_Underwriting.xlsx
+++ b/RV_Park_Underwriting.xlsx
@@ -12,11 +12,12 @@
     <sheet name="Deal Scorecard" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Underwriting" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Normalization" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Income Detail" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Actuals vs Pro Forma" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Pro Forma &amp; Returns" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Sensitivity" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Loan Sizing" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Offer Structures" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Income Detail" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Actuals vs Pro Forma" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Pro Forma &amp; Returns" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Sensitivity" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Loan Sizing" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,7 +32,7 @@
     <numFmt numFmtId="166" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -91,6 +92,10 @@
     <font>
       <b val="1"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
     <font>
       <sz val="11"/>
@@ -165,13 +170,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -266,6 +271,25 @@
     <xf numFmtId="164" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -287,12 +311,6 @@
     </xf>
     <xf numFmtId="165" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -694,7 +712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A61"/>
+  <dimension ref="A1:A63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="104" customWidth="1" min="1" max="1"/>
@@ -962,126 +980,140 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Income Detail — optional. Build income from your site mix (long-term + seasonal nightly).</t>
+          <t xml:space="preserve">  • Offer Structures — AJ's 4-column engine: Seller / Conventional / Partial carry / Full carry, two-lien</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Actuals vs Pro Forma — seller's CURRENT numbers vs your stabilized plan, side by side.</t>
+          <t xml:space="preserve">      debt stack, blended rate, and the auto-solved Maximum Allowable Offer (MAO).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Pro Forma &amp; Returns — 10-year projection, sale reversion, IRR &amp; equity multiple.</t>
+          <t xml:space="preserve">  • Income Detail — optional. Build income from your site mix (long-term + seasonal nightly).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Sensitivity   — the Bad-Day Test: CoC &amp; DSCR vs price, interest rate, rent &amp; vacancy.</t>
+          <t xml:space="preserve">  • Actuals vs Pro Forma — seller's CURRENT numbers vs your stabilized plan, side by side.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • Pro Forma &amp; Returns — 10-year projection, sale reversion, IRR &amp; equity multiple.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Sensitivity   — the Bad-Day Test: CoC &amp; DSCR vs price, interest rate, rent &amp; vacancy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • Loan Sizing   — max purchase price the NOI supports at your target DSCR / debt yield.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
         <is>
           <t>HOW TO USE IT</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>1. Normalization tab: enter the seller's reported expenses; read off your normalized NOI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>2. Underwriting tab: fill the yellow cells using those NORMALIZED numbers, not the seller's.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>3. Deal Scorecard: read the GOOD/OK/BAD ratings and the GO / CONDITIONAL / NO-GO verdict.</t>
+          <t>1. Normalization tab: enter the seller's reported expenses; read off your normalized NOI.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
+          <t>2. Underwriting tab: fill the yellow cells using those NORMALIZED numbers, not the seller's.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>3. Deal Scorecard: read the GOOD/OK/BAD ratings and the GO / CONDITIONAL / NO-GO verdict.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
           <t>4. Sensitivity: run the bad-day stress test. Deal Summary: the one-page headline.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>RV-PARK / MHP WATCH-OUTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Nondisclosure states: sellers needn't volunteer problems (failing septic, AC, zoning). Dig.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Transient/nightly income is seasonal and far less stable than annual/monthly tenants.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Utility metering — are sites individually metered, or is the owner eating utilities? (ratio bill-back).</t>
+          <t xml:space="preserve">  • Nondisclosure states: sellers needn't volunteer problems (failing septic, AC, zoning). Dig.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Infrastructure age — septic/sewer, electric pedestals (30/50 amp), water lines = big CapEx.</t>
+          <t xml:space="preserve">  • Transient/nightly income is seasonal and far less stable than annual/monthly tenants.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Property taxes usually RESET on sale — don't trust the seller's current tax line.</t>
+          <t xml:space="preserve">  • Utility metering — are sites individually metered, or is the owner eating utilities? (ratio bill-back).</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr"/>
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Infrastructure age — septic/sewer, electric pedestals (30/50 amp), water lines = big CapEx.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Property taxes usually RESET on sale — don't trust the seller's current tax line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>This is a screening tool, not investment advice. Verify every number and consult professionals.</t>
         </is>
@@ -1093,6 +1125,549 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>SENSITIVITY TABLES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Rows = purchase price scenarios. Columns = interest rate. Cells recompute live from Underwriting inputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>CASH-ON-CASH RETURN  —  Price x Interest Rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="51" t="inlineStr">
+        <is>
+          <t>Price \ Rate</t>
+        </is>
+      </c>
+      <c r="B5" s="52">
+        <f>Underwriting!B45+-0.01</f>
+        <v/>
+      </c>
+      <c r="C5" s="52">
+        <f>Underwriting!B45+-0.005</f>
+        <v/>
+      </c>
+      <c r="D5" s="52">
+        <f>Underwriting!B45+0</f>
+        <v/>
+      </c>
+      <c r="E5" s="52">
+        <f>Underwriting!B45+0.005</f>
+        <v/>
+      </c>
+      <c r="F5" s="52">
+        <f>Underwriting!B45+0.01</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="30">
+        <f>Underwriting!B9*0.9</f>
+        <v/>
+      </c>
+      <c r="B6" s="37">
+        <f>(Underwriting!B40-((($A6*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="C6" s="37">
+        <f>(Underwriting!B40-((($A6*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="D6" s="37">
+        <f>(Underwriting!B40-((($A6*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="E6" s="37">
+        <f>(Underwriting!B40-((($A6*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="F6" s="37">
+        <f>(Underwriting!B40-((($A6*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="30">
+        <f>Underwriting!B9*0.95</f>
+        <v/>
+      </c>
+      <c r="B7" s="37">
+        <f>(Underwriting!B40-((($A7*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="C7" s="37">
+        <f>(Underwriting!B40-((($A7*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="D7" s="37">
+        <f>(Underwriting!B40-((($A7*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="E7" s="37">
+        <f>(Underwriting!B40-((($A7*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="F7" s="37">
+        <f>(Underwriting!B40-((($A7*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="30">
+        <f>Underwriting!B9*1.0</f>
+        <v/>
+      </c>
+      <c r="B8" s="37">
+        <f>(Underwriting!B40-((($A8*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="C8" s="37">
+        <f>(Underwriting!B40-((($A8*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="D8" s="37">
+        <f>(Underwriting!B40-((($A8*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="E8" s="37">
+        <f>(Underwriting!B40-((($A8*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="F8" s="37">
+        <f>(Underwriting!B40-((($A8*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="30">
+        <f>Underwriting!B9*1.05</f>
+        <v/>
+      </c>
+      <c r="B9" s="37">
+        <f>(Underwriting!B40-((($A9*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="C9" s="37">
+        <f>(Underwriting!B40-((($A9*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="D9" s="37">
+        <f>(Underwriting!B40-((($A9*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="E9" s="37">
+        <f>(Underwriting!B40-((($A9*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="F9" s="37">
+        <f>(Underwriting!B40-((($A9*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="30">
+        <f>Underwriting!B9*1.1</f>
+        <v/>
+      </c>
+      <c r="B10" s="37">
+        <f>(Underwriting!B40-((($A10*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="C10" s="37">
+        <f>(Underwriting!B40-((($A10*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="D10" s="37">
+        <f>(Underwriting!B40-((($A10*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="E10" s="37">
+        <f>(Underwriting!B40-((($A10*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+      <c r="F10" s="37">
+        <f>(Underwriting!B40-((($A10*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>DEBT SERVICE COVERAGE (DSCR)  —  Price x Interest Rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="51" t="inlineStr">
+        <is>
+          <t>Price \ Rate</t>
+        </is>
+      </c>
+      <c r="B14" s="52">
+        <f>Underwriting!B45+-0.01</f>
+        <v/>
+      </c>
+      <c r="C14" s="52">
+        <f>Underwriting!B45+-0.005</f>
+        <v/>
+      </c>
+      <c r="D14" s="52">
+        <f>Underwriting!B45+0</f>
+        <v/>
+      </c>
+      <c r="E14" s="52">
+        <f>Underwriting!B45+0.005</f>
+        <v/>
+      </c>
+      <c r="F14" s="52">
+        <f>Underwriting!B45+0.01</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30">
+        <f>Underwriting!B9*0.9</f>
+        <v/>
+      </c>
+      <c r="B15" s="53">
+        <f>Underwriting!B40/((($A15*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="C15" s="53">
+        <f>Underwriting!B40/((($A15*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="D15" s="53">
+        <f>Underwriting!B40/((($A15*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="E15" s="53">
+        <f>Underwriting!B40/((($A15*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="F15" s="53">
+        <f>Underwriting!B40/((($A15*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30">
+        <f>Underwriting!B9*0.95</f>
+        <v/>
+      </c>
+      <c r="B16" s="53">
+        <f>Underwriting!B40/((($A16*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="C16" s="53">
+        <f>Underwriting!B40/((($A16*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="D16" s="53">
+        <f>Underwriting!B40/((($A16*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="E16" s="53">
+        <f>Underwriting!B40/((($A16*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="F16" s="53">
+        <f>Underwriting!B40/((($A16*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="30">
+        <f>Underwriting!B9*1.0</f>
+        <v/>
+      </c>
+      <c r="B17" s="53">
+        <f>Underwriting!B40/((($A17*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="C17" s="53">
+        <f>Underwriting!B40/((($A17*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="D17" s="53">
+        <f>Underwriting!B40/((($A17*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="E17" s="53">
+        <f>Underwriting!B40/((($A17*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="F17" s="53">
+        <f>Underwriting!B40/((($A17*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="30">
+        <f>Underwriting!B9*1.05</f>
+        <v/>
+      </c>
+      <c r="B18" s="53">
+        <f>Underwriting!B40/((($A18*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="C18" s="53">
+        <f>Underwriting!B40/((($A18*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="D18" s="53">
+        <f>Underwriting!B40/((($A18*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="E18" s="53">
+        <f>Underwriting!B40/((($A18*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="F18" s="53">
+        <f>Underwriting!B40/((($A18*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="30">
+        <f>Underwriting!B9*1.1</f>
+        <v/>
+      </c>
+      <c r="B19" s="53">
+        <f>Underwriting!B40/((($A19*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="C19" s="53">
+        <f>Underwriting!B40/((($A19*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="D19" s="53">
+        <f>Underwriting!B40/((($A19*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="E19" s="53">
+        <f>Underwriting!B40/((($A19*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+      <c r="F19" s="53">
+        <f>Underwriting!B40/((($A19*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>NOTE: the two tables above hold NOI constant to isolate price &amp; financing risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>CASH-ON-CASH RETURN  —  Monthly Rent x Vacancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="51" t="inlineStr">
+        <is>
+          <t>Rent \ Vacancy</t>
+        </is>
+      </c>
+      <c r="B24" s="54" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C24" s="54" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D24" s="54" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E24" s="54" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F24" s="54" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="30">
+        <f>Underwriting!B11+-100</f>
+        <v/>
+      </c>
+      <c r="B25" s="37">
+        <f>(((Underwriting!B8*$A25*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="C25" s="37">
+        <f>(((Underwriting!B8*$A25*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="D25" s="37">
+        <f>(((Underwriting!B8*$A25*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="E25" s="37">
+        <f>(((Underwriting!B8*$A25*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="F25" s="37">
+        <f>(((Underwriting!B8*$A25*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="30">
+        <f>Underwriting!B11+-50</f>
+        <v/>
+      </c>
+      <c r="B26" s="37">
+        <f>(((Underwriting!B8*$A26*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="C26" s="37">
+        <f>(((Underwriting!B8*$A26*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="D26" s="37">
+        <f>(((Underwriting!B8*$A26*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="E26" s="37">
+        <f>(((Underwriting!B8*$A26*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="F26" s="37">
+        <f>(((Underwriting!B8*$A26*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="30">
+        <f>Underwriting!B11+0</f>
+        <v/>
+      </c>
+      <c r="B27" s="37">
+        <f>(((Underwriting!B8*$A27*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="C27" s="37">
+        <f>(((Underwriting!B8*$A27*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="D27" s="37">
+        <f>(((Underwriting!B8*$A27*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="E27" s="37">
+        <f>(((Underwriting!B8*$A27*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="F27" s="37">
+        <f>(((Underwriting!B8*$A27*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30">
+        <f>Underwriting!B11+50</f>
+        <v/>
+      </c>
+      <c r="B28" s="37">
+        <f>(((Underwriting!B8*$A28*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="C28" s="37">
+        <f>(((Underwriting!B8*$A28*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="D28" s="37">
+        <f>(((Underwriting!B8*$A28*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="E28" s="37">
+        <f>(((Underwriting!B8*$A28*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="F28" s="37">
+        <f>(((Underwriting!B8*$A28*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="30">
+        <f>Underwriting!B11+100</f>
+        <v/>
+      </c>
+      <c r="B29" s="37">
+        <f>(((Underwriting!B8*$A29*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="C29" s="37">
+        <f>(((Underwriting!B8*$A29*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="D29" s="37">
+        <f>(((Underwriting!B8*$A29*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="E29" s="37">
+        <f>(((Underwriting!B8*$A29*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+      <c r="F29" s="37">
+        <f>(((Underwriting!B8*$A29*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>NOTE: this table recomputes NOI (management fee scales with EGI). Uses sites x rent income, not the Income Detail build.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A4:F4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1196,7 +1771,7 @@
           <t>Interest Rate</t>
         </is>
       </c>
-      <c r="B11" s="48">
+      <c r="B11" s="44">
         <f>Underwriting!B45</f>
         <v/>
       </c>
@@ -1207,7 +1782,7 @@
           <t>Amortization (yrs)</t>
         </is>
       </c>
-      <c r="B12" s="41">
+      <c r="B12" s="48">
         <f>Underwriting!B46</f>
         <v/>
       </c>
@@ -1218,7 +1793,7 @@
           <t>Annual Debt Constant (per $1 loan)</t>
         </is>
       </c>
-      <c r="B13" s="49">
+      <c r="B13" s="40">
         <f>PMT(B11/12,B12*12,-1)*12</f>
         <v/>
       </c>
@@ -3247,6 +3822,889 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>OFFER STRUCTURES — MAO &amp; SELLER CARRY (AJ KUKRA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>NOI is held constant (operations don't change with financing). Each column is a price + financing scenario; yellow = editable levers. Verdict uses AJ's rule: DSCR &gt;= target AND Cash-on-Cash &gt;= target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>MAXIMUM ALLOWABLE OFFER — auto-solved (conventional financing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Target DSCR</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>AJ floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Target Cash-on-Cash</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>AJ target</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Bank LTV % (conventional)</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>loan-to-value for the conventional offer</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Bank Interest Rate</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Amortization (yrs)</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>NOI (from Underwriting)</t>
+        </is>
+      </c>
+      <c r="B10" s="28">
+        <f>Underwriting!B40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Annual Debt Constant k (per $1 loan)</t>
+        </is>
+      </c>
+      <c r="B11" s="40">
+        <f>PMT(B8/12,B9*12,-1)*12</f>
+        <v/>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>annual debt service per $1 borrowed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Max Price @ DSCR target</t>
+        </is>
+      </c>
+      <c r="B12" s="28">
+        <f>B10/(B5*B7*B11)</f>
+        <v/>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>DSCR-constrained ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Max Price @ Cash-on-Cash target</t>
+        </is>
+      </c>
+      <c r="B13" s="28">
+        <f>(B10-B6*Underwriting!B48)/(B7*B11+B6*(1-B7+Underwriting!B47))</f>
+        <v/>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>CoC-constrained ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>MAXIMUM ALLOWABLE OFFER (MAO)</t>
+        </is>
+      </c>
+      <c r="B14" s="42">
+        <f>MIN(B12,B13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>highest price where BOTH clear</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>OFFER COMPARISON  (type any price/structure — verdict updates live)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>Lever / Metric</t>
+        </is>
+      </c>
+      <c r="B17" s="43" t="inlineStr">
+        <is>
+          <t>Seller Asking</t>
+        </is>
+      </c>
+      <c r="C17" s="43" t="inlineStr">
+        <is>
+          <t>Offer 1: Conventional</t>
+        </is>
+      </c>
+      <c r="D17" s="43" t="inlineStr">
+        <is>
+          <t>Offer 2: Partial Carry</t>
+        </is>
+      </c>
+      <c r="E17" s="43" t="inlineStr">
+        <is>
+          <t>Offer 3: Full Carry</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Purchase Price</t>
+        </is>
+      </c>
+      <c r="B18" s="27" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="C18" s="27" t="n">
+        <v>1150000</v>
+      </c>
+      <c r="D18" s="27" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="E18" s="27" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>Offer 1 defaults near the MAO above — type your own to test</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Bank Loan % (of price)</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D19" s="21" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Bank Interest Rate</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="C20" s="22" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D20" s="22" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E20" s="22" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Bank Amortization (yrs)</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C21" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="D21" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="E21" s="26" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Bank Interest-Only? (Y/N)</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C22" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E22" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Seller Carry % (of price)</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="21" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E23" s="21" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>Seller Carry Rate</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="22" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E24" s="22" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Seller Carry Amort (yrs)</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C25" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="D25" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="E25" s="26" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>Seller Carry Interest-Only? (Y/N)</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C26" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D26" s="29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E26" s="29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Down Payment %</t>
+        </is>
+      </c>
+      <c r="B27" s="31">
+        <f>1-B19-B23</f>
+        <v/>
+      </c>
+      <c r="C27" s="31">
+        <f>1-C19-C23</f>
+        <v/>
+      </c>
+      <c r="D27" s="31">
+        <f>1-D19-D23</f>
+        <v/>
+      </c>
+      <c r="E27" s="31">
+        <f>1-E19-E23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>DEBT STACK</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Bank Loan $</t>
+        </is>
+      </c>
+      <c r="B29" s="28">
+        <f>B18*B19</f>
+        <v/>
+      </c>
+      <c r="C29" s="28">
+        <f>C18*C19</f>
+        <v/>
+      </c>
+      <c r="D29" s="28">
+        <f>D18*D19</f>
+        <v/>
+      </c>
+      <c r="E29" s="28">
+        <f>E18*E19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Bank Annual Debt Service</t>
+        </is>
+      </c>
+      <c r="B30" s="28">
+        <f>IF(B22="Y",B29*B20,PMT(B20/12,B21*12,-B29)*12)</f>
+        <v/>
+      </c>
+      <c r="C30" s="28">
+        <f>IF(C22="Y",C29*C20,PMT(C20/12,C21*12,-C29)*12)</f>
+        <v/>
+      </c>
+      <c r="D30" s="28">
+        <f>IF(D22="Y",D29*D20,PMT(D20/12,D21*12,-D29)*12)</f>
+        <v/>
+      </c>
+      <c r="E30" s="28">
+        <f>IF(E22="Y",E29*E20,PMT(E20/12,E21*12,-E29)*12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>Seller Carry $</t>
+        </is>
+      </c>
+      <c r="B31" s="28">
+        <f>B18*B23</f>
+        <v/>
+      </c>
+      <c r="C31" s="28">
+        <f>C18*C23</f>
+        <v/>
+      </c>
+      <c r="D31" s="28">
+        <f>D18*D23</f>
+        <v/>
+      </c>
+      <c r="E31" s="28">
+        <f>E18*E23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>Seller Carry Annual Debt Service</t>
+        </is>
+      </c>
+      <c r="B32" s="28">
+        <f>IF(B31=0,0,IF(B26="Y",B31*B24,PMT(B24/12,B25*12,-B31)*12))</f>
+        <v/>
+      </c>
+      <c r="C32" s="28">
+        <f>IF(C31=0,0,IF(C26="Y",C31*C24,PMT(C24/12,C25*12,-C31)*12))</f>
+        <v/>
+      </c>
+      <c r="D32" s="28">
+        <f>IF(D31=0,0,IF(D26="Y",D31*D24,PMT(D24/12,D25*12,-D31)*12))</f>
+        <v/>
+      </c>
+      <c r="E32" s="28">
+        <f>IF(E31=0,0,IF(E26="Y",E31*E24,PMT(E24/12,E25*12,-E31)*12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Total Annual Debt Service</t>
+        </is>
+      </c>
+      <c r="B33" s="30">
+        <f>B30+B32</f>
+        <v/>
+      </c>
+      <c r="C33" s="30">
+        <f>C30+C32</f>
+        <v/>
+      </c>
+      <c r="D33" s="30">
+        <f>D30+D32</f>
+        <v/>
+      </c>
+      <c r="E33" s="30">
+        <f>E30+E32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Blended Rate</t>
+        </is>
+      </c>
+      <c r="B34" s="44">
+        <f>IF((B29+B31)=0,0,(B29*B20+B31*B24)/(B29+B31))</f>
+        <v/>
+      </c>
+      <c r="C34" s="44">
+        <f>IF((C29+C31)=0,0,(C29*C20+C31*C24)/(C29+C31))</f>
+        <v/>
+      </c>
+      <c r="D34" s="44">
+        <f>IF((D29+D31)=0,0,(D29*D20+D31*D24)/(D29+D31))</f>
+        <v/>
+      </c>
+      <c r="E34" s="44">
+        <f>IF((E29+E31)=0,0,(E29*E20+E31*E24)/(E29+E31))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>Down Payment $</t>
+        </is>
+      </c>
+      <c r="B35" s="28">
+        <f>B18*B27</f>
+        <v/>
+      </c>
+      <c r="C35" s="28">
+        <f>C18*C27</f>
+        <v/>
+      </c>
+      <c r="D35" s="28">
+        <f>D18*D27</f>
+        <v/>
+      </c>
+      <c r="E35" s="28">
+        <f>E18*E27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>Closing + CapEx</t>
+        </is>
+      </c>
+      <c r="B36" s="28">
+        <f>B18*Underwriting!B47+Underwriting!B48</f>
+        <v/>
+      </c>
+      <c r="C36" s="28">
+        <f>C18*Underwriting!B47+Underwriting!B48</f>
+        <v/>
+      </c>
+      <c r="D36" s="28">
+        <f>D18*Underwriting!B47+Underwriting!B48</f>
+        <v/>
+      </c>
+      <c r="E36" s="28">
+        <f>E18*Underwriting!B47+Underwriting!B48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Total Cash Invested</t>
+        </is>
+      </c>
+      <c r="B37" s="30">
+        <f>B35+B36</f>
+        <v/>
+      </c>
+      <c r="C37" s="30">
+        <f>C35+C36</f>
+        <v/>
+      </c>
+      <c r="D37" s="30">
+        <f>D35+D36</f>
+        <v/>
+      </c>
+      <c r="E37" s="30">
+        <f>E35+E36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>KEY METRICS</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>NOI (constant)</t>
+        </is>
+      </c>
+      <c r="B39" s="28">
+        <f>Underwriting!B40</f>
+        <v/>
+      </c>
+      <c r="C39" s="28">
+        <f>Underwriting!B40</f>
+        <v/>
+      </c>
+      <c r="D39" s="28">
+        <f>Underwriting!B40</f>
+        <v/>
+      </c>
+      <c r="E39" s="28">
+        <f>Underwriting!B40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>Cap Rate</t>
+        </is>
+      </c>
+      <c r="B40" s="31">
+        <f>B39/B18</f>
+        <v/>
+      </c>
+      <c r="C40" s="31">
+        <f>C39/C18</f>
+        <v/>
+      </c>
+      <c r="D40" s="31">
+        <f>D39/D18</f>
+        <v/>
+      </c>
+      <c r="E40" s="31">
+        <f>E39/E18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>DSCR (total debt)</t>
+        </is>
+      </c>
+      <c r="B41" s="18">
+        <f>IF(B33=0,"n/a",B39/B33)</f>
+        <v/>
+      </c>
+      <c r="C41" s="18">
+        <f>IF(C33=0,"n/a",C39/C33)</f>
+        <v/>
+      </c>
+      <c r="D41" s="18">
+        <f>IF(D33=0,"n/a",D39/D33)</f>
+        <v/>
+      </c>
+      <c r="E41" s="18">
+        <f>IF(E33=0,"n/a",E39/E33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>Net Profit (cash flow)</t>
+        </is>
+      </c>
+      <c r="B42" s="28">
+        <f>B39-B33</f>
+        <v/>
+      </c>
+      <c r="C42" s="28">
+        <f>C39-C33</f>
+        <v/>
+      </c>
+      <c r="D42" s="28">
+        <f>D39-D33</f>
+        <v/>
+      </c>
+      <c r="E42" s="28">
+        <f>E39-E33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>Cash-on-Cash Return</t>
+        </is>
+      </c>
+      <c r="B43" s="14">
+        <f>B42/B37</f>
+        <v/>
+      </c>
+      <c r="C43" s="14">
+        <f>C42/C37</f>
+        <v/>
+      </c>
+      <c r="D43" s="14">
+        <f>D42/D37</f>
+        <v/>
+      </c>
+      <c r="E43" s="14">
+        <f>E42/E37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>DSCR clears target?</t>
+        </is>
+      </c>
+      <c r="B44" s="45">
+        <f>IF(B33=0,"YES",IF(B39/B33&gt;=$B$5,"YES","NO"))</f>
+        <v/>
+      </c>
+      <c r="C44" s="45">
+        <f>IF(C33=0,"YES",IF(C39/C33&gt;=$B$5,"YES","NO"))</f>
+        <v/>
+      </c>
+      <c r="D44" s="45">
+        <f>IF(D33=0,"YES",IF(D39/D33&gt;=$B$5,"YES","NO"))</f>
+        <v/>
+      </c>
+      <c r="E44" s="45">
+        <f>IF(E33=0,"YES",IF(E39/E33&gt;=$B$5,"YES","NO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="inlineStr">
+        <is>
+          <t>Cash-on-Cash clears target?</t>
+        </is>
+      </c>
+      <c r="B45" s="45">
+        <f>IF(B43&gt;=$B$6,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="C45" s="45">
+        <f>IF(C43&gt;=$B$6,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="D45" s="45">
+        <f>IF(D43&gt;=$B$6,"YES","NO")</f>
+        <v/>
+      </c>
+      <c r="E45" s="45">
+        <f>IF(E43&gt;=$B$6,"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>VERDICT</t>
+        </is>
+      </c>
+      <c r="B46" s="46">
+        <f>IF(AND(B44="YES",B45="YES"),"GO",IF(OR(B44="YES",B45="YES"),"CONDITIONAL","NO-GO"))</f>
+        <v/>
+      </c>
+      <c r="C46" s="46">
+        <f>IF(AND(C44="YES",C45="YES"),"GO",IF(OR(C44="YES",C45="YES"),"CONDITIONAL","NO-GO"))</f>
+        <v/>
+      </c>
+      <c r="D46" s="46">
+        <f>IF(AND(D44="YES",D45="YES"),"GO",IF(OR(D44="YES",D45="YES"),"CONDITIONAL","NO-GO"))</f>
+        <v/>
+      </c>
+      <c r="E46" s="46">
+        <f>IF(AND(E44="YES",E45="YES"),"GO",IF(OR(E44="YES",E45="YES"),"CONDITIONAL","NO-GO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>AJ's 3 levers to save a CONDITIONAL deal: (1) lower the price toward the MAO, (2) ask the seller to carry a slice — the blended rate drops so DSCR clears and CoC jumps, (3) add down payment. Full seller carry (interest-only) often clears both even at the asking price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>Don't pay the seller for value YOU create (rent bumps, occupancy, utility bill-back, new revenue).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C6:E6"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B44:E45">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"YES"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="2">
+      <formula>"NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B46:E46">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="0">
+      <formula>"GO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
+      <formula>"CONDITIONAL"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="2">
+      <formula>"NO-GO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3415,7 +4873,7 @@
           <t>Jan</t>
         </is>
       </c>
-      <c r="B15" s="40" t="n">
+      <c r="B15" s="47" t="n">
         <v>31</v>
       </c>
       <c r="C15" s="21" t="n">
@@ -3432,7 +4890,7 @@
           <t>Feb</t>
         </is>
       </c>
-      <c r="B16" s="40" t="n">
+      <c r="B16" s="47" t="n">
         <v>28</v>
       </c>
       <c r="C16" s="21" t="n">
@@ -3449,7 +4907,7 @@
           <t>Mar</t>
         </is>
       </c>
-      <c r="B17" s="40" t="n">
+      <c r="B17" s="47" t="n">
         <v>31</v>
       </c>
       <c r="C17" s="21" t="n">
@@ -3466,7 +4924,7 @@
           <t>Apr</t>
         </is>
       </c>
-      <c r="B18" s="40" t="n">
+      <c r="B18" s="47" t="n">
         <v>30</v>
       </c>
       <c r="C18" s="21" t="n">
@@ -3483,7 +4941,7 @@
           <t>May</t>
         </is>
       </c>
-      <c r="B19" s="40" t="n">
+      <c r="B19" s="47" t="n">
         <v>31</v>
       </c>
       <c r="C19" s="21" t="n">
@@ -3500,7 +4958,7 @@
           <t>Jun</t>
         </is>
       </c>
-      <c r="B20" s="40" t="n">
+      <c r="B20" s="47" t="n">
         <v>30</v>
       </c>
       <c r="C20" s="21" t="n">
@@ -3517,7 +4975,7 @@
           <t>Jul</t>
         </is>
       </c>
-      <c r="B21" s="40" t="n">
+      <c r="B21" s="47" t="n">
         <v>31</v>
       </c>
       <c r="C21" s="21" t="n">
@@ -3534,7 +4992,7 @@
           <t>Aug</t>
         </is>
       </c>
-      <c r="B22" s="40" t="n">
+      <c r="B22" s="47" t="n">
         <v>31</v>
       </c>
       <c r="C22" s="21" t="n">
@@ -3551,7 +5009,7 @@
           <t>Sep</t>
         </is>
       </c>
-      <c r="B23" s="40" t="n">
+      <c r="B23" s="47" t="n">
         <v>30</v>
       </c>
       <c r="C23" s="21" t="n">
@@ -3568,7 +5026,7 @@
           <t>Oct</t>
         </is>
       </c>
-      <c r="B24" s="40" t="n">
+      <c r="B24" s="47" t="n">
         <v>31</v>
       </c>
       <c r="C24" s="21" t="n">
@@ -3585,7 +5043,7 @@
           <t>Nov</t>
         </is>
       </c>
-      <c r="B25" s="40" t="n">
+      <c r="B25" s="47" t="n">
         <v>30</v>
       </c>
       <c r="C25" s="21" t="n">
@@ -3602,7 +5060,7 @@
           <t>Dec</t>
         </is>
       </c>
-      <c r="B26" s="40" t="n">
+      <c r="B26" s="47" t="n">
         <v>31</v>
       </c>
       <c r="C26" s="21" t="n">
@@ -3659,7 +5117,7 @@
           <t>Total sites in build</t>
         </is>
       </c>
-      <c r="E31" s="41">
+      <c r="E31" s="48">
         <f>B8+B11</f>
         <v/>
       </c>
@@ -3693,7 +5151,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4029,7 +5487,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4060,7 +5518,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="42" t="inlineStr">
+      <c r="A3" s="49" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
@@ -4532,43 +5990,43 @@
           <t>Net Sale Proceeds (reversion)</t>
         </is>
       </c>
-      <c r="C14" s="43">
+      <c r="C14" s="50">
         <f>IF(1=Underwriting!B49,((C10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-C12,0)</f>
         <v/>
       </c>
-      <c r="D14" s="43">
+      <c r="D14" s="50">
         <f>IF(2=Underwriting!B49,((D10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-D12,0)</f>
         <v/>
       </c>
-      <c r="E14" s="43">
+      <c r="E14" s="50">
         <f>IF(3=Underwriting!B49,((E10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-E12,0)</f>
         <v/>
       </c>
-      <c r="F14" s="43">
+      <c r="F14" s="50">
         <f>IF(4=Underwriting!B49,((F10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-F12,0)</f>
         <v/>
       </c>
-      <c r="G14" s="43">
+      <c r="G14" s="50">
         <f>IF(5=Underwriting!B49,((G10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-G12,0)</f>
         <v/>
       </c>
-      <c r="H14" s="43">
+      <c r="H14" s="50">
         <f>IF(6=Underwriting!B49,((H10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-H12,0)</f>
         <v/>
       </c>
-      <c r="I14" s="43">
+      <c r="I14" s="50">
         <f>IF(7=Underwriting!B49,((I10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-I12,0)</f>
         <v/>
       </c>
-      <c r="J14" s="43">
+      <c r="J14" s="50">
         <f>IF(8=Underwriting!B49,((J10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-J12,0)</f>
         <v/>
       </c>
-      <c r="K14" s="43">
+      <c r="K14" s="50">
         <f>IF(9=Underwriting!B49,((K10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-K12,0)</f>
         <v/>
       </c>
-      <c r="L14" s="43">
+      <c r="L14" s="50">
         <f>IF(10=Underwriting!B49,((L10*(1+Underwriting!B16))/Underwriting!B50)*(1-Underwriting!B51)-L12,0)</f>
         <v/>
       </c>
@@ -4724,547 +6182,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>SENSITIVITY TABLES</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="15" t="inlineStr">
-        <is>
-          <t>Rows = purchase price scenarios. Columns = interest rate. Cells recompute live from Underwriting inputs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>CASH-ON-CASH RETURN  —  Price x Interest Rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="44" t="inlineStr">
-        <is>
-          <t>Price \ Rate</t>
-        </is>
-      </c>
-      <c r="B5" s="45">
-        <f>Underwriting!B45+-0.01</f>
-        <v/>
-      </c>
-      <c r="C5" s="45">
-        <f>Underwriting!B45+-0.005</f>
-        <v/>
-      </c>
-      <c r="D5" s="45">
-        <f>Underwriting!B45+0</f>
-        <v/>
-      </c>
-      <c r="E5" s="45">
-        <f>Underwriting!B45+0.005</f>
-        <v/>
-      </c>
-      <c r="F5" s="45">
-        <f>Underwriting!B45+0.01</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="30">
-        <f>Underwriting!B9*0.9</f>
-        <v/>
-      </c>
-      <c r="B6" s="37">
-        <f>(Underwriting!B40-((($A6*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="C6" s="37">
-        <f>(Underwriting!B40-((($A6*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="D6" s="37">
-        <f>(Underwriting!B40-((($A6*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="E6" s="37">
-        <f>(Underwriting!B40-((($A6*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="F6" s="37">
-        <f>(Underwriting!B40-((($A6*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A6*(1-Underwriting!B44)+$A6*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="30">
-        <f>Underwriting!B9*0.95</f>
-        <v/>
-      </c>
-      <c r="B7" s="37">
-        <f>(Underwriting!B40-((($A7*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="C7" s="37">
-        <f>(Underwriting!B40-((($A7*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="D7" s="37">
-        <f>(Underwriting!B40-((($A7*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="E7" s="37">
-        <f>(Underwriting!B40-((($A7*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="F7" s="37">
-        <f>(Underwriting!B40-((($A7*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A7*(1-Underwriting!B44)+$A7*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="30">
-        <f>Underwriting!B9*1.0</f>
-        <v/>
-      </c>
-      <c r="B8" s="37">
-        <f>(Underwriting!B40-((($A8*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="C8" s="37">
-        <f>(Underwriting!B40-((($A8*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="D8" s="37">
-        <f>(Underwriting!B40-((($A8*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="E8" s="37">
-        <f>(Underwriting!B40-((($A8*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="F8" s="37">
-        <f>(Underwriting!B40-((($A8*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A8*(1-Underwriting!B44)+$A8*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="30">
-        <f>Underwriting!B9*1.05</f>
-        <v/>
-      </c>
-      <c r="B9" s="37">
-        <f>(Underwriting!B40-((($A9*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="C9" s="37">
-        <f>(Underwriting!B40-((($A9*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="D9" s="37">
-        <f>(Underwriting!B40-((($A9*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="E9" s="37">
-        <f>(Underwriting!B40-((($A9*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="F9" s="37">
-        <f>(Underwriting!B40-((($A9*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A9*(1-Underwriting!B44)+$A9*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="30">
-        <f>Underwriting!B9*1.1</f>
-        <v/>
-      </c>
-      <c r="B10" s="37">
-        <f>(Underwriting!B40-((($A10*Underwriting!B44)*(B$5/12)/(1-(1+B$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="C10" s="37">
-        <f>(Underwriting!B40-((($A10*Underwriting!B44)*(C$5/12)/(1-(1+C$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="D10" s="37">
-        <f>(Underwriting!B40-((($A10*Underwriting!B44)*(D$5/12)/(1-(1+D$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="E10" s="37">
-        <f>(Underwriting!B40-((($A10*Underwriting!B44)*(E$5/12)/(1-(1+E$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-      <c r="F10" s="37">
-        <f>(Underwriting!B40-((($A10*Underwriting!B44)*(F$5/12)/(1-(1+F$5/12)^(-Underwriting!B46*12)))*12))/($A10*(1-Underwriting!B44)+$A10*Underwriting!B47+Underwriting!B48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>DEBT SERVICE COVERAGE (DSCR)  —  Price x Interest Rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="44" t="inlineStr">
-        <is>
-          <t>Price \ Rate</t>
-        </is>
-      </c>
-      <c r="B14" s="45">
-        <f>Underwriting!B45+-0.01</f>
-        <v/>
-      </c>
-      <c r="C14" s="45">
-        <f>Underwriting!B45+-0.005</f>
-        <v/>
-      </c>
-      <c r="D14" s="45">
-        <f>Underwriting!B45+0</f>
-        <v/>
-      </c>
-      <c r="E14" s="45">
-        <f>Underwriting!B45+0.005</f>
-        <v/>
-      </c>
-      <c r="F14" s="45">
-        <f>Underwriting!B45+0.01</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="30">
-        <f>Underwriting!B9*0.9</f>
-        <v/>
-      </c>
-      <c r="B15" s="46">
-        <f>Underwriting!B40/((($A15*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="C15" s="46">
-        <f>Underwriting!B40/((($A15*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="D15" s="46">
-        <f>Underwriting!B40/((($A15*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="E15" s="46">
-        <f>Underwriting!B40/((($A15*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="F15" s="46">
-        <f>Underwriting!B40/((($A15*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="30">
-        <f>Underwriting!B9*0.95</f>
-        <v/>
-      </c>
-      <c r="B16" s="46">
-        <f>Underwriting!B40/((($A16*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="C16" s="46">
-        <f>Underwriting!B40/((($A16*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="D16" s="46">
-        <f>Underwriting!B40/((($A16*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="E16" s="46">
-        <f>Underwriting!B40/((($A16*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="F16" s="46">
-        <f>Underwriting!B40/((($A16*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="30">
-        <f>Underwriting!B9*1.0</f>
-        <v/>
-      </c>
-      <c r="B17" s="46">
-        <f>Underwriting!B40/((($A17*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="C17" s="46">
-        <f>Underwriting!B40/((($A17*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="D17" s="46">
-        <f>Underwriting!B40/((($A17*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="E17" s="46">
-        <f>Underwriting!B40/((($A17*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="F17" s="46">
-        <f>Underwriting!B40/((($A17*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="30">
-        <f>Underwriting!B9*1.05</f>
-        <v/>
-      </c>
-      <c r="B18" s="46">
-        <f>Underwriting!B40/((($A18*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="C18" s="46">
-        <f>Underwriting!B40/((($A18*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="D18" s="46">
-        <f>Underwriting!B40/((($A18*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="E18" s="46">
-        <f>Underwriting!B40/((($A18*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="F18" s="46">
-        <f>Underwriting!B40/((($A18*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="30">
-        <f>Underwriting!B9*1.1</f>
-        <v/>
-      </c>
-      <c r="B19" s="46">
-        <f>Underwriting!B40/((($A19*Underwriting!B44)*(B$14/12)/(1-(1+B$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="C19" s="46">
-        <f>Underwriting!B40/((($A19*Underwriting!B44)*(C$14/12)/(1-(1+C$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="D19" s="46">
-        <f>Underwriting!B40/((($A19*Underwriting!B44)*(D$14/12)/(1-(1+D$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="E19" s="46">
-        <f>Underwriting!B40/((($A19*Underwriting!B44)*(E$14/12)/(1-(1+E$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-      <c r="F19" s="46">
-        <f>Underwriting!B40/((($A19*Underwriting!B44)*(F$14/12)/(1-(1+F$14/12)^(-Underwriting!B46*12)))*12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>NOTE: the two tables above hold NOI constant to isolate price &amp; financing risk.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>CASH-ON-CASH RETURN  —  Monthly Rent x Vacancy</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="44" t="inlineStr">
-        <is>
-          <t>Rent \ Vacancy</t>
-        </is>
-      </c>
-      <c r="B24" s="47" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C24" s="47" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D24" s="47" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E24" s="47" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F24" s="47" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="30">
-        <f>Underwriting!B11+-100</f>
-        <v/>
-      </c>
-      <c r="B25" s="37">
-        <f>(((Underwriting!B8*$A25*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="C25" s="37">
-        <f>(((Underwriting!B8*$A25*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="D25" s="37">
-        <f>(((Underwriting!B8*$A25*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="E25" s="37">
-        <f>(((Underwriting!B8*$A25*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="F25" s="37">
-        <f>(((Underwriting!B8*$A25*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A25*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="30">
-        <f>Underwriting!B11+-50</f>
-        <v/>
-      </c>
-      <c r="B26" s="37">
-        <f>(((Underwriting!B8*$A26*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="C26" s="37">
-        <f>(((Underwriting!B8*$A26*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="D26" s="37">
-        <f>(((Underwriting!B8*$A26*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="E26" s="37">
-        <f>(((Underwriting!B8*$A26*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="F26" s="37">
-        <f>(((Underwriting!B8*$A26*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A26*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="30">
-        <f>Underwriting!B11+0</f>
-        <v/>
-      </c>
-      <c r="B27" s="37">
-        <f>(((Underwriting!B8*$A27*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="C27" s="37">
-        <f>(((Underwriting!B8*$A27*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="D27" s="37">
-        <f>(((Underwriting!B8*$A27*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="E27" s="37">
-        <f>(((Underwriting!B8*$A27*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="F27" s="37">
-        <f>(((Underwriting!B8*$A27*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A27*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="30">
-        <f>Underwriting!B11+50</f>
-        <v/>
-      </c>
-      <c r="B28" s="37">
-        <f>(((Underwriting!B8*$A28*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="C28" s="37">
-        <f>(((Underwriting!B8*$A28*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="D28" s="37">
-        <f>(((Underwriting!B8*$A28*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="E28" s="37">
-        <f>(((Underwriting!B8*$A28*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="F28" s="37">
-        <f>(((Underwriting!B8*$A28*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A28*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="30">
-        <f>Underwriting!B11+100</f>
-        <v/>
-      </c>
-      <c r="B29" s="37">
-        <f>(((Underwriting!B8*$A29*12*(1-B$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-B$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="C29" s="37">
-        <f>(((Underwriting!B8*$A29*12*(1-C$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-C$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="D29" s="37">
-        <f>(((Underwriting!B8*$A29*12*(1-D$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-D$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="E29" s="37">
-        <f>(((Underwriting!B8*$A29*12*(1-E$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-E$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-      <c r="F29" s="37">
-        <f>(((Underwriting!B8*$A29*12*(1-F$24)+Underwriting!B23)-((Underwriting!B35-Underwriting!B33)+Underwriting!B14*(Underwriting!B8*$A29*12*(1-F$24)+Underwriting!B23)))-Underwriting!B59)/Underwriting!B57</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="15" t="inlineStr">
-        <is>
-          <t>NOTE: this table recomputes NOI (management fee scales with EGI). Uses sites x rent income, not the Income Detail build.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A4:F4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Rebrand framework to LindaAI (remove all AJ refs) + master underwrite-deal skill
- Scrub every external-author reference from the workbook and skills; the
  framework is now presented as LindaAI's own (Deal Scorecard, Normalization,
  Offer Structures, Read Me, report footer all rebranded).
- Add 'underwrite-deal' master skill: one-shot pipeline that chains
  youtube-transcribe -> rv-park-autofill -> deal-report. run_pipeline.py runs
  fill+normalize+report in a single command, outputting branded Wise Certified
  xlsx + PDF + PPTX. Registered in manifest (gold); manifest -> 1.11.0.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFUKyb6gzsdDbmscePYHf6
</commit_message>
<xml_diff>
--- a/RV_Park_Underwriting.xlsx
+++ b/RV_Park_Underwriting.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Deal Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Deal Scorecard" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Underwriting" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Normalization" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Offer Structures" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Income Detail" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Actuals vs Pro Forma" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Pro Forma &amp; Returns" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Sensitivity" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Loan Sizing" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deal Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deal Scorecard" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Underwriting" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normalization" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Offer Structures" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income Detail" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals vs Pro Forma" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pro Forma &amp; Returns" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loan Sizing" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -738,28 +738,28 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>An RV-park deal-screening model built on AJ Kukra's 'RV Park Profit Blueprint' framework. Drop in a</t>
+          <t>An RV-park deal-screening model built on the LindaAI underwriting framework. Drop in a</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>deal's numbers and it tells you in minutes whether it makes money — using AJ's 5 key metrics, his 5</t>
+          <t>deal's numbers and it tells you in minutes whether it makes money — using Linda's 5 key metrics, its 5</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>quick hacks, NOI normalization, and his go / conditional / no-go rule. Works for RV parks and adapts</t>
+          <t>quick hacks, NOI normalization, and its go / conditional / no-go rule. Works for RV parks and adapts</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>directly to mobile home parks (same lot-rent math). Source: AJ Kukra, RV Park Profit Blueprint workshop.</t>
+          <t>directly to mobile home parks (same lot-rent math). Part of the LindaAI underwriting framework.</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>AJ'S 5 KEY METRICS (the heartbeat of the deal)</t>
+          <t>LINDA'S 5 KEY METRICS (the heartbeat of the deal)</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3. DSCR = NOI / annual debt. AJ's floor is 1.35x — that's YOUR target, not just the lender's.</t>
+          <t xml:space="preserve">  3. DSCR = NOI / annual debt. Linda's floor is 1.35x — that's YOUR target, not just the lender's.</t>
         </is>
       </c>
     </row>
@@ -804,7 +804,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5. Cash-on-Cash = net profit / cash invested. AJ's target is 10%+.</t>
+          <t xml:space="preserve">  5. Cash-on-Cash = net profit / cash invested. Linda's target is 10%+.</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>AJ'S 5 QUICK HACKS (screen any listing in ~2 minutes) — see the Deal Scorecard tab</t>
+          <t>LINDA'S 5 QUICK HACKS (screen any listing in ~2 minutes) — see the Deal Scorecard tab</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>NORMALIZE THE NOI (AJ: never trust the seller's NOI) — see the Normalization tab</t>
+          <t>NORMALIZE THE NOI (Linda: never trust the seller's NOI) — see the Normalization tab</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AJ's 4 standard adjustments: management -&gt; 10% of EGI, repairs -&gt; 5% (or prior year), capex -&gt; +3%,</t>
+          <t xml:space="preserve">  Linda's 4 standard adjustments: management -&gt; 10% of EGI, repairs -&gt; 5% (or prior year), capex -&gt; +3%,</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Both fail -&gt; likely NO-GO. To save a conditional deal, use AJ's 3 levers: lower the price to your</t>
+          <t xml:space="preserve">  Both fail -&gt; likely NO-GO. To save a conditional deal, use Linda's 3 levers: lower the price to your</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Deal Scorecard — AJ's metrics + 5 hacks rated GOOD/OK/BAD with his go / conditional / no-go verdict.</t>
+          <t xml:space="preserve">  • Deal Scorecard — Linda's metrics + 5 hacks rated GOOD/OK/BAD with its go / conditional / no-go verdict.</t>
         </is>
       </c>
     </row>
@@ -973,14 +973,14 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Normalization — rebuild the seller's NOI with AJ's 4 adjustments; shows the overpayment risk.</t>
+          <t xml:space="preserve">  • Normalization — rebuild the seller's NOI with Linda's 4 adjustments; shows the overpayment risk.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Offer Structures — AJ's 4-column engine: Seller / Conventional / Partial carry / Full carry, two-lien</t>
+          <t xml:space="preserve">  • Offer Structures — Linda's 4-column engine: Seller / Conventional / Partial carry / Full carry, two-lien</t>
         </is>
       </c>
     </row>
@@ -2273,14 +2273,14 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>DEAL SCORECARD — AJ KUKRA 'RV PARK PROFIT BLUEPRINT'</t>
+          <t>DEAL SCORECARD — LINDAAI FRAMEWORK</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>AJ's framework. Underwrite to the NORMALIZED NOI (see Normalization tab) before trusting these. GREEN cutoff cells are editable. Source: AJ Kukra, RV Park Profit Blueprint workshop.</t>
+          <t>Linda's framework. Underwrite to the NORMALIZED NOI (see Normalization tab) before trusting these. GREEN cutoff cells are editable. Part of the LindaAI underwriting framework.</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>AJ's rule</t>
+          <t>Linda's rule</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>AJ floor 1.35x to GO</t>
+          <t>Linda floor: 1.35x to GO</t>
         </is>
       </c>
       <c r="D6" s="19" t="n">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>AJ target 10%+ to GO</t>
+          <t>Linda target: 10%+ to GO</t>
         </is>
       </c>
       <c r="D7" s="21" t="n">
@@ -2538,7 +2538,7 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>VERDICT  (AJ's rule: both DSCR and Cash-on-Cash must clear)</t>
+          <t>VERDICT  (Linda's rule: both DSCR and Cash-on-Cash must clear)</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2589,7 @@
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>CONDITIONAL means restructure to save it (AJ's 3 levers): (1) lower price to your MAO, (2) ask the seller to carry a slice — blended rate drops, DSCR clears, CoC jumps, (3) more down payment. If none work and the seller won't budge, your underwriting just saved you from an expensive mistake.</t>
+          <t>CONDITIONAL means restructure to save it (Linda's 3 levers): (1) lower price to your MAO, (2) ask the seller to carry a slice — blended rate drops, DSCR clears, CoC jumps, (3) more down payment. If none work and the seller won't budge, your underwriting just saved you from an expensive mistake.</t>
         </is>
       </c>
     </row>
@@ -3419,14 +3419,14 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>AJ: the T12 is your starting point but never trusted as-is. Enter the SELLER'S reported figures (yellow); the Normalized column rebuilds the NOI with AJ's 4 adjustments. Source: AJ Kukra.</t>
+          <t>Linda: the T-12 is your starting point but never trusted as-is. Enter the SELLER'S reported figures (yellow); the Normalized column rebuilds the NOI with Linda's 4 adjustments. Part of the LindaAI framework.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>AJ'S NORMALIZATION RULES (editable)</t>
+          <t>LINDA'S NORMALIZATION RULES (editable)</t>
         </is>
       </c>
     </row>
@@ -3512,7 +3512,7 @@
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>seller's real top line (AJ: gross income = EGI)</t>
+          <t>seller's real top line (Linda: gross income = EGI)</t>
         </is>
       </c>
     </row>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>AJ adjustment</t>
+          <t>Linda adjustment</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>AJ: under 30% means something's missing</t>
+          <t>Linda: under 30% means something's missing</t>
         </is>
       </c>
     </row>
@@ -3793,7 +3793,7 @@
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>AJ: a small NOI cut = a huge price difference</t>
+          <t>Linda: a small NOI cut = a huge price difference</t>
         </is>
       </c>
     </row>
@@ -3835,14 +3835,14 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>OFFER STRUCTURES — MAO &amp; SELLER CARRY (AJ KUKRA)</t>
+          <t>OFFER STRUCTURES — MAO &amp; SELLER CARRY (LINDA FRAMEWORK)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>NOI is held constant (operations don't change with financing). Each column is a price + financing scenario; yellow = editable levers. Verdict uses AJ's rule: DSCR &gt;= target AND Cash-on-Cash &gt;= target.</t>
+          <t>NOI is held constant (operations don't change with financing). Each column is a price + financing scenario; yellow = editable levers. Verdict uses Linda's rule: DSCR &gt;= target AND Cash-on-Cash &gt;= target.</t>
         </is>
       </c>
     </row>
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>AJ floor</t>
+          <t>Linda floor</t>
         </is>
       </c>
     </row>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>AJ target</t>
+          <t>Linda target</t>
         </is>
       </c>
     </row>
@@ -4650,7 +4650,7 @@
     <row r="48">
       <c r="A48" s="15" t="inlineStr">
         <is>
-          <t>AJ's 3 levers to save a CONDITIONAL deal: (1) lower the price toward the MAO, (2) ask the seller to carry a slice — the blended rate drops so DSCR clears and CoC jumps, (3) add down payment. Full seller carry (interest-only) often clears both even at the asking price.</t>
+          <t>Linda's 3 levers to save a CONDITIONAL deal: (1) lower the price toward the MAO, (2) ask the seller to carry a slice — the blended rate drops so DSCR clears and CoC jumps, (3) add down payment. Full seller carry (interest-only) often clears both even at the asking price.</t>
         </is>
       </c>
     </row>

</xml_diff>